<commit_message>
updated the sadhana sheet
</commit_message>
<xml_diff>
--- a/public/Daily Sadhana.xlsx
+++ b/public/Daily Sadhana.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sahaa\OneDrive\Documents\github_anandasvarupa\give_web\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3988EC0A-9B1E-47D3-85CE-936D145340B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4918CD72-C173-41B0-9C5A-ED1C74A8EEB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BS-4" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="211">
   <si>
     <t>url</t>
   </si>
@@ -382,6 +382,285 @@
   <si>
     <t>Today's listening to Srila Prabhupada - 53</t>
   </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=r0Js40PlGD0</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=S0btQn0XaY0</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=nlsOMWl1y3w</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=BcXT1WN1xo0</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=7dcwvdqCwZs</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Jye7BHkjxhM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=WycwPwr66j4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=mr0D1YTBL18</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=_-ESvQqE23I</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=zbmCkISF2Xg</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=xIURA7wzdL4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=bGI7KXeiVT0</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=a6W4QQzZ68s</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=rjjGebNywWs</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=72kjLmoSqmQ</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=kErCqAcgn0o</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=CSytDm8nTVo</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=801iMaTm8OQ</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=_-7L9SBelA8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=uuWqbYvEVwk</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=2RfTtRwh8AY</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=kunVE0i_Ex8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Rzz9pHvuedQ</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=HeCx7oWx_yU</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=A4ev3osvrNM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=91_xCuo2IZE</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=G7Xx33wHY5M</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=voizu2-Kpk4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=JawtmRA_drk</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=-fN6xmmjBuU</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=9ryiznz1di4</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 106</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 107</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 108</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 109</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 110</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 111</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 112</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 113</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 114</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 115</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 116</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 117</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 118</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 119</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 120</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 121</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 122</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 123</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 124</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 125</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 126</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 127</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 128</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 129</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 130</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 131</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 132</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 133</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 134</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 135</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 136</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 54</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 55</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 56</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 57</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 58</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 59</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 60</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 61</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 62</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 63</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 64</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 65</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 66</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 67</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 68</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 69</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 70</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 71</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 72</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 73</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 74</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 75</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 76</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 77</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 78</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 79</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 80</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 81</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 82</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 83</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 84</t>
+  </si>
 </sst>
 </file>
 
@@ -391,7 +670,7 @@
     <numFmt numFmtId="164" formatCode="mmm\ d\,\ yy"/>
     <numFmt numFmtId="165" formatCode="mmm\ d\,\ yyyy"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -415,6 +694,19 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -441,10 +733,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -470,8 +763,12 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -692,7 +989,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z12"/>
+  <dimension ref="A1:Z43"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="56.81640625" customWidth="1"/>
@@ -855,7 +1152,349 @@
         <v>46116</v>
       </c>
     </row>
+    <row r="13" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="C13" s="5">
+        <v>46117</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="C14" s="5">
+        <v>46118</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="C15" s="5">
+        <v>46119</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C16" s="5">
+        <v>46120</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C17" s="5">
+        <v>46121</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="C18" s="5">
+        <v>46122</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="C19" s="5">
+        <v>46123</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C20" s="5">
+        <v>46124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="C21" s="5">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="C22" s="5">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="C23" s="5">
+        <v>46127</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C24" s="5">
+        <v>46128</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="C25" s="5">
+        <v>46129</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C26" s="5">
+        <v>46130</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="C27" s="5">
+        <v>46131</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="C28" s="5">
+        <v>46132</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="C29" s="5">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="C30" s="5">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C31" s="5">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="C32" s="5">
+        <v>46136</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="C33" s="5">
+        <v>46137</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="C34" s="5">
+        <v>46138</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="C35" s="5">
+        <v>46139</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C36" s="5">
+        <v>46140</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="C37" s="5">
+        <v>46141</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="C38" s="5">
+        <v>46142</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="C39" s="5">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="C40" s="5">
+        <v>46144</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="C41" s="5">
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="C42" s="5">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C43" s="5">
+        <v>46147</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{37EE8AC8-1046-4376-BB05-A1B929BE223D}"/>
     <hyperlink ref="A3" r:id="rId2" xr:uid="{9A78235B-491D-4F27-8C59-6F4F0F990EB0}"/>
@@ -868,8 +1507,40 @@
     <hyperlink ref="A10" r:id="rId9" xr:uid="{6C1AD550-2521-4A95-81A0-2B88850657B8}"/>
     <hyperlink ref="A11" r:id="rId10" xr:uid="{7ABDA8B7-01AD-4540-9F21-90BBDC33B566}"/>
     <hyperlink ref="A12" r:id="rId11" xr:uid="{B919B1C7-A0CE-4C8E-8DBA-2C2A92A56C1C}"/>
+    <hyperlink ref="A13" r:id="rId12" xr:uid="{A8EA6E5E-B6C0-4940-BC4B-F1EFB9F1D2B6}"/>
+    <hyperlink ref="A14" r:id="rId13" xr:uid="{8AEF8F22-6BC3-464F-BC72-72100615F6E6}"/>
+    <hyperlink ref="A15" r:id="rId14" xr:uid="{0A9125A2-F2EC-4118-B2EF-00A0EBF59071}"/>
+    <hyperlink ref="A16" r:id="rId15" xr:uid="{021AE096-45A1-4D33-AC9A-544A6996A7C2}"/>
+    <hyperlink ref="A17" r:id="rId16" xr:uid="{3720685F-4023-44EA-850B-2F16FE2D16A4}"/>
+    <hyperlink ref="A18" r:id="rId17" xr:uid="{43D91C1D-83E6-4250-AD0A-77C7B5A65E5B}"/>
+    <hyperlink ref="A19" r:id="rId18" xr:uid="{9E6BF98B-3082-40E2-8222-D23CBB2CEDD6}"/>
+    <hyperlink ref="A20" r:id="rId19" xr:uid="{7DAF047C-7BCF-4142-9B87-60D9C16693C8}"/>
+    <hyperlink ref="A21" r:id="rId20" xr:uid="{869E4EF2-8083-45C0-8A34-27F6C5C63A52}"/>
+    <hyperlink ref="A22" r:id="rId21" xr:uid="{F5584D6F-1479-4642-BF07-372ABA8CB5E2}"/>
+    <hyperlink ref="A23" r:id="rId22" xr:uid="{978F330E-1165-43F9-A487-E60F0A88BB7F}"/>
+    <hyperlink ref="A24" r:id="rId23" xr:uid="{93CBFC38-4568-42B9-B79C-3C48A65EF929}"/>
+    <hyperlink ref="A25" r:id="rId24" xr:uid="{A2CCC198-C00D-406F-8C2F-8B4CFBCD4F40}"/>
+    <hyperlink ref="A26" r:id="rId25" xr:uid="{4AF1D8E3-CA30-4194-936A-FF94688DB629}"/>
+    <hyperlink ref="A27" r:id="rId26" xr:uid="{B8FEB771-FBEE-425A-948E-9942F4F4284F}"/>
+    <hyperlink ref="A28" r:id="rId27" xr:uid="{5D842A3F-0368-4A2D-88C0-4C5481F7747B}"/>
+    <hyperlink ref="A29" r:id="rId28" xr:uid="{B1BE55ED-465B-4D54-85DB-3A57317EA039}"/>
+    <hyperlink ref="A30" r:id="rId29" xr:uid="{81CCC1C5-7C5A-4860-8527-6D893D26E9BC}"/>
+    <hyperlink ref="A31" r:id="rId30" xr:uid="{26E81E71-0318-4BC9-BCBB-ABA2A53DAB80}"/>
+    <hyperlink ref="A32" r:id="rId31" xr:uid="{88B0C5E2-BDF1-4274-B078-58F35C486EA6}"/>
+    <hyperlink ref="A33" r:id="rId32" xr:uid="{AD04802E-A73E-4145-B882-8F07E17801DE}"/>
+    <hyperlink ref="A34" r:id="rId33" xr:uid="{3B17BFEB-4133-4DA8-9180-6F19F82D82B2}"/>
+    <hyperlink ref="A35" r:id="rId34" xr:uid="{6BCBF5F3-2389-4272-974A-D2929396AB12}"/>
+    <hyperlink ref="A36" r:id="rId35" xr:uid="{FA244E43-B5D0-4D07-8A78-70EC17585A35}"/>
+    <hyperlink ref="A37" r:id="rId36" xr:uid="{DCD8F245-DEFB-4F18-A66B-EB33C71E4D2A}"/>
+    <hyperlink ref="A38" r:id="rId37" xr:uid="{27A41A2B-51BE-4260-BFD0-0BFBF2B126B1}"/>
+    <hyperlink ref="A39" r:id="rId38" xr:uid="{BF7F89E7-CBBD-4A22-BAFC-14C185E6CB07}"/>
+    <hyperlink ref="A40" r:id="rId39" xr:uid="{98FA275E-9A6B-4D32-9514-4F25BB0B7BE7}"/>
+    <hyperlink ref="A41" r:id="rId40" xr:uid="{66D88341-E233-40C7-A0F1-8E34AE93A867}"/>
+    <hyperlink ref="A42" r:id="rId41" xr:uid="{5DA0CFD4-768B-49CC-A3CC-6F8D00361B4A}"/>
+    <hyperlink ref="A43" r:id="rId42" xr:uid="{A11DA0CB-FD50-471B-9BFA-F61671963A09}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId43"/>
 </worksheet>
 </file>
 
@@ -881,7 +1552,7 @@
   <dimension ref="A1:Z947"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="50.90625" customWidth="1"/>
+    <col min="1" max="1" width="54.08984375" customWidth="1"/>
     <col min="2" max="2" width="38.90625" customWidth="1"/>
     <col min="3" max="3" width="28.90625" customWidth="1"/>
     <col min="4" max="4" width="21.36328125" customWidth="1"/>
@@ -2724,9 +3395,15 @@
       <c r="Z54" s="6"/>
     </row>
     <row r="55" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A55" s="6"/>
-      <c r="B55" s="6"/>
-      <c r="C55" s="6"/>
+      <c r="A55" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="C55" s="5">
+        <v>46117</v>
+      </c>
       <c r="D55" s="6"/>
       <c r="E55" s="6"/>
       <c r="F55" s="6"/>
@@ -2752,9 +3429,15 @@
       <c r="Z55" s="6"/>
     </row>
     <row r="56" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A56" s="6"/>
-      <c r="B56" s="6"/>
-      <c r="C56" s="6"/>
+      <c r="A56" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="C56" s="5">
+        <v>46118</v>
+      </c>
       <c r="D56" s="6"/>
       <c r="E56" s="6"/>
       <c r="F56" s="6"/>
@@ -2780,9 +3463,15 @@
       <c r="Z56" s="6"/>
     </row>
     <row r="57" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A57" s="6"/>
-      <c r="B57" s="6"/>
-      <c r="C57" s="6"/>
+      <c r="A57" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="C57" s="5">
+        <v>46119</v>
+      </c>
       <c r="D57" s="6"/>
       <c r="E57" s="6"/>
       <c r="F57" s="6"/>
@@ -2808,9 +3497,15 @@
       <c r="Z57" s="6"/>
     </row>
     <row r="58" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A58" s="6"/>
-      <c r="B58" s="6"/>
-      <c r="C58" s="6"/>
+      <c r="A58" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="C58" s="5">
+        <v>46120</v>
+      </c>
       <c r="D58" s="6"/>
       <c r="E58" s="6"/>
       <c r="F58" s="6"/>
@@ -2836,9 +3531,15 @@
       <c r="Z58" s="6"/>
     </row>
     <row r="59" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A59" s="6"/>
-      <c r="B59" s="6"/>
-      <c r="C59" s="6"/>
+      <c r="A59" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="C59" s="5">
+        <v>46121</v>
+      </c>
       <c r="D59" s="6"/>
       <c r="E59" s="6"/>
       <c r="F59" s="6"/>
@@ -2864,9 +3565,15 @@
       <c r="Z59" s="6"/>
     </row>
     <row r="60" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A60" s="6"/>
-      <c r="B60" s="6"/>
-      <c r="C60" s="6"/>
+      <c r="A60" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="C60" s="5">
+        <v>46122</v>
+      </c>
       <c r="D60" s="6"/>
       <c r="E60" s="6"/>
       <c r="F60" s="6"/>
@@ -2892,9 +3599,15 @@
       <c r="Z60" s="6"/>
     </row>
     <row r="61" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A61" s="6"/>
-      <c r="B61" s="6"/>
-      <c r="C61" s="6"/>
+      <c r="A61" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="C61" s="5">
+        <v>46123</v>
+      </c>
       <c r="D61" s="6"/>
       <c r="E61" s="6"/>
       <c r="F61" s="6"/>
@@ -2920,9 +3633,15 @@
       <c r="Z61" s="6"/>
     </row>
     <row r="62" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A62" s="6"/>
-      <c r="B62" s="6"/>
-      <c r="C62" s="6"/>
+      <c r="A62" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="C62" s="5">
+        <v>46124</v>
+      </c>
       <c r="D62" s="6"/>
       <c r="E62" s="6"/>
       <c r="F62" s="6"/>
@@ -2948,9 +3667,15 @@
       <c r="Z62" s="6"/>
     </row>
     <row r="63" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A63" s="6"/>
-      <c r="B63" s="6"/>
-      <c r="C63" s="6"/>
+      <c r="A63" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="C63" s="5">
+        <v>46125</v>
+      </c>
       <c r="D63" s="6"/>
       <c r="E63" s="6"/>
       <c r="F63" s="6"/>
@@ -2976,9 +3701,15 @@
       <c r="Z63" s="6"/>
     </row>
     <row r="64" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A64" s="6"/>
-      <c r="B64" s="6"/>
-      <c r="C64" s="6"/>
+      <c r="A64" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="C64" s="5">
+        <v>46126</v>
+      </c>
       <c r="D64" s="6"/>
       <c r="E64" s="6"/>
       <c r="F64" s="6"/>
@@ -3004,9 +3735,15 @@
       <c r="Z64" s="6"/>
     </row>
     <row r="65" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A65" s="6"/>
-      <c r="B65" s="6"/>
-      <c r="C65" s="6"/>
+      <c r="A65" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C65" s="5">
+        <v>46127</v>
+      </c>
       <c r="D65" s="6"/>
       <c r="E65" s="6"/>
       <c r="F65" s="6"/>
@@ -3032,9 +3769,15 @@
       <c r="Z65" s="6"/>
     </row>
     <row r="66" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A66" s="6"/>
-      <c r="B66" s="6"/>
-      <c r="C66" s="6"/>
+      <c r="A66" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="C66" s="5">
+        <v>46128</v>
+      </c>
       <c r="D66" s="6"/>
       <c r="E66" s="6"/>
       <c r="F66" s="6"/>
@@ -3060,9 +3803,15 @@
       <c r="Z66" s="6"/>
     </row>
     <row r="67" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A67" s="6"/>
-      <c r="B67" s="6"/>
-      <c r="C67" s="6"/>
+      <c r="A67" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="C67" s="5">
+        <v>46129</v>
+      </c>
       <c r="D67" s="6"/>
       <c r="E67" s="6"/>
       <c r="F67" s="6"/>
@@ -3088,9 +3837,15 @@
       <c r="Z67" s="6"/>
     </row>
     <row r="68" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A68" s="6"/>
-      <c r="B68" s="6"/>
-      <c r="C68" s="6"/>
+      <c r="A68" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="C68" s="5">
+        <v>46130</v>
+      </c>
       <c r="D68" s="6"/>
       <c r="E68" s="6"/>
       <c r="F68" s="6"/>
@@ -3116,9 +3871,15 @@
       <c r="Z68" s="6"/>
     </row>
     <row r="69" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A69" s="6"/>
-      <c r="B69" s="6"/>
-      <c r="C69" s="6"/>
+      <c r="A69" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="C69" s="5">
+        <v>46131</v>
+      </c>
       <c r="D69" s="6"/>
       <c r="E69" s="6"/>
       <c r="F69" s="6"/>
@@ -3144,9 +3905,15 @@
       <c r="Z69" s="6"/>
     </row>
     <row r="70" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A70" s="6"/>
-      <c r="B70" s="6"/>
-      <c r="C70" s="6"/>
+      <c r="A70" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="C70" s="5">
+        <v>46132</v>
+      </c>
       <c r="D70" s="6"/>
       <c r="E70" s="6"/>
       <c r="F70" s="6"/>
@@ -3172,9 +3939,15 @@
       <c r="Z70" s="6"/>
     </row>
     <row r="71" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A71" s="6"/>
-      <c r="B71" s="6"/>
-      <c r="C71" s="6"/>
+      <c r="A71" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="C71" s="5">
+        <v>46133</v>
+      </c>
       <c r="D71" s="6"/>
       <c r="E71" s="6"/>
       <c r="F71" s="6"/>
@@ -3200,9 +3973,15 @@
       <c r="Z71" s="6"/>
     </row>
     <row r="72" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A72" s="6"/>
-      <c r="B72" s="6"/>
-      <c r="C72" s="6"/>
+      <c r="A72" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="C72" s="5">
+        <v>46134</v>
+      </c>
       <c r="D72" s="6"/>
       <c r="E72" s="6"/>
       <c r="F72" s="6"/>
@@ -3228,9 +4007,15 @@
       <c r="Z72" s="6"/>
     </row>
     <row r="73" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A73" s="6"/>
-      <c r="B73" s="6"/>
-      <c r="C73" s="6"/>
+      <c r="A73" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C73" s="5">
+        <v>46135</v>
+      </c>
       <c r="D73" s="6"/>
       <c r="E73" s="6"/>
       <c r="F73" s="6"/>
@@ -3256,9 +4041,15 @@
       <c r="Z73" s="6"/>
     </row>
     <row r="74" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A74" s="6"/>
-      <c r="B74" s="6"/>
-      <c r="C74" s="6"/>
+      <c r="A74" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="C74" s="5">
+        <v>46136</v>
+      </c>
       <c r="D74" s="6"/>
       <c r="E74" s="6"/>
       <c r="F74" s="6"/>
@@ -3284,9 +4075,15 @@
       <c r="Z74" s="6"/>
     </row>
     <row r="75" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A75" s="6"/>
-      <c r="B75" s="6"/>
-      <c r="C75" s="6"/>
+      <c r="A75" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C75" s="5">
+        <v>46137</v>
+      </c>
       <c r="D75" s="6"/>
       <c r="E75" s="6"/>
       <c r="F75" s="6"/>
@@ -3312,9 +4109,15 @@
       <c r="Z75" s="6"/>
     </row>
     <row r="76" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A76" s="6"/>
-      <c r="B76" s="6"/>
-      <c r="C76" s="6"/>
+      <c r="A76" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="C76" s="5">
+        <v>46138</v>
+      </c>
       <c r="D76" s="6"/>
       <c r="E76" s="6"/>
       <c r="F76" s="6"/>
@@ -3340,9 +4143,15 @@
       <c r="Z76" s="6"/>
     </row>
     <row r="77" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A77" s="6"/>
-      <c r="B77" s="6"/>
-      <c r="C77" s="6"/>
+      <c r="A77" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="C77" s="5">
+        <v>46139</v>
+      </c>
       <c r="D77" s="6"/>
       <c r="E77" s="6"/>
       <c r="F77" s="6"/>
@@ -3368,9 +4177,15 @@
       <c r="Z77" s="6"/>
     </row>
     <row r="78" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A78" s="6"/>
-      <c r="B78" s="6"/>
-      <c r="C78" s="6"/>
+      <c r="A78" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="C78" s="5">
+        <v>46140</v>
+      </c>
       <c r="D78" s="6"/>
       <c r="E78" s="6"/>
       <c r="F78" s="6"/>
@@ -3396,9 +4211,15 @@
       <c r="Z78" s="6"/>
     </row>
     <row r="79" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A79" s="6"/>
-      <c r="B79" s="6"/>
-      <c r="C79" s="6"/>
+      <c r="A79" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C79" s="5">
+        <v>46141</v>
+      </c>
       <c r="D79" s="6"/>
       <c r="E79" s="6"/>
       <c r="F79" s="6"/>
@@ -3424,9 +4245,15 @@
       <c r="Z79" s="6"/>
     </row>
     <row r="80" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A80" s="6"/>
-      <c r="B80" s="6"/>
-      <c r="C80" s="6"/>
+      <c r="A80" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="C80" s="5">
+        <v>46142</v>
+      </c>
       <c r="D80" s="6"/>
       <c r="E80" s="6"/>
       <c r="F80" s="6"/>
@@ -3452,9 +4279,15 @@
       <c r="Z80" s="6"/>
     </row>
     <row r="81" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A81" s="6"/>
-      <c r="B81" s="6"/>
-      <c r="C81" s="6"/>
+      <c r="A81" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="C81" s="5">
+        <v>46143</v>
+      </c>
       <c r="D81" s="6"/>
       <c r="E81" s="6"/>
       <c r="F81" s="6"/>
@@ -3480,9 +4313,15 @@
       <c r="Z81" s="6"/>
     </row>
     <row r="82" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A82" s="6"/>
-      <c r="B82" s="6"/>
-      <c r="C82" s="6"/>
+      <c r="A82" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="C82" s="5">
+        <v>46144</v>
+      </c>
       <c r="D82" s="6"/>
       <c r="E82" s="6"/>
       <c r="F82" s="6"/>
@@ -3508,9 +4347,15 @@
       <c r="Z82" s="6"/>
     </row>
     <row r="83" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A83" s="6"/>
-      <c r="B83" s="6"/>
-      <c r="C83" s="6"/>
+      <c r="A83" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C83" s="5">
+        <v>46145</v>
+      </c>
       <c r="D83" s="6"/>
       <c r="E83" s="6"/>
       <c r="F83" s="6"/>
@@ -3536,9 +4381,15 @@
       <c r="Z83" s="6"/>
     </row>
     <row r="84" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A84" s="6"/>
-      <c r="B84" s="6"/>
-      <c r="C84" s="6"/>
+      <c r="A84" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="C84" s="5">
+        <v>46146</v>
+      </c>
       <c r="D84" s="6"/>
       <c r="E84" s="6"/>
       <c r="F84" s="6"/>
@@ -3564,9 +4415,15 @@
       <c r="Z84" s="6"/>
     </row>
     <row r="85" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A85" s="6"/>
-      <c r="B85" s="6"/>
-      <c r="C85" s="6"/>
+      <c r="A85" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="C85" s="5">
+        <v>46147</v>
+      </c>
       <c r="D85" s="6"/>
       <c r="E85" s="6"/>
       <c r="F85" s="6"/>
@@ -27728,6 +28585,7 @@
       <c r="Z947" s="6"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
     <hyperlink ref="A3" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
@@ -27782,6 +28640,37 @@
     <hyperlink ref="A52" r:id="rId51" xr:uid="{00000000-0004-0000-0100-000032000000}"/>
     <hyperlink ref="A53" r:id="rId52" xr:uid="{00000000-0004-0000-0100-000033000000}"/>
     <hyperlink ref="A54" r:id="rId53" xr:uid="{00000000-0004-0000-0100-000034000000}"/>
+    <hyperlink ref="A55" r:id="rId54" xr:uid="{3A251988-9F41-43FB-A5D0-ADD4FC62E139}"/>
+    <hyperlink ref="A56" r:id="rId55" xr:uid="{F63058F2-D825-4ED0-B770-19B7D76E1785}"/>
+    <hyperlink ref="A57" r:id="rId56" xr:uid="{6E09FD5E-EF29-4711-8099-E22B38E3D9AB}"/>
+    <hyperlink ref="A58" r:id="rId57" xr:uid="{7935BADA-1132-4EAA-AFCD-31716FBAC236}"/>
+    <hyperlink ref="A59" r:id="rId58" xr:uid="{556690BD-DF7E-4004-9D15-B539DA0D48D6}"/>
+    <hyperlink ref="A60" r:id="rId59" xr:uid="{95BBBF97-E98A-4E35-96A0-964EE32C9FCF}"/>
+    <hyperlink ref="A61" r:id="rId60" xr:uid="{ED7E98BF-CE27-455F-9A19-6BA591E90AB2}"/>
+    <hyperlink ref="A62" r:id="rId61" xr:uid="{C4515FB7-6256-4F68-AFE1-BA52809D05A8}"/>
+    <hyperlink ref="A63" r:id="rId62" xr:uid="{E904486F-A253-4B0B-8AA5-6B57AC67DF86}"/>
+    <hyperlink ref="A64" r:id="rId63" xr:uid="{56A4B279-F072-4573-8D0F-785CA22C48E1}"/>
+    <hyperlink ref="A65" r:id="rId64" xr:uid="{A9AAB9A2-81CB-4846-B4E2-3FB1C5DBC0F6}"/>
+    <hyperlink ref="A66" r:id="rId65" xr:uid="{212A0F96-4789-48C3-8DB9-5CC15E2097B4}"/>
+    <hyperlink ref="A67" r:id="rId66" xr:uid="{F38DFA64-0A7B-4977-9897-F2B7B8E2A7FD}"/>
+    <hyperlink ref="A68" r:id="rId67" xr:uid="{B0B1C041-A42E-4D9D-ABB1-98E17B80D2B9}"/>
+    <hyperlink ref="A69" r:id="rId68" xr:uid="{A5A4B04C-394F-443B-95AE-F4E061C31747}"/>
+    <hyperlink ref="A70" r:id="rId69" xr:uid="{810037CA-4B1A-44D7-AE10-EBE3E7D162A4}"/>
+    <hyperlink ref="A71" r:id="rId70" xr:uid="{D527B3CA-4DF4-401B-9218-937C3D4767F9}"/>
+    <hyperlink ref="A72" r:id="rId71" xr:uid="{79F9AF66-DBA9-44B7-889B-0D324BEDDF1B}"/>
+    <hyperlink ref="A73" r:id="rId72" xr:uid="{FE11A1E4-63D9-43B3-851E-168CBB55F2EA}"/>
+    <hyperlink ref="A74" r:id="rId73" xr:uid="{3CF17B0E-81CC-409C-A4F7-918331CDC8BC}"/>
+    <hyperlink ref="A75" r:id="rId74" xr:uid="{76832944-A5D1-436B-BEBF-756DDDE3D57D}"/>
+    <hyperlink ref="A76" r:id="rId75" xr:uid="{4F74B0F1-0378-4600-86A7-38D27C60D5C1}"/>
+    <hyperlink ref="A77" r:id="rId76" xr:uid="{DC947359-F695-4833-A375-8DFBC23F5403}"/>
+    <hyperlink ref="A78" r:id="rId77" xr:uid="{D61CA468-F945-432A-AC31-9C164D4B0639}"/>
+    <hyperlink ref="A79" r:id="rId78" xr:uid="{EADB989E-3FEB-490F-963A-8EDD8379A60E}"/>
+    <hyperlink ref="A80" r:id="rId79" xr:uid="{E99E2636-7813-411A-BE61-F800C17BA307}"/>
+    <hyperlink ref="A81" r:id="rId80" xr:uid="{52E94B33-FDF2-49BA-A69D-F26870E2D3A4}"/>
+    <hyperlink ref="A82" r:id="rId81" xr:uid="{911C1B0C-8277-427D-BA7E-4496E05D5C1C}"/>
+    <hyperlink ref="A83" r:id="rId82" xr:uid="{BB554CF1-6E12-4C03-B8AC-C9071BAB1D24}"/>
+    <hyperlink ref="A84" r:id="rId83" xr:uid="{4E4005AA-7A05-4DF6-BF5D-F8BCCE2FB8D9}"/>
+    <hyperlink ref="A85" r:id="rId84" xr:uid="{BB9E547F-469A-49C3-9895-4B1134582C5A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -28380,9 +29269,15 @@
       <c r="Z17" s="6"/>
     </row>
     <row r="18" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="3"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="7"/>
+      <c r="A18" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C18" s="7">
+        <v>46117</v>
+      </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
@@ -28408,9 +29303,15 @@
       <c r="Z18" s="6"/>
     </row>
     <row r="19" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="3"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="7"/>
+      <c r="A19" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="7">
+        <v>46118</v>
+      </c>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
@@ -28436,9 +29337,15 @@
       <c r="Z19" s="6"/>
     </row>
     <row r="20" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="3"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="7"/>
+      <c r="A20" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C20" s="7">
+        <v>46119</v>
+      </c>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
@@ -28464,9 +29371,15 @@
       <c r="Z20" s="6"/>
     </row>
     <row r="21" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="3"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="7"/>
+      <c r="A21" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C21" s="7">
+        <v>46120</v>
+      </c>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
@@ -28492,9 +29405,15 @@
       <c r="Z21" s="6"/>
     </row>
     <row r="22" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="3"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="7"/>
+      <c r="A22" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C22" s="7">
+        <v>46121</v>
+      </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
@@ -28520,9 +29439,15 @@
       <c r="Z22" s="6"/>
     </row>
     <row r="23" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="3"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="7"/>
+      <c r="A23" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C23" s="7">
+        <v>46122</v>
+      </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
       <c r="F23" s="6"/>
@@ -28548,9 +29473,15 @@
       <c r="Z23" s="6"/>
     </row>
     <row r="24" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="3"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="7"/>
+      <c r="A24" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="7">
+        <v>46123</v>
+      </c>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
       <c r="F24" s="6"/>
@@ -28576,9 +29507,15 @@
       <c r="Z24" s="6"/>
     </row>
     <row r="25" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A25" s="3"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="7"/>
+      <c r="A25" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" s="7">
+        <v>46124</v>
+      </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
       <c r="F25" s="6"/>
@@ -28604,9 +29541,15 @@
       <c r="Z25" s="6"/>
     </row>
     <row r="26" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A26" s="3"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="7"/>
+      <c r="A26" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C26" s="7">
+        <v>46125</v>
+      </c>
       <c r="D26" s="6"/>
       <c r="E26" s="6"/>
       <c r="F26" s="6"/>
@@ -28632,9 +29575,15 @@
       <c r="Z26" s="6"/>
     </row>
     <row r="27" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A27" s="3"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="7"/>
+      <c r="A27" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C27" s="7">
+        <v>46126</v>
+      </c>
       <c r="D27" s="6"/>
       <c r="E27" s="6"/>
       <c r="F27" s="6"/>
@@ -28660,9 +29609,15 @@
       <c r="Z27" s="6"/>
     </row>
     <row r="28" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="3"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="7"/>
+      <c r="A28" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C28" s="7">
+        <v>46127</v>
+      </c>
       <c r="D28" s="6"/>
       <c r="E28" s="6"/>
       <c r="F28" s="6"/>
@@ -28688,9 +29643,15 @@
       <c r="Z28" s="6"/>
     </row>
     <row r="29" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A29" s="3"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="7"/>
+      <c r="A29" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C29" s="7">
+        <v>46128</v>
+      </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6"/>
       <c r="F29" s="6"/>
@@ -28716,9 +29677,15 @@
       <c r="Z29" s="6"/>
     </row>
     <row r="30" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A30" s="3"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="7"/>
+      <c r="A30" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C30" s="7">
+        <v>46129</v>
+      </c>
       <c r="D30" s="6"/>
       <c r="E30" s="6"/>
       <c r="F30" s="6"/>
@@ -28744,9 +29711,15 @@
       <c r="Z30" s="6"/>
     </row>
     <row r="31" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A31" s="3"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="7"/>
+      <c r="A31" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C31" s="7">
+        <v>46130</v>
+      </c>
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
@@ -28772,9 +29745,15 @@
       <c r="Z31" s="6"/>
     </row>
     <row r="32" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A32" s="3"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="7"/>
+      <c r="A32" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C32" s="7">
+        <v>46131</v>
+      </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
@@ -28800,9 +29779,15 @@
       <c r="Z32" s="6"/>
     </row>
     <row r="33" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A33" s="3"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="7"/>
+      <c r="A33" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C33" s="7">
+        <v>46132</v>
+      </c>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
       <c r="F33" s="6"/>
@@ -28828,9 +29813,15 @@
       <c r="Z33" s="6"/>
     </row>
     <row r="34" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A34" s="3"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="7"/>
+      <c r="A34" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C34" s="7">
+        <v>46133</v>
+      </c>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
@@ -28856,9 +29847,15 @@
       <c r="Z34" s="6"/>
     </row>
     <row r="35" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A35" s="3"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="7"/>
+      <c r="A35" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C35" s="7">
+        <v>46134</v>
+      </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
@@ -28884,9 +29881,15 @@
       <c r="Z35" s="6"/>
     </row>
     <row r="36" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A36" s="3"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="7"/>
+      <c r="A36" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C36" s="7">
+        <v>46135</v>
+      </c>
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
       <c r="F36" s="6"/>
@@ -28912,9 +29915,15 @@
       <c r="Z36" s="6"/>
     </row>
     <row r="37" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A37" s="3"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="7"/>
+      <c r="A37" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C37" s="7">
+        <v>46136</v>
+      </c>
       <c r="D37" s="6"/>
       <c r="E37" s="6"/>
       <c r="F37" s="6"/>
@@ -28940,9 +29949,15 @@
       <c r="Z37" s="6"/>
     </row>
     <row r="38" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A38" s="3"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="7"/>
+      <c r="A38" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C38" s="7">
+        <v>46137</v>
+      </c>
       <c r="D38" s="6"/>
       <c r="E38" s="6"/>
       <c r="F38" s="6"/>
@@ -28968,9 +29983,15 @@
       <c r="Z38" s="6"/>
     </row>
     <row r="39" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A39" s="3"/>
-      <c r="B39" s="4"/>
-      <c r="C39" s="7"/>
+      <c r="A39" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C39" s="7">
+        <v>46138</v>
+      </c>
       <c r="D39" s="6"/>
       <c r="E39" s="6"/>
       <c r="F39" s="6"/>
@@ -28996,9 +30017,15 @@
       <c r="Z39" s="6"/>
     </row>
     <row r="40" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A40" s="3"/>
-      <c r="B40" s="4"/>
-      <c r="C40" s="7"/>
+      <c r="A40" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C40" s="7">
+        <v>46139</v>
+      </c>
       <c r="D40" s="6"/>
       <c r="E40" s="6"/>
       <c r="F40" s="6"/>
@@ -29024,9 +30051,15 @@
       <c r="Z40" s="6"/>
     </row>
     <row r="41" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A41" s="3"/>
-      <c r="B41" s="4"/>
-      <c r="C41" s="7"/>
+      <c r="A41" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C41" s="7">
+        <v>46140</v>
+      </c>
       <c r="D41" s="6"/>
       <c r="E41" s="6"/>
       <c r="F41" s="6"/>
@@ -29052,9 +30085,15 @@
       <c r="Z41" s="6"/>
     </row>
     <row r="42" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A42" s="3"/>
-      <c r="B42" s="4"/>
-      <c r="C42" s="7"/>
+      <c r="A42" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C42" s="7">
+        <v>46141</v>
+      </c>
       <c r="D42" s="6"/>
       <c r="E42" s="6"/>
       <c r="F42" s="6"/>
@@ -29080,9 +30119,15 @@
       <c r="Z42" s="6"/>
     </row>
     <row r="43" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A43" s="3"/>
-      <c r="B43" s="4"/>
-      <c r="C43" s="7"/>
+      <c r="A43" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C43" s="7">
+        <v>46142</v>
+      </c>
       <c r="D43" s="6"/>
       <c r="E43" s="6"/>
       <c r="F43" s="6"/>
@@ -29108,9 +30153,15 @@
       <c r="Z43" s="6"/>
     </row>
     <row r="44" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A44" s="3"/>
-      <c r="B44" s="4"/>
-      <c r="C44" s="7"/>
+      <c r="A44" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C44" s="7">
+        <v>46143</v>
+      </c>
       <c r="D44" s="6"/>
       <c r="E44" s="6"/>
       <c r="F44" s="6"/>
@@ -29136,9 +30187,15 @@
       <c r="Z44" s="6"/>
     </row>
     <row r="45" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A45" s="3"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="7"/>
+      <c r="A45" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C45" s="7">
+        <v>46144</v>
+      </c>
       <c r="D45" s="6"/>
       <c r="E45" s="6"/>
       <c r="F45" s="6"/>
@@ -29164,9 +30221,15 @@
       <c r="Z45" s="6"/>
     </row>
     <row r="46" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A46" s="3"/>
-      <c r="B46" s="4"/>
-      <c r="C46" s="7"/>
+      <c r="A46" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C46" s="7">
+        <v>46145</v>
+      </c>
       <c r="D46" s="6"/>
       <c r="E46" s="6"/>
       <c r="F46" s="6"/>
@@ -29192,9 +30255,15 @@
       <c r="Z46" s="6"/>
     </row>
     <row r="47" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A47" s="3"/>
-      <c r="B47" s="4"/>
-      <c r="C47" s="7"/>
+      <c r="A47" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C47" s="7">
+        <v>46146</v>
+      </c>
       <c r="D47" s="6"/>
       <c r="E47" s="6"/>
       <c r="F47" s="6"/>
@@ -29220,9 +30289,15 @@
       <c r="Z47" s="6"/>
     </row>
     <row r="48" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A48" s="3"/>
-      <c r="B48" s="4"/>
-      <c r="C48" s="7"/>
+      <c r="A48" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C48" s="7">
+        <v>46147</v>
+      </c>
       <c r="D48" s="6"/>
       <c r="E48" s="6"/>
       <c r="F48" s="6"/>
@@ -54420,6 +55495,7 @@
       <c r="Z947" s="6"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{01621AAE-AE4A-4198-951B-0760787D2375}"/>
     <hyperlink ref="A3" r:id="rId2" xr:uid="{8B4ED3DE-230D-4C09-B0D3-61E231B9A40B}"/>
@@ -54437,6 +55513,37 @@
     <hyperlink ref="A15" r:id="rId14" xr:uid="{F822B1D8-D450-4261-8381-81990360F0F1}"/>
     <hyperlink ref="A16" r:id="rId15" xr:uid="{2A04457A-4EFB-4DE1-89C6-6D311DABB927}"/>
     <hyperlink ref="A17" r:id="rId16" xr:uid="{FE0C0D25-AAFA-4F23-A1E7-5157852EB968}"/>
+    <hyperlink ref="A18" r:id="rId17" xr:uid="{2EE89E9C-9DB4-4C32-9D11-C996449C82E3}"/>
+    <hyperlink ref="A19" r:id="rId18" xr:uid="{0EACFF13-28B5-4F6C-8B7F-7505230A64D4}"/>
+    <hyperlink ref="A20" r:id="rId19" xr:uid="{25C252F8-FEB4-464F-9533-C954234CE058}"/>
+    <hyperlink ref="A21" r:id="rId20" xr:uid="{AA9264A4-D635-44B0-8E07-A41C689A0348}"/>
+    <hyperlink ref="A22" r:id="rId21" xr:uid="{09D23F55-69B7-4CEA-8608-94467165AF78}"/>
+    <hyperlink ref="A23" r:id="rId22" xr:uid="{0A6D18A9-0A53-4CBE-876E-72A26F74B4ED}"/>
+    <hyperlink ref="A24" r:id="rId23" xr:uid="{C62B07D9-78D9-4010-8D9C-BD4C7E524B4B}"/>
+    <hyperlink ref="A25" r:id="rId24" xr:uid="{098118F1-C567-42EB-A4C4-8B45A3450512}"/>
+    <hyperlink ref="A26" r:id="rId25" xr:uid="{F335F155-10DE-4D5E-8580-993874609686}"/>
+    <hyperlink ref="A27" r:id="rId26" xr:uid="{5D134E65-9F5D-41D5-83E9-D441626CCA9B}"/>
+    <hyperlink ref="A28" r:id="rId27" xr:uid="{159637D1-73A1-4BAF-8B86-9DF6A72EEF34}"/>
+    <hyperlink ref="A29" r:id="rId28" xr:uid="{7FF4A5C9-F372-48A4-B832-8D1AEE58688A}"/>
+    <hyperlink ref="A30" r:id="rId29" xr:uid="{07A3026E-D5EE-4E21-BF58-5ECFC3F896B0}"/>
+    <hyperlink ref="A31" r:id="rId30" xr:uid="{F8DE7E85-D524-4D0E-9888-3805DEAE94FA}"/>
+    <hyperlink ref="A32" r:id="rId31" xr:uid="{6E63D312-F1C7-4165-85CB-70FABACF16F3}"/>
+    <hyperlink ref="A33" r:id="rId32" xr:uid="{855ED130-7931-4052-98BE-F17A0B9DACF5}"/>
+    <hyperlink ref="A34" r:id="rId33" xr:uid="{BAE47839-1C44-4EEB-A7F8-82777D0C4455}"/>
+    <hyperlink ref="A35" r:id="rId34" xr:uid="{DF33ED01-4268-4D81-B7E2-0A52CECFC677}"/>
+    <hyperlink ref="A36" r:id="rId35" xr:uid="{BE855F4A-FA72-4FA2-9DAC-66175273D93F}"/>
+    <hyperlink ref="A37" r:id="rId36" xr:uid="{AD5B12ED-8D15-4EAB-93A3-F5361F012D04}"/>
+    <hyperlink ref="A38" r:id="rId37" xr:uid="{1B5F7E60-5776-412A-8344-8FB5AA3309F4}"/>
+    <hyperlink ref="A39" r:id="rId38" xr:uid="{9D85CEBD-FB3F-4B5F-9BF9-422A1DCBA366}"/>
+    <hyperlink ref="A40" r:id="rId39" xr:uid="{8858C27B-FF73-4A11-9B96-9F5D2A7F9FD9}"/>
+    <hyperlink ref="A41" r:id="rId40" xr:uid="{3AD85FF3-77DD-4528-92DB-2AFF576E14F0}"/>
+    <hyperlink ref="A42" r:id="rId41" xr:uid="{8357E95A-C959-4CA0-A48D-E2C14292636D}"/>
+    <hyperlink ref="A43" r:id="rId42" xr:uid="{22BFD094-B499-4A83-83E2-E9BC25A807D0}"/>
+    <hyperlink ref="A44" r:id="rId43" xr:uid="{F099416F-193D-4AA5-8DA1-842E122B4EDE}"/>
+    <hyperlink ref="A45" r:id="rId44" xr:uid="{3660A77B-522D-45BA-9838-2322347B8B67}"/>
+    <hyperlink ref="A46" r:id="rId45" xr:uid="{562F6695-A679-4430-BF00-4378A4968B67}"/>
+    <hyperlink ref="A47" r:id="rId46" xr:uid="{FD905F37-8316-4227-8463-302ED81CEA43}"/>
+    <hyperlink ref="A48" r:id="rId47" xr:uid="{44B510CF-CF69-4DA2-B4F2-A4CAB2CBAB43}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
more daily sadhana added
</commit_message>
<xml_diff>
--- a/public/Daily Sadhana.xlsx
+++ b/public/Daily Sadhana.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sahaa\OneDrive\Documents\github_anandasvarupa\give_web\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sahaa\Documents\github_anandasvarupa\give_web\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{202FD920-C4B1-4571-A2F3-94C1937C2E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4964C7EC-F501-41A3-A220-DE168442A2EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BS-4" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="286">
   <si>
     <t>url</t>
   </si>
@@ -661,6 +661,231 @@
   <si>
     <t>Today's listening to Srila Prabhupada - 84</t>
   </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=CPz96HMqmRQ</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Ry6zwPcHuDE</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=P6WPgfCgEeU</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Uo7y3wdEdOc</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ayP6KACfqKk</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=yfgNfdHS4Mc</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=q2hjaNiTGNo</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=y4NDqYSxHFg</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Act0uDxqPzA</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=-in9otdV6X4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=k5rmD05dV54</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=z1V7smrwi5s</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=0UdMNxMppUY</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=DRajsrs28_s</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=b3q0expa3Xc</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=eBgq4V__Rqw</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=IhjVWsWrMSA</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=mRv3pWamUPs</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=qeUSRLl-FXI</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=-xcosp9cVgk</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=QH8Ywe3DJ-I</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=UPUPeFC9Xc4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=YxUIT_yaG_o</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=JUF1tiHYI58</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=06zHOMSXea0</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=9HZggjR_zFY</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=A8stQbXrzF4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=BstmUna371g</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=hkBkq0JLArE</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=5oWm9kpFm1g</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 85</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 86</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 87</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 88</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 89</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 90</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 91</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 92</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 93</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 94</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 95</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 96</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 97</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 98</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 99</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 137</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 138</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 139</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 140</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 141</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 142</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 143</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 144</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 145</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 146</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 147</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 148</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 149</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 150</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 151</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 152</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 153</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 154</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 155</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 156</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 157</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 158</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 159</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 160</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 161</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 162</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 163</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 164</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 165</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 166</t>
+  </si>
 </sst>
 </file>
 
@@ -724,7 +949,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -732,12 +957,72 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -764,6 +1049,18 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -989,7 +1286,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z43"/>
+  <dimension ref="A1:Z73"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="56.81640625" customWidth="1"/>
@@ -1482,7 +1779,7 @@
         <v>46146</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="9" t="s">
         <v>148</v>
       </c>
@@ -1491,6 +1788,336 @@
       </c>
       <c r="C43" s="5">
         <v>46147</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="C44" s="5">
+        <v>46148</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="11" t="s">
+        <v>212</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="C45" s="5">
+        <v>46149</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="C46" s="5">
+        <v>46150</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C47" s="5">
+        <v>46151</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="C48" s="5">
+        <v>46152</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="C49" s="5">
+        <v>46153</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="C50" s="5">
+        <v>46154</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="C51" s="5">
+        <v>46155</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="C52" s="5">
+        <v>46156</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="C53" s="5">
+        <v>46157</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="C54" s="5">
+        <v>46158</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="C55" s="5">
+        <v>46159</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="C56" s="5">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="C57" s="5">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="13" t="s">
+        <v>225</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="C58" s="5">
+        <v>46162</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C59" s="5">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="C60" s="5">
+        <v>46164</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="C61" s="5">
+        <v>46165</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="C62" s="5">
+        <v>46166</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="C63" s="5">
+        <v>46167</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="C64" s="5">
+        <v>46168</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="C65" s="5">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="C66" s="5">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="C67" s="5">
+        <v>46171</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="C68" s="5">
+        <v>46172</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="C69" s="5">
+        <v>46173</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="C70" s="5">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="C71" s="5">
+        <v>46175</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="C72" s="5">
+        <v>46176</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="C73" s="5">
+        <v>46177</v>
       </c>
     </row>
   </sheetData>
@@ -1538,9 +2165,39 @@
     <hyperlink ref="A41" r:id="rId40" xr:uid="{66D88341-E233-40C7-A0F1-8E34AE93A867}"/>
     <hyperlink ref="A42" r:id="rId41" xr:uid="{5DA0CFD4-768B-49CC-A3CC-6F8D00361B4A}"/>
     <hyperlink ref="A43" r:id="rId42" xr:uid="{A11DA0CB-FD50-471B-9BFA-F61671963A09}"/>
+    <hyperlink ref="A44" r:id="rId43" xr:uid="{03C4C452-8153-4BF7-9836-DEB94128F4BE}"/>
+    <hyperlink ref="A45" r:id="rId44" xr:uid="{33234097-0E8D-4BD2-A8AB-88FA06F4D450}"/>
+    <hyperlink ref="A46" r:id="rId45" xr:uid="{E23FF7AF-A55E-4F92-BB8E-9924902EAA27}"/>
+    <hyperlink ref="A47" r:id="rId46" xr:uid="{2CA2FC0D-90C2-4147-B9E7-7B3A4EDA8C70}"/>
+    <hyperlink ref="A48" r:id="rId47" xr:uid="{97492F2C-C20C-4B17-8A9B-6551908001A3}"/>
+    <hyperlink ref="A49" r:id="rId48" xr:uid="{FBF619AE-2313-47C0-A1C2-C2653F49ABBA}"/>
+    <hyperlink ref="A50" r:id="rId49" xr:uid="{91596DF6-5734-4D56-9D5E-4AE488A35E77}"/>
+    <hyperlink ref="A51" r:id="rId50" xr:uid="{94B27AD5-D929-4027-A9A6-F3D501B14EDD}"/>
+    <hyperlink ref="A52" r:id="rId51" xr:uid="{A99A5454-CE98-416E-851B-7525AA28B785}"/>
+    <hyperlink ref="A53" r:id="rId52" xr:uid="{96A78ECA-8184-4059-85E4-5EE564AB648C}"/>
+    <hyperlink ref="A54" r:id="rId53" xr:uid="{ACC3824B-30AD-49FE-979A-74A7EB4AB1EE}"/>
+    <hyperlink ref="A55" r:id="rId54" xr:uid="{E8F9C8D6-706C-4346-8AD7-66057749C235}"/>
+    <hyperlink ref="A56" r:id="rId55" xr:uid="{41ADB383-9C97-490F-A58B-AFA42CE2EB74}"/>
+    <hyperlink ref="A57" r:id="rId56" xr:uid="{61E2365E-FEA3-4E94-A63D-0C7EC3BF542E}"/>
+    <hyperlink ref="A58" r:id="rId57" xr:uid="{D2A0A82F-0F1D-4D87-90F8-ED9C0331993D}"/>
+    <hyperlink ref="A59" r:id="rId58" xr:uid="{C6D32A8B-2E78-4B22-A1E6-0FD78D6BF64E}"/>
+    <hyperlink ref="A60" r:id="rId59" xr:uid="{9F98F4A2-4445-4FE8-93BF-D58275146EF9}"/>
+    <hyperlink ref="A61" r:id="rId60" xr:uid="{15005286-75DF-49E3-A88C-26DD4D6C1B0D}"/>
+    <hyperlink ref="A62" r:id="rId61" xr:uid="{959FE6AB-ED0A-42A4-8F40-D8429B62F310}"/>
+    <hyperlink ref="A63" r:id="rId62" xr:uid="{E617E831-8BEF-4680-9F50-F1C1806ECDC8}"/>
+    <hyperlink ref="A64" r:id="rId63" xr:uid="{C6D139F9-4558-4CE6-B4F5-168860047A03}"/>
+    <hyperlink ref="A65" r:id="rId64" xr:uid="{CE6F748C-AC28-4802-9155-9DC4E21AB4F9}"/>
+    <hyperlink ref="A66" r:id="rId65" xr:uid="{196BFBA2-3D7D-40B0-96A2-8AA734648C7B}"/>
+    <hyperlink ref="A67" r:id="rId66" xr:uid="{ABD891DD-8608-473A-91B7-26258DA5B0DA}"/>
+    <hyperlink ref="A68" r:id="rId67" xr:uid="{D7035041-8FF7-49AF-8999-3445A07B7EDA}"/>
+    <hyperlink ref="A69" r:id="rId68" xr:uid="{3BAD04EC-6111-4044-9C3D-A2E2C7A32F24}"/>
+    <hyperlink ref="A70" r:id="rId69" xr:uid="{821EA2B2-A007-49D0-A037-4CA25B3E21E1}"/>
+    <hyperlink ref="A71" r:id="rId70" xr:uid="{68C69F41-91D9-4109-B186-0401363D2F1C}"/>
+    <hyperlink ref="A72" r:id="rId71" xr:uid="{B26834E6-4244-449F-8BCE-66D19D0721D4}"/>
+    <hyperlink ref="A73" r:id="rId72" xr:uid="{C7ECCC81-082C-4F50-8852-6FD10D4C935E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId43"/>
+  <pageSetup orientation="portrait" r:id="rId73"/>
 </worksheet>
 </file>
 
@@ -4414,7 +5071,7 @@
       <c r="Y84" s="6"/>
       <c r="Z84" s="6"/>
     </row>
-    <row r="85" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="9" t="s">
         <v>148</v>
       </c>
@@ -4448,10 +5105,16 @@
       <c r="Y85" s="6"/>
       <c r="Z85" s="6"/>
     </row>
-    <row r="86" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A86" s="6"/>
-      <c r="B86" s="6"/>
-      <c r="C86" s="6"/>
+    <row r="86" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="C86" s="5">
+        <v>46148</v>
+      </c>
       <c r="D86" s="6"/>
       <c r="E86" s="6"/>
       <c r="F86" s="6"/>
@@ -4476,10 +5139,16 @@
       <c r="Y86" s="6"/>
       <c r="Z86" s="6"/>
     </row>
-    <row r="87" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A87" s="6"/>
-      <c r="B87" s="6"/>
-      <c r="C87" s="6"/>
+    <row r="87" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="11" t="s">
+        <v>212</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="C87" s="5">
+        <v>46149</v>
+      </c>
       <c r="D87" s="6"/>
       <c r="E87" s="6"/>
       <c r="F87" s="6"/>
@@ -4504,10 +5173,16 @@
       <c r="Y87" s="6"/>
       <c r="Z87" s="6"/>
     </row>
-    <row r="88" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A88" s="6"/>
-      <c r="B88" s="6"/>
-      <c r="C88" s="6"/>
+    <row r="88" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="C88" s="5">
+        <v>46150</v>
+      </c>
       <c r="D88" s="6"/>
       <c r="E88" s="6"/>
       <c r="F88" s="6"/>
@@ -4532,10 +5207,16 @@
       <c r="Y88" s="6"/>
       <c r="Z88" s="6"/>
     </row>
-    <row r="89" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A89" s="6"/>
-      <c r="B89" s="6"/>
-      <c r="C89" s="6"/>
+    <row r="89" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="C89" s="5">
+        <v>46151</v>
+      </c>
       <c r="D89" s="6"/>
       <c r="E89" s="6"/>
       <c r="F89" s="6"/>
@@ -4560,10 +5241,16 @@
       <c r="Y89" s="6"/>
       <c r="Z89" s="6"/>
     </row>
-    <row r="90" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A90" s="6"/>
-      <c r="B90" s="6"/>
-      <c r="C90" s="6"/>
+    <row r="90" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="C90" s="5">
+        <v>46152</v>
+      </c>
       <c r="D90" s="6"/>
       <c r="E90" s="6"/>
       <c r="F90" s="6"/>
@@ -4588,10 +5275,16 @@
       <c r="Y90" s="6"/>
       <c r="Z90" s="6"/>
     </row>
-    <row r="91" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A91" s="6"/>
-      <c r="B91" s="6"/>
-      <c r="C91" s="6"/>
+    <row r="91" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="C91" s="5">
+        <v>46153</v>
+      </c>
       <c r="D91" s="6"/>
       <c r="E91" s="6"/>
       <c r="F91" s="6"/>
@@ -4616,10 +5309,16 @@
       <c r="Y91" s="6"/>
       <c r="Z91" s="6"/>
     </row>
-    <row r="92" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A92" s="6"/>
-      <c r="B92" s="6"/>
-      <c r="C92" s="6"/>
+    <row r="92" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="C92" s="5">
+        <v>46154</v>
+      </c>
       <c r="D92" s="6"/>
       <c r="E92" s="6"/>
       <c r="F92" s="6"/>
@@ -4644,10 +5343,16 @@
       <c r="Y92" s="6"/>
       <c r="Z92" s="6"/>
     </row>
-    <row r="93" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A93" s="6"/>
-      <c r="B93" s="6"/>
-      <c r="C93" s="6"/>
+    <row r="93" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="B93" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="C93" s="5">
+        <v>46155</v>
+      </c>
       <c r="D93" s="6"/>
       <c r="E93" s="6"/>
       <c r="F93" s="6"/>
@@ -4672,10 +5377,16 @@
       <c r="Y93" s="6"/>
       <c r="Z93" s="6"/>
     </row>
-    <row r="94" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A94" s="6"/>
-      <c r="B94" s="6"/>
-      <c r="C94" s="6"/>
+    <row r="94" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="B94" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="C94" s="5">
+        <v>46156</v>
+      </c>
       <c r="D94" s="6"/>
       <c r="E94" s="6"/>
       <c r="F94" s="6"/>
@@ -4700,10 +5411,16 @@
       <c r="Y94" s="6"/>
       <c r="Z94" s="6"/>
     </row>
-    <row r="95" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A95" s="6"/>
-      <c r="B95" s="6"/>
-      <c r="C95" s="6"/>
+    <row r="95" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="C95" s="5">
+        <v>46157</v>
+      </c>
       <c r="D95" s="6"/>
       <c r="E95" s="6"/>
       <c r="F95" s="6"/>
@@ -4728,10 +5445,16 @@
       <c r="Y95" s="6"/>
       <c r="Z95" s="6"/>
     </row>
-    <row r="96" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A96" s="6"/>
-      <c r="B96" s="6"/>
-      <c r="C96" s="6"/>
+    <row r="96" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="B96" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C96" s="5">
+        <v>46158</v>
+      </c>
       <c r="D96" s="6"/>
       <c r="E96" s="6"/>
       <c r="F96" s="6"/>
@@ -4756,10 +5479,16 @@
       <c r="Y96" s="6"/>
       <c r="Z96" s="6"/>
     </row>
-    <row r="97" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A97" s="6"/>
-      <c r="B97" s="6"/>
-      <c r="C97" s="6"/>
+    <row r="97" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="B97" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="C97" s="5">
+        <v>46159</v>
+      </c>
       <c r="D97" s="6"/>
       <c r="E97" s="6"/>
       <c r="F97" s="6"/>
@@ -4784,10 +5513,16 @@
       <c r="Y97" s="6"/>
       <c r="Z97" s="6"/>
     </row>
-    <row r="98" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A98" s="6"/>
-      <c r="B98" s="6"/>
-      <c r="C98" s="6"/>
+    <row r="98" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="B98" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="C98" s="5">
+        <v>46160</v>
+      </c>
       <c r="D98" s="6"/>
       <c r="E98" s="6"/>
       <c r="F98" s="6"/>
@@ -4812,10 +5547,16 @@
       <c r="Y98" s="6"/>
       <c r="Z98" s="6"/>
     </row>
-    <row r="99" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A99" s="6"/>
-      <c r="B99" s="6"/>
-      <c r="C99" s="6"/>
+    <row r="99" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="B99" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="C99" s="5">
+        <v>46161</v>
+      </c>
       <c r="D99" s="6"/>
       <c r="E99" s="6"/>
       <c r="F99" s="6"/>
@@ -4840,10 +5581,16 @@
       <c r="Y99" s="6"/>
       <c r="Z99" s="6"/>
     </row>
-    <row r="100" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A100" s="6"/>
-      <c r="B100" s="6"/>
-      <c r="C100" s="6"/>
+    <row r="100" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="13" t="s">
+        <v>225</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="C100" s="5">
+        <v>46162</v>
+      </c>
       <c r="D100" s="6"/>
       <c r="E100" s="6"/>
       <c r="F100" s="6"/>
@@ -4868,10 +5615,16 @@
       <c r="Y100" s="6"/>
       <c r="Z100" s="6"/>
     </row>
-    <row r="101" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A101" s="6"/>
-      <c r="B101" s="6"/>
-      <c r="C101" s="6"/>
+    <row r="101" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C101" s="5">
+        <v>46163</v>
+      </c>
       <c r="D101" s="6"/>
       <c r="E101" s="6"/>
       <c r="F101" s="6"/>
@@ -4896,10 +5649,16 @@
       <c r="Y101" s="6"/>
       <c r="Z101" s="6"/>
     </row>
-    <row r="102" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A102" s="6"/>
-      <c r="B102" s="6"/>
-      <c r="C102" s="6"/>
+    <row r="102" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="B102" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C102" s="5">
+        <v>46164</v>
+      </c>
       <c r="D102" s="6"/>
       <c r="E102" s="6"/>
       <c r="F102" s="6"/>
@@ -4924,10 +5683,16 @@
       <c r="Y102" s="6"/>
       <c r="Z102" s="6"/>
     </row>
-    <row r="103" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A103" s="6"/>
-      <c r="B103" s="6"/>
-      <c r="C103" s="6"/>
+    <row r="103" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="B103" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C103" s="5">
+        <v>46165</v>
+      </c>
       <c r="D103" s="6"/>
       <c r="E103" s="6"/>
       <c r="F103" s="6"/>
@@ -4952,10 +5717,16 @@
       <c r="Y103" s="6"/>
       <c r="Z103" s="6"/>
     </row>
-    <row r="104" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A104" s="6"/>
-      <c r="B104" s="6"/>
-      <c r="C104" s="6"/>
+    <row r="104" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="B104" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C104" s="5">
+        <v>46166</v>
+      </c>
       <c r="D104" s="6"/>
       <c r="E104" s="6"/>
       <c r="F104" s="6"/>
@@ -4980,10 +5751,16 @@
       <c r="Y104" s="6"/>
       <c r="Z104" s="6"/>
     </row>
-    <row r="105" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A105" s="6"/>
-      <c r="B105" s="6"/>
-      <c r="C105" s="6"/>
+    <row r="105" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A105" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="B105" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C105" s="5">
+        <v>46167</v>
+      </c>
       <c r="D105" s="6"/>
       <c r="E105" s="6"/>
       <c r="F105" s="6"/>
@@ -5008,10 +5785,16 @@
       <c r="Y105" s="6"/>
       <c r="Z105" s="6"/>
     </row>
-    <row r="106" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A106" s="6"/>
-      <c r="B106" s="6"/>
-      <c r="C106" s="6"/>
+    <row r="106" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A106" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="B106" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C106" s="5">
+        <v>46168</v>
+      </c>
       <c r="D106" s="6"/>
       <c r="E106" s="6"/>
       <c r="F106" s="6"/>
@@ -5036,10 +5819,16 @@
       <c r="Y106" s="6"/>
       <c r="Z106" s="6"/>
     </row>
-    <row r="107" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A107" s="6"/>
-      <c r="B107" s="6"/>
-      <c r="C107" s="6"/>
+    <row r="107" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A107" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="B107" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="C107" s="5">
+        <v>46169</v>
+      </c>
       <c r="D107" s="6"/>
       <c r="E107" s="6"/>
       <c r="F107" s="6"/>
@@ -5064,10 +5853,16 @@
       <c r="Y107" s="6"/>
       <c r="Z107" s="6"/>
     </row>
-    <row r="108" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A108" s="6"/>
-      <c r="B108" s="6"/>
-      <c r="C108" s="6"/>
+    <row r="108" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A108" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="B108" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="C108" s="5">
+        <v>46170</v>
+      </c>
       <c r="D108" s="6"/>
       <c r="E108" s="6"/>
       <c r="F108" s="6"/>
@@ -5092,10 +5887,16 @@
       <c r="Y108" s="6"/>
       <c r="Z108" s="6"/>
     </row>
-    <row r="109" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A109" s="6"/>
-      <c r="B109" s="6"/>
-      <c r="C109" s="6"/>
+    <row r="109" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A109" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="B109" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="C109" s="5">
+        <v>46171</v>
+      </c>
       <c r="D109" s="6"/>
       <c r="E109" s="6"/>
       <c r="F109" s="6"/>
@@ -5120,10 +5921,16 @@
       <c r="Y109" s="6"/>
       <c r="Z109" s="6"/>
     </row>
-    <row r="110" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A110" s="6"/>
-      <c r="B110" s="6"/>
-      <c r="C110" s="6"/>
+    <row r="110" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A110" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="B110" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C110" s="5">
+        <v>46172</v>
+      </c>
       <c r="D110" s="6"/>
       <c r="E110" s="6"/>
       <c r="F110" s="6"/>
@@ -5148,10 +5955,16 @@
       <c r="Y110" s="6"/>
       <c r="Z110" s="6"/>
     </row>
-    <row r="111" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A111" s="6"/>
-      <c r="B111" s="6"/>
-      <c r="C111" s="6"/>
+    <row r="111" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A111" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="B111" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C111" s="5">
+        <v>46173</v>
+      </c>
       <c r="D111" s="6"/>
       <c r="E111" s="6"/>
       <c r="F111" s="6"/>
@@ -5176,10 +5989,16 @@
       <c r="Y111" s="6"/>
       <c r="Z111" s="6"/>
     </row>
-    <row r="112" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A112" s="6"/>
-      <c r="B112" s="6"/>
-      <c r="C112" s="6"/>
+    <row r="112" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A112" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="B112" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="C112" s="5">
+        <v>46174</v>
+      </c>
       <c r="D112" s="6"/>
       <c r="E112" s="6"/>
       <c r="F112" s="6"/>
@@ -5204,10 +6023,16 @@
       <c r="Y112" s="6"/>
       <c r="Z112" s="6"/>
     </row>
-    <row r="113" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A113" s="6"/>
-      <c r="B113" s="6"/>
-      <c r="C113" s="6"/>
+    <row r="113" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A113" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="B113" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="C113" s="5">
+        <v>46175</v>
+      </c>
       <c r="D113" s="6"/>
       <c r="E113" s="6"/>
       <c r="F113" s="6"/>
@@ -5232,10 +6057,16 @@
       <c r="Y113" s="6"/>
       <c r="Z113" s="6"/>
     </row>
-    <row r="114" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A114" s="6"/>
-      <c r="B114" s="6"/>
-      <c r="C114" s="6"/>
+    <row r="114" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A114" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="B114" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C114" s="5">
+        <v>46176</v>
+      </c>
       <c r="D114" s="6"/>
       <c r="E114" s="6"/>
       <c r="F114" s="6"/>
@@ -5260,10 +6091,16 @@
       <c r="Y114" s="6"/>
       <c r="Z114" s="6"/>
     </row>
-    <row r="115" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A115" s="6"/>
-      <c r="B115" s="6"/>
-      <c r="C115" s="6"/>
+    <row r="115" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A115" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="B115" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="C115" s="5">
+        <v>46177</v>
+      </c>
       <c r="D115" s="6"/>
       <c r="E115" s="6"/>
       <c r="F115" s="6"/>
@@ -28671,8 +29508,39 @@
     <hyperlink ref="A83" r:id="rId82" xr:uid="{BB554CF1-6E12-4C03-B8AC-C9071BAB1D24}"/>
     <hyperlink ref="A84" r:id="rId83" xr:uid="{4E4005AA-7A05-4DF6-BF5D-F8BCCE2FB8D9}"/>
     <hyperlink ref="A85" r:id="rId84" xr:uid="{BB9E547F-469A-49C3-9895-4B1134582C5A}"/>
+    <hyperlink ref="A86" r:id="rId85" xr:uid="{76D8295F-DF07-469B-9095-44A7CCF63CF4}"/>
+    <hyperlink ref="A87" r:id="rId86" xr:uid="{919107AF-0D87-4920-8580-F0BE6FCA140A}"/>
+    <hyperlink ref="A88" r:id="rId87" xr:uid="{19E5BA0C-6E62-44BA-A4F7-EC281EE621DC}"/>
+    <hyperlink ref="A89" r:id="rId88" xr:uid="{53FE2AFF-AF47-414B-B338-39D1FDA6B0E9}"/>
+    <hyperlink ref="A90" r:id="rId89" xr:uid="{954CEDFD-532B-411B-AFDA-605B0C3446C7}"/>
+    <hyperlink ref="A91" r:id="rId90" xr:uid="{E7019686-5E2D-4335-A436-597FCEE34E59}"/>
+    <hyperlink ref="A92" r:id="rId91" xr:uid="{65DCBC55-7FB9-441D-B41D-5725BB861AAA}"/>
+    <hyperlink ref="A93" r:id="rId92" xr:uid="{F7276512-7067-4BDB-BA45-E679FB83B6E7}"/>
+    <hyperlink ref="A94" r:id="rId93" xr:uid="{4749CE69-73B9-400D-A973-E77F8AD7B1E4}"/>
+    <hyperlink ref="A95" r:id="rId94" xr:uid="{A479A846-AAD4-4F07-93F6-429A7B2830D1}"/>
+    <hyperlink ref="A96" r:id="rId95" xr:uid="{FF422D6E-BE7F-4C00-8655-ACB559A62F58}"/>
+    <hyperlink ref="A97" r:id="rId96" xr:uid="{7BFD9F54-15B0-48F5-A647-1139CB51A025}"/>
+    <hyperlink ref="A98" r:id="rId97" xr:uid="{65B1EBAD-4D12-4125-9E6E-8F4600CE48F2}"/>
+    <hyperlink ref="A99" r:id="rId98" xr:uid="{EC400486-DA1D-4BDD-B1AB-01FA1E39F082}"/>
+    <hyperlink ref="A100" r:id="rId99" xr:uid="{131D7CA3-EE3D-48F4-AB30-B8399B85653B}"/>
+    <hyperlink ref="A101" r:id="rId100" xr:uid="{AA95B318-ACC5-4133-9BF1-8A508A13A13A}"/>
+    <hyperlink ref="A102" r:id="rId101" xr:uid="{11F5A7C6-3138-4AE5-BCB5-37E261D8E633}"/>
+    <hyperlink ref="A103" r:id="rId102" xr:uid="{5DC5A7BD-5519-4B9B-A23C-06970C147AC8}"/>
+    <hyperlink ref="A104" r:id="rId103" xr:uid="{11A214C9-12FE-4CAB-8896-0FA9EDCD053C}"/>
+    <hyperlink ref="A105" r:id="rId104" xr:uid="{5A936A0F-3398-4659-B2A5-91F610336228}"/>
+    <hyperlink ref="A106" r:id="rId105" xr:uid="{5B6A3540-B9F0-405F-93D0-154E2929213E}"/>
+    <hyperlink ref="A107" r:id="rId106" xr:uid="{A941ABC6-CD06-40DC-87A3-E44BFC79B392}"/>
+    <hyperlink ref="A108" r:id="rId107" xr:uid="{D69B4B9B-F87D-4F77-9615-CBB6D2028D10}"/>
+    <hyperlink ref="A109" r:id="rId108" xr:uid="{3C1CBC17-D8B6-4AA1-A02E-6A8153804B7A}"/>
+    <hyperlink ref="A110" r:id="rId109" xr:uid="{08556FCF-F59B-4CA7-A4D0-9BE2B24B9BB5}"/>
+    <hyperlink ref="A111" r:id="rId110" xr:uid="{6B6CF554-4A9B-4AA8-BADD-591FEECC05C9}"/>
+    <hyperlink ref="A112" r:id="rId111" xr:uid="{7A4538F7-CE73-442F-8328-E4AD370A1CBE}"/>
+    <hyperlink ref="A113" r:id="rId112" xr:uid="{D12CF023-7448-4AC2-B7FB-1284C1269E70}"/>
+    <hyperlink ref="A114" r:id="rId113" xr:uid="{C30B01CE-4989-4ECD-80C5-EDBAE8EFD21B}"/>
+    <hyperlink ref="A115" r:id="rId114" xr:uid="{6C99A764-2055-4805-923C-CC469CD6B5FE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId115"/>
 </worksheet>
 </file>
 
@@ -30288,7 +31156,7 @@
       <c r="Y47" s="6"/>
       <c r="Z47" s="6"/>
     </row>
-    <row r="48" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="9" t="s">
         <v>148</v>
       </c>
@@ -30322,10 +31190,16 @@
       <c r="Y48" s="6"/>
       <c r="Z48" s="6"/>
     </row>
-    <row r="49" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A49" s="3"/>
-      <c r="B49" s="4"/>
-      <c r="C49" s="7"/>
+    <row r="49" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C49" s="7">
+        <v>46148</v>
+      </c>
       <c r="D49" s="6"/>
       <c r="E49" s="6"/>
       <c r="F49" s="6"/>
@@ -30350,10 +31224,16 @@
       <c r="Y49" s="6"/>
       <c r="Z49" s="6"/>
     </row>
-    <row r="50" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A50" s="3"/>
-      <c r="B50" s="4"/>
-      <c r="C50" s="7"/>
+    <row r="50" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="11" t="s">
+        <v>212</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C50" s="7">
+        <v>46149</v>
+      </c>
       <c r="D50" s="6"/>
       <c r="E50" s="6"/>
       <c r="F50" s="6"/>
@@ -30378,10 +31258,16 @@
       <c r="Y50" s="6"/>
       <c r="Z50" s="6"/>
     </row>
-    <row r="51" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A51" s="3"/>
-      <c r="B51" s="4"/>
-      <c r="C51" s="7"/>
+    <row r="51" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C51" s="7">
+        <v>46150</v>
+      </c>
       <c r="D51" s="6"/>
       <c r="E51" s="6"/>
       <c r="F51" s="6"/>
@@ -30406,10 +31292,16 @@
       <c r="Y51" s="6"/>
       <c r="Z51" s="6"/>
     </row>
-    <row r="52" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A52" s="3"/>
-      <c r="B52" s="4"/>
-      <c r="C52" s="7"/>
+    <row r="52" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C52" s="7">
+        <v>46151</v>
+      </c>
       <c r="D52" s="6"/>
       <c r="E52" s="6"/>
       <c r="F52" s="6"/>
@@ -30434,10 +31326,16 @@
       <c r="Y52" s="6"/>
       <c r="Z52" s="6"/>
     </row>
-    <row r="53" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A53" s="3"/>
-      <c r="B53" s="4"/>
-      <c r="C53" s="7"/>
+    <row r="53" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="C53" s="7">
+        <v>46152</v>
+      </c>
       <c r="D53" s="6"/>
       <c r="E53" s="6"/>
       <c r="F53" s="6"/>
@@ -30462,10 +31360,16 @@
       <c r="Y53" s="6"/>
       <c r="Z53" s="6"/>
     </row>
-    <row r="54" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A54" s="3"/>
-      <c r="B54" s="4"/>
-      <c r="C54" s="7"/>
+    <row r="54" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C54" s="7">
+        <v>46153</v>
+      </c>
       <c r="D54" s="6"/>
       <c r="E54" s="6"/>
       <c r="F54" s="6"/>
@@ -30490,10 +31394,16 @@
       <c r="Y54" s="6"/>
       <c r="Z54" s="6"/>
     </row>
-    <row r="55" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A55" s="6"/>
-      <c r="B55" s="6"/>
-      <c r="C55" s="8"/>
+    <row r="55" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="C55" s="7">
+        <v>46154</v>
+      </c>
       <c r="D55" s="6"/>
       <c r="E55" s="6"/>
       <c r="F55" s="6"/>
@@ -30518,10 +31428,16 @@
       <c r="Y55" s="6"/>
       <c r="Z55" s="6"/>
     </row>
-    <row r="56" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A56" s="6"/>
-      <c r="B56" s="6"/>
-      <c r="C56" s="8"/>
+    <row r="56" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="C56" s="7">
+        <v>46155</v>
+      </c>
       <c r="D56" s="6"/>
       <c r="E56" s="6"/>
       <c r="F56" s="6"/>
@@ -30546,10 +31462,16 @@
       <c r="Y56" s="6"/>
       <c r="Z56" s="6"/>
     </row>
-    <row r="57" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A57" s="6"/>
-      <c r="B57" s="6"/>
-      <c r="C57" s="8"/>
+    <row r="57" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="C57" s="7">
+        <v>46156</v>
+      </c>
       <c r="D57" s="6"/>
       <c r="E57" s="6"/>
       <c r="F57" s="6"/>
@@ -30574,10 +31496,16 @@
       <c r="Y57" s="6"/>
       <c r="Z57" s="6"/>
     </row>
-    <row r="58" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A58" s="6"/>
-      <c r="B58" s="6"/>
-      <c r="C58" s="8"/>
+    <row r="58" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="C58" s="7">
+        <v>46157</v>
+      </c>
       <c r="D58" s="6"/>
       <c r="E58" s="6"/>
       <c r="F58" s="6"/>
@@ -30602,10 +31530,16 @@
       <c r="Y58" s="6"/>
       <c r="Z58" s="6"/>
     </row>
-    <row r="59" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A59" s="6"/>
-      <c r="B59" s="6"/>
-      <c r="C59" s="8"/>
+    <row r="59" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="C59" s="7">
+        <v>46158</v>
+      </c>
       <c r="D59" s="6"/>
       <c r="E59" s="6"/>
       <c r="F59" s="6"/>
@@ -30630,10 +31564,16 @@
       <c r="Y59" s="6"/>
       <c r="Z59" s="6"/>
     </row>
-    <row r="60" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A60" s="6"/>
-      <c r="B60" s="6"/>
-      <c r="C60" s="8"/>
+    <row r="60" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="C60" s="7">
+        <v>46159</v>
+      </c>
       <c r="D60" s="6"/>
       <c r="E60" s="6"/>
       <c r="F60" s="6"/>
@@ -30658,10 +31598,16 @@
       <c r="Y60" s="6"/>
       <c r="Z60" s="6"/>
     </row>
-    <row r="61" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A61" s="6"/>
-      <c r="B61" s="6"/>
-      <c r="C61" s="8"/>
+    <row r="61" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="C61" s="7">
+        <v>46160</v>
+      </c>
       <c r="D61" s="6"/>
       <c r="E61" s="6"/>
       <c r="F61" s="6"/>
@@ -30686,10 +31632,16 @@
       <c r="Y61" s="6"/>
       <c r="Z61" s="6"/>
     </row>
-    <row r="62" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A62" s="6"/>
-      <c r="B62" s="6"/>
-      <c r="C62" s="8"/>
+    <row r="62" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="C62" s="7">
+        <v>46161</v>
+      </c>
       <c r="D62" s="6"/>
       <c r="E62" s="6"/>
       <c r="F62" s="6"/>
@@ -30714,10 +31666,16 @@
       <c r="Y62" s="6"/>
       <c r="Z62" s="6"/>
     </row>
-    <row r="63" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A63" s="6"/>
-      <c r="B63" s="6"/>
-      <c r="C63" s="8"/>
+    <row r="63" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="13" t="s">
+        <v>225</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="C63" s="7">
+        <v>46162</v>
+      </c>
       <c r="D63" s="6"/>
       <c r="E63" s="6"/>
       <c r="F63" s="6"/>
@@ -30742,10 +31700,16 @@
       <c r="Y63" s="6"/>
       <c r="Z63" s="6"/>
     </row>
-    <row r="64" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A64" s="6"/>
-      <c r="B64" s="6"/>
-      <c r="C64" s="8"/>
+    <row r="64" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="C64" s="7">
+        <v>46163</v>
+      </c>
       <c r="D64" s="6"/>
       <c r="E64" s="6"/>
       <c r="F64" s="6"/>
@@ -30770,10 +31734,16 @@
       <c r="Y64" s="6"/>
       <c r="Z64" s="6"/>
     </row>
-    <row r="65" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A65" s="6"/>
-      <c r="B65" s="6"/>
-      <c r="C65" s="8"/>
+    <row r="65" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C65" s="7">
+        <v>46164</v>
+      </c>
       <c r="D65" s="6"/>
       <c r="E65" s="6"/>
       <c r="F65" s="6"/>
@@ -30798,10 +31768,16 @@
       <c r="Y65" s="6"/>
       <c r="Z65" s="6"/>
     </row>
-    <row r="66" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A66" s="6"/>
-      <c r="B66" s="6"/>
-      <c r="C66" s="8"/>
+    <row r="66" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="C66" s="7">
+        <v>46165</v>
+      </c>
       <c r="D66" s="6"/>
       <c r="E66" s="6"/>
       <c r="F66" s="6"/>
@@ -30826,10 +31802,16 @@
       <c r="Y66" s="6"/>
       <c r="Z66" s="6"/>
     </row>
-    <row r="67" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A67" s="6"/>
-      <c r="B67" s="6"/>
-      <c r="C67" s="8"/>
+    <row r="67" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="C67" s="7">
+        <v>46166</v>
+      </c>
       <c r="D67" s="6"/>
       <c r="E67" s="6"/>
       <c r="F67" s="6"/>
@@ -30854,10 +31836,16 @@
       <c r="Y67" s="6"/>
       <c r="Z67" s="6"/>
     </row>
-    <row r="68" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A68" s="6"/>
-      <c r="B68" s="6"/>
-      <c r="C68" s="8"/>
+    <row r="68" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="C68" s="7">
+        <v>46167</v>
+      </c>
       <c r="D68" s="6"/>
       <c r="E68" s="6"/>
       <c r="F68" s="6"/>
@@ -30882,10 +31870,16 @@
       <c r="Y68" s="6"/>
       <c r="Z68" s="6"/>
     </row>
-    <row r="69" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A69" s="6"/>
-      <c r="B69" s="6"/>
-      <c r="C69" s="8"/>
+    <row r="69" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="C69" s="7">
+        <v>46168</v>
+      </c>
       <c r="D69" s="6"/>
       <c r="E69" s="6"/>
       <c r="F69" s="6"/>
@@ -30910,10 +31904,16 @@
       <c r="Y69" s="6"/>
       <c r="Z69" s="6"/>
     </row>
-    <row r="70" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A70" s="6"/>
-      <c r="B70" s="6"/>
-      <c r="C70" s="8"/>
+    <row r="70" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="C70" s="7">
+        <v>46169</v>
+      </c>
       <c r="D70" s="6"/>
       <c r="E70" s="6"/>
       <c r="F70" s="6"/>
@@ -30938,10 +31938,16 @@
       <c r="Y70" s="6"/>
       <c r="Z70" s="6"/>
     </row>
-    <row r="71" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A71" s="6"/>
-      <c r="B71" s="6"/>
-      <c r="C71" s="8"/>
+    <row r="71" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="C71" s="7">
+        <v>46170</v>
+      </c>
       <c r="D71" s="6"/>
       <c r="E71" s="6"/>
       <c r="F71" s="6"/>
@@ -30966,10 +31972,16 @@
       <c r="Y71" s="6"/>
       <c r="Z71" s="6"/>
     </row>
-    <row r="72" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A72" s="6"/>
-      <c r="B72" s="6"/>
-      <c r="C72" s="8"/>
+    <row r="72" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="C72" s="7">
+        <v>46171</v>
+      </c>
       <c r="D72" s="6"/>
       <c r="E72" s="6"/>
       <c r="F72" s="6"/>
@@ -30994,10 +32006,16 @@
       <c r="Y72" s="6"/>
       <c r="Z72" s="6"/>
     </row>
-    <row r="73" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A73" s="6"/>
-      <c r="B73" s="6"/>
-      <c r="C73" s="8"/>
+    <row r="73" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C73" s="7">
+        <v>46172</v>
+      </c>
       <c r="D73" s="6"/>
       <c r="E73" s="6"/>
       <c r="F73" s="6"/>
@@ -31022,10 +32040,16 @@
       <c r="Y73" s="6"/>
       <c r="Z73" s="6"/>
     </row>
-    <row r="74" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A74" s="6"/>
-      <c r="B74" s="6"/>
-      <c r="C74" s="8"/>
+    <row r="74" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="C74" s="7">
+        <v>46173</v>
+      </c>
       <c r="D74" s="6"/>
       <c r="E74" s="6"/>
       <c r="F74" s="6"/>
@@ -31050,10 +32074,16 @@
       <c r="Y74" s="6"/>
       <c r="Z74" s="6"/>
     </row>
-    <row r="75" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A75" s="6"/>
-      <c r="B75" s="6"/>
-      <c r="C75" s="8"/>
+    <row r="75" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C75" s="7">
+        <v>46174</v>
+      </c>
       <c r="D75" s="6"/>
       <c r="E75" s="6"/>
       <c r="F75" s="6"/>
@@ -31078,10 +32108,16 @@
       <c r="Y75" s="6"/>
       <c r="Z75" s="6"/>
     </row>
-    <row r="76" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A76" s="6"/>
-      <c r="B76" s="6"/>
-      <c r="C76" s="8"/>
+    <row r="76" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="C76" s="7">
+        <v>46175</v>
+      </c>
       <c r="D76" s="6"/>
       <c r="E76" s="6"/>
       <c r="F76" s="6"/>
@@ -31106,10 +32142,16 @@
       <c r="Y76" s="6"/>
       <c r="Z76" s="6"/>
     </row>
-    <row r="77" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A77" s="6"/>
-      <c r="B77" s="6"/>
-      <c r="C77" s="8"/>
+    <row r="77" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="C77" s="7">
+        <v>46176</v>
+      </c>
       <c r="D77" s="6"/>
       <c r="E77" s="6"/>
       <c r="F77" s="6"/>
@@ -31134,10 +32176,16 @@
       <c r="Y77" s="6"/>
       <c r="Z77" s="6"/>
     </row>
-    <row r="78" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A78" s="6"/>
-      <c r="B78" s="6"/>
-      <c r="C78" s="8"/>
+    <row r="78" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="C78" s="7">
+        <v>46177</v>
+      </c>
       <c r="D78" s="6"/>
       <c r="E78" s="6"/>
       <c r="F78" s="6"/>
@@ -55544,6 +56592,36 @@
     <hyperlink ref="A46" r:id="rId45" xr:uid="{562F6695-A679-4430-BF00-4378A4968B67}"/>
     <hyperlink ref="A47" r:id="rId46" xr:uid="{FD905F37-8316-4227-8463-302ED81CEA43}"/>
     <hyperlink ref="A48" r:id="rId47" xr:uid="{44B510CF-CF69-4DA2-B4F2-A4CAB2CBAB43}"/>
+    <hyperlink ref="A49" r:id="rId48" xr:uid="{EE0317F6-8A35-4FCC-94D1-3F65F5090692}"/>
+    <hyperlink ref="A50" r:id="rId49" xr:uid="{C495C893-0F1A-460B-AB92-6543A6BCFA63}"/>
+    <hyperlink ref="A51" r:id="rId50" xr:uid="{F4A04766-24A1-44DF-9D3B-1FC913E7F399}"/>
+    <hyperlink ref="A52" r:id="rId51" xr:uid="{32CF6D1E-C7FF-4275-9C8C-1BE56ADAEC0D}"/>
+    <hyperlink ref="A53" r:id="rId52" xr:uid="{12A58EF4-9D37-467A-BB18-F1B0B174F1D3}"/>
+    <hyperlink ref="A54" r:id="rId53" xr:uid="{63275128-EED8-44BC-8DCC-41D143D644F6}"/>
+    <hyperlink ref="A55" r:id="rId54" xr:uid="{0832DF41-BB86-4D68-9E74-73FFDEBE661D}"/>
+    <hyperlink ref="A56" r:id="rId55" xr:uid="{8BA5B6F4-7191-419B-920F-7D034A7B41AB}"/>
+    <hyperlink ref="A57" r:id="rId56" xr:uid="{43B5570E-03E0-47D8-9493-CD16BEA74327}"/>
+    <hyperlink ref="A58" r:id="rId57" xr:uid="{C022705B-9CBF-4BFC-AE80-7A9210B241F7}"/>
+    <hyperlink ref="A59" r:id="rId58" xr:uid="{38D91709-54C9-4A3D-A5EA-E6F6531166C6}"/>
+    <hyperlink ref="A60" r:id="rId59" xr:uid="{13A32003-78A9-4936-9940-34CAE61A8E15}"/>
+    <hyperlink ref="A61" r:id="rId60" xr:uid="{6E9C1A81-0DDB-413B-8C07-1323672659E3}"/>
+    <hyperlink ref="A62" r:id="rId61" xr:uid="{3C527EE9-8B30-44D8-97B6-B457F30F8E84}"/>
+    <hyperlink ref="A63" r:id="rId62" xr:uid="{428340F2-3F56-4B59-8B93-6654EB8CFBCC}"/>
+    <hyperlink ref="A64" r:id="rId63" xr:uid="{96F22892-0FAB-4289-AAEB-BDDBCA8B6078}"/>
+    <hyperlink ref="A65" r:id="rId64" xr:uid="{71AD3A47-4AA9-430D-9DB4-FDD626D4EA13}"/>
+    <hyperlink ref="A66" r:id="rId65" xr:uid="{9CEC8706-1977-47BB-BA5C-0A2C9FDAEC59}"/>
+    <hyperlink ref="A67" r:id="rId66" xr:uid="{930CBEFF-E90B-407B-9401-053BD9B11FC9}"/>
+    <hyperlink ref="A68" r:id="rId67" xr:uid="{0F9E2411-1FDD-4CDD-80ED-C057BCA683F9}"/>
+    <hyperlink ref="A69" r:id="rId68" xr:uid="{7FBA81B6-8F35-41EE-9061-0324C2CABF69}"/>
+    <hyperlink ref="A70" r:id="rId69" xr:uid="{F28EC431-E276-4ACA-9CA1-31BFB88C4318}"/>
+    <hyperlink ref="A71" r:id="rId70" xr:uid="{F36AC178-63A5-4936-A912-AA0A52AC431E}"/>
+    <hyperlink ref="A72" r:id="rId71" xr:uid="{F9041319-FAE0-4B7C-A499-7CA7617135AF}"/>
+    <hyperlink ref="A73" r:id="rId72" xr:uid="{AB7ABC5A-ACA1-42BE-9729-3F32450D7C60}"/>
+    <hyperlink ref="A74" r:id="rId73" xr:uid="{03FF708E-B3F8-4F2F-A97E-99E9733AF3C8}"/>
+    <hyperlink ref="A75" r:id="rId74" xr:uid="{D9037A33-20F3-4A3E-8FA4-1AFCC86FDF26}"/>
+    <hyperlink ref="A76" r:id="rId75" xr:uid="{75E7BB78-DF66-4014-A336-4686E780F9BF}"/>
+    <hyperlink ref="A77" r:id="rId76" xr:uid="{DE1E9B7F-5063-48B2-8A6A-ED3B133AEE70}"/>
+    <hyperlink ref="A78" r:id="rId77" xr:uid="{4C325121-69F3-47B7-B8BA-1C9C5CF3F4C5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added new daily sadhana
</commit_message>
<xml_diff>
--- a/public/Daily Sadhana.xlsx
+++ b/public/Daily Sadhana.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sahaa\Documents\github_anandasvarupa\give_web\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{854DCA3A-6F3A-4F61-9CEC-CFA1BB19DFEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F1A35D-2D7F-4CF1-844E-E96E6B46E97E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="347">
   <si>
     <t>url</t>
   </si>
@@ -886,6 +886,189 @@
   <si>
     <t>Today's listening to Srila Prabhupada - 166</t>
   </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Saem-BuxjAY</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=v0k-3xubT_A</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=g-a3_i0nbDI</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=nriQoD9a1P0</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=UK5oPnC023c</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=S6HfFvYOCcA</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=IkcVFxp-K2U</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=JwME3EdY2Iw</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=IEVZuutf3mc</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=De-oTCuZ0uc</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=AQjB4UAv0ts</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=b5Bdo8mJrIY</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=l9JJ2kI5x6c</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=UD5noYvuVFc</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=aiy6IqoBZgk</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=c_Nf0a-wPqw</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Vt4XZNHQ_lk</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=BERqX0kQIJU</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=_4fom5vhdyQ</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Ut4UXig7mWQ</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=46_GzvqGc7I</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=igYTZO49JS8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=XhSUytfI-AY</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=i8v5Fb_aDW8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Iu8AoQz7N0g</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=fH_TTaOlwiY</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=-NHHdVWUcwo</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=U9FN1AMGujA</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Lyts-LMVgrM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=gOFEVX_YC4k</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 167</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 168</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 169</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 170</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 171</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 172</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 173</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 174</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 175</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 176</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 177</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 178</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 179</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 180</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 181</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 182</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 183</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 184</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 185</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 186</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 187</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 188</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 189</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 190</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 191</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 192</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 193</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 194</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 195</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 196</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 197</t>
+  </si>
 </sst>
 </file>
 
@@ -1286,7 +1469,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z73"/>
+  <dimension ref="A1:Z104"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="56.81640625" customWidth="1"/>
@@ -2118,6 +2301,347 @@
       </c>
       <c r="C73" s="5">
         <v>46177</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="C74" s="5">
+        <v>46178</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="C75" s="5">
+        <v>46179</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="C76" s="5">
+        <v>46180</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="C77" s="5">
+        <v>46181</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="11" t="s">
+        <v>290</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="C78" s="5">
+        <v>46182</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="C79" s="5">
+        <v>46183</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="11" t="s">
+        <v>292</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="C80" s="5">
+        <v>46184</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="C81" s="5">
+        <v>46185</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="11" t="s">
+        <v>294</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="C82" s="5">
+        <v>46186</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="11" t="s">
+        <v>295</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="C83" s="5">
+        <v>46187</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="11" t="s">
+        <v>296</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="C84" s="5">
+        <v>46188</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="C85" s="5">
+        <v>46189</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="11" t="s">
+        <v>298</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="C86" s="5">
+        <v>46190</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="11" t="s">
+        <v>299</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="C87" s="5">
+        <v>46191</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="C88" s="5">
+        <v>46192</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="C89" s="5">
+        <v>46193</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="11" t="s">
+        <v>302</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="C90" s="5">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="C91" s="5">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="C92" s="5">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="B93" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="C93" s="5">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="B94" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="C94" s="5">
+        <v>46198</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="11" t="s">
+        <v>306</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C95" s="5">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="B96" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="C96" s="5">
+        <v>46200</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="11" t="s">
+        <v>308</v>
+      </c>
+      <c r="B97" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="C97" s="5">
+        <v>46201</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="11" t="s">
+        <v>309</v>
+      </c>
+      <c r="B98" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="C98" s="5">
+        <v>46202</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="11" t="s">
+        <v>310</v>
+      </c>
+      <c r="B99" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="C99" s="5">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="11" t="s">
+        <v>311</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="C100" s="5">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="C101" s="5">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="B102" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="C102" s="5">
+        <v>46206</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="11" t="s">
+        <v>314</v>
+      </c>
+      <c r="B103" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="C103" s="5">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="11" t="s">
+        <v>315</v>
+      </c>
+      <c r="B104" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="C104" s="5">
+        <v>46208</v>
       </c>
     </row>
   </sheetData>
@@ -2195,9 +2719,40 @@
     <hyperlink ref="A71" r:id="rId70" xr:uid="{68C69F41-91D9-4109-B186-0401363D2F1C}"/>
     <hyperlink ref="A72" r:id="rId71" xr:uid="{B26834E6-4244-449F-8BCE-66D19D0721D4}"/>
     <hyperlink ref="A73" r:id="rId72" xr:uid="{C7ECCC81-082C-4F50-8852-6FD10D4C935E}"/>
+    <hyperlink ref="A74" r:id="rId73" xr:uid="{03A40CBC-A7A8-4DD1-BEF7-A5DA69184A11}"/>
+    <hyperlink ref="A75" r:id="rId74" display="https://www.youtube.com/watch?v=v0k-3xubT_A&amp;t=2s" xr:uid="{302260F7-63FA-44CF-A065-344A5E93BF1E}"/>
+    <hyperlink ref="A76" r:id="rId75" display="https://www.youtube.com/watch?v=g-a3_i0nbDI&amp;t=3s" xr:uid="{FBA5EB06-77AB-4697-A459-2DEF21E141D3}"/>
+    <hyperlink ref="A77" r:id="rId76" display="https://www.youtube.com/watch?v=nriQoD9a1P0&amp;t=156s" xr:uid="{40E877AC-96B3-4914-AC17-EC77D734C3AA}"/>
+    <hyperlink ref="A78" r:id="rId77" display="https://www.youtube.com/watch?v=UK5oPnC023c&amp;t=1s" xr:uid="{BE478E08-4759-4889-B718-A1A790A6E24D}"/>
+    <hyperlink ref="A79" r:id="rId78" xr:uid="{692348B6-782A-41BB-A1B5-B08B5D25D24D}"/>
+    <hyperlink ref="A80" r:id="rId79" xr:uid="{0260C706-8B40-4AFB-95D0-6B5FF3C8FEB2}"/>
+    <hyperlink ref="A81" r:id="rId80" display="https://www.youtube.com/watch?v=JwME3EdY2Iw&amp;t=1387s" xr:uid="{CB1D49DC-313E-4442-9402-12B0154F9336}"/>
+    <hyperlink ref="A82" r:id="rId81" display="https://www.youtube.com/watch?v=IEVZuutf3mc&amp;t=1s" xr:uid="{C7D57737-EBC3-4BF6-A3BE-3AB9B595066C}"/>
+    <hyperlink ref="A83" r:id="rId82" display="https://www.youtube.com/watch?v=De-oTCuZ0uc&amp;t=2s" xr:uid="{0245207D-5CCB-4C67-8FC4-54C122CF84D4}"/>
+    <hyperlink ref="A84" r:id="rId83" display="https://www.youtube.com/watch?v=AQjB4UAv0ts&amp;t=1s" xr:uid="{F5B8F609-824C-481E-B8EA-4EEE43E2E63D}"/>
+    <hyperlink ref="A85" r:id="rId84" xr:uid="{EAE002BB-3578-4096-B992-7A11D8B450BB}"/>
+    <hyperlink ref="A86" r:id="rId85" display="https://www.youtube.com/watch?v=l9JJ2kI5x6c&amp;t=29s" xr:uid="{EEB818B6-5ECB-4AF6-8595-6F2E8EEDCBF2}"/>
+    <hyperlink ref="A87" r:id="rId86" display="https://www.youtube.com/watch?v=UD5noYvuVFc&amp;t=1s" xr:uid="{C06BBEDC-F204-4DE1-AABD-9F1127310081}"/>
+    <hyperlink ref="A88" r:id="rId87" display="https://www.youtube.com/watch?v=aiy6IqoBZgk&amp;t=526s" xr:uid="{B2AE042A-7EF8-4ACD-A116-1A986AC9D0E1}"/>
+    <hyperlink ref="A89" r:id="rId88" xr:uid="{C11432AA-1EDD-4988-863A-5C4361347879}"/>
+    <hyperlink ref="A90" r:id="rId89" display="https://www.youtube.com/watch?v=Vt4XZNHQ_lk&amp;t=1s" xr:uid="{B6CABB49-1983-4CAB-885D-E1BCAC5908FC}"/>
+    <hyperlink ref="A91" r:id="rId90" display="https://www.youtube.com/watch?v=BERqX0kQIJU&amp;t=21s" xr:uid="{C745ABD5-37D3-4104-97F3-934089A477A8}"/>
+    <hyperlink ref="A92" r:id="rId91" display="https://www.youtube.com/watch?v=_4fom5vhdyQ&amp;t=243s" xr:uid="{0C450033-D2EA-451F-AE0E-707C7B0A49E7}"/>
+    <hyperlink ref="A93" r:id="rId92" display="https://www.youtube.com/watch?v=_4fom5vhdyQ&amp;t=243s" xr:uid="{A553E056-752E-41E1-A674-6F4B9FE6EDF1}"/>
+    <hyperlink ref="A94" r:id="rId93" display="https://www.youtube.com/watch?v=Ut4UXig7mWQ&amp;t=38s" xr:uid="{DD97B4B1-5529-44F9-BA1E-E90E1ED25556}"/>
+    <hyperlink ref="A95" r:id="rId94" xr:uid="{832EF4A1-B23F-4301-8908-F6A3CCEF1829}"/>
+    <hyperlink ref="A96" r:id="rId95" display="https://www.youtube.com/watch?v=igYTZO49JS8&amp;t=3s" xr:uid="{296974A3-18F7-49DD-B163-DF0D611472A2}"/>
+    <hyperlink ref="A97" r:id="rId96" xr:uid="{9E9441EB-2C4C-4AAF-A886-6184BAB3BC34}"/>
+    <hyperlink ref="A98" r:id="rId97" display="https://www.youtube.com/watch?v=i8v5Fb_aDW8&amp;t=1s" xr:uid="{82683ECC-ED20-4EEF-864A-F0C53A0E3DDE}"/>
+    <hyperlink ref="A99" r:id="rId98" display="https://www.youtube.com/watch?v=Iu8AoQz7N0g&amp;t=2s" xr:uid="{3A360530-97D5-40CF-A39A-E4EB63F047D4}"/>
+    <hyperlink ref="A100" r:id="rId99" display="https://www.youtube.com/watch?v=fH_TTaOlwiY&amp;t=1s" xr:uid="{4ACD65C0-3FEB-4058-8840-291357EEEA75}"/>
+    <hyperlink ref="A101" r:id="rId100" xr:uid="{B6FBF0B5-487A-4A5C-BB3F-CA5DD3DF1EC1}"/>
+    <hyperlink ref="A102" r:id="rId101" display="https://www.youtube.com/watch?v=U9FN1AMGujA&amp;t=8s" xr:uid="{7A64A9C9-FDA9-4CD1-A658-16C1F8328ECB}"/>
+    <hyperlink ref="A103" r:id="rId102" xr:uid="{855D2333-75B0-4DB1-BDE3-97863E7388CB}"/>
+    <hyperlink ref="A104" r:id="rId103" display="https://www.youtube.com/watch?v=gOFEVX_YC4k&amp;t=54s" xr:uid="{D7F561D8-EE4F-4F94-A891-A4CD0CFBE8F2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId73"/>
+  <pageSetup orientation="portrait" r:id="rId104"/>
 </worksheet>
 </file>
 
@@ -6125,10 +6680,16 @@
       <c r="Y115" s="6"/>
       <c r="Z115" s="6"/>
     </row>
-    <row r="116" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A116" s="6"/>
-      <c r="B116" s="6"/>
-      <c r="C116" s="6"/>
+    <row r="116" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A116" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="B116" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="C116" s="5">
+        <v>46178</v>
+      </c>
       <c r="D116" s="6"/>
       <c r="E116" s="6"/>
       <c r="F116" s="6"/>
@@ -6153,10 +6714,16 @@
       <c r="Y116" s="6"/>
       <c r="Z116" s="6"/>
     </row>
-    <row r="117" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A117" s="6"/>
-      <c r="B117" s="6"/>
-      <c r="C117" s="6"/>
+    <row r="117" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A117" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="B117" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="C117" s="5">
+        <v>46179</v>
+      </c>
       <c r="D117" s="6"/>
       <c r="E117" s="6"/>
       <c r="F117" s="6"/>
@@ -6181,10 +6748,16 @@
       <c r="Y117" s="6"/>
       <c r="Z117" s="6"/>
     </row>
-    <row r="118" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A118" s="6"/>
-      <c r="B118" s="6"/>
-      <c r="C118" s="6"/>
+    <row r="118" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A118" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="B118" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C118" s="5">
+        <v>46180</v>
+      </c>
       <c r="D118" s="6"/>
       <c r="E118" s="6"/>
       <c r="F118" s="6"/>
@@ -6209,10 +6782,16 @@
       <c r="Y118" s="6"/>
       <c r="Z118" s="6"/>
     </row>
-    <row r="119" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A119" s="6"/>
-      <c r="B119" s="6"/>
-      <c r="C119" s="6"/>
+    <row r="119" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A119" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="B119" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="C119" s="5">
+        <v>46181</v>
+      </c>
       <c r="D119" s="6"/>
       <c r="E119" s="6"/>
       <c r="F119" s="6"/>
@@ -6237,10 +6816,16 @@
       <c r="Y119" s="6"/>
       <c r="Z119" s="6"/>
     </row>
-    <row r="120" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A120" s="6"/>
-      <c r="B120" s="6"/>
-      <c r="C120" s="6"/>
+    <row r="120" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A120" s="11" t="s">
+        <v>290</v>
+      </c>
+      <c r="B120" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C120" s="5">
+        <v>46182</v>
+      </c>
       <c r="D120" s="6"/>
       <c r="E120" s="6"/>
       <c r="F120" s="6"/>
@@ -6265,10 +6850,16 @@
       <c r="Y120" s="6"/>
       <c r="Z120" s="6"/>
     </row>
-    <row r="121" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A121" s="6"/>
-      <c r="B121" s="6"/>
-      <c r="C121" s="6"/>
+    <row r="121" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A121" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="B121" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="C121" s="5">
+        <v>46183</v>
+      </c>
       <c r="D121" s="6"/>
       <c r="E121" s="6"/>
       <c r="F121" s="6"/>
@@ -6293,10 +6884,16 @@
       <c r="Y121" s="6"/>
       <c r="Z121" s="6"/>
     </row>
-    <row r="122" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A122" s="6"/>
-      <c r="B122" s="6"/>
-      <c r="C122" s="6"/>
+    <row r="122" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A122" s="11" t="s">
+        <v>292</v>
+      </c>
+      <c r="B122" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="C122" s="5">
+        <v>46184</v>
+      </c>
       <c r="D122" s="6"/>
       <c r="E122" s="6"/>
       <c r="F122" s="6"/>
@@ -6321,10 +6918,16 @@
       <c r="Y122" s="6"/>
       <c r="Z122" s="6"/>
     </row>
-    <row r="123" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A123" s="6"/>
-      <c r="B123" s="6"/>
-      <c r="C123" s="6"/>
+    <row r="123" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A123" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="B123" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="C123" s="5">
+        <v>46185</v>
+      </c>
       <c r="D123" s="6"/>
       <c r="E123" s="6"/>
       <c r="F123" s="6"/>
@@ -6349,10 +6952,16 @@
       <c r="Y123" s="6"/>
       <c r="Z123" s="6"/>
     </row>
-    <row r="124" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A124" s="6"/>
-      <c r="B124" s="6"/>
-      <c r="C124" s="6"/>
+    <row r="124" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A124" s="11" t="s">
+        <v>294</v>
+      </c>
+      <c r="B124" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="C124" s="5">
+        <v>46186</v>
+      </c>
       <c r="D124" s="6"/>
       <c r="E124" s="6"/>
       <c r="F124" s="6"/>
@@ -6377,10 +6986,16 @@
       <c r="Y124" s="6"/>
       <c r="Z124" s="6"/>
     </row>
-    <row r="125" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A125" s="6"/>
-      <c r="B125" s="6"/>
-      <c r="C125" s="6"/>
+    <row r="125" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A125" s="11" t="s">
+        <v>295</v>
+      </c>
+      <c r="B125" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C125" s="5">
+        <v>46187</v>
+      </c>
       <c r="D125" s="6"/>
       <c r="E125" s="6"/>
       <c r="F125" s="6"/>
@@ -6405,10 +7020,16 @@
       <c r="Y125" s="6"/>
       <c r="Z125" s="6"/>
     </row>
-    <row r="126" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A126" s="6"/>
-      <c r="B126" s="6"/>
-      <c r="C126" s="6"/>
+    <row r="126" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A126" s="11" t="s">
+        <v>296</v>
+      </c>
+      <c r="B126" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="C126" s="5">
+        <v>46188</v>
+      </c>
       <c r="D126" s="6"/>
       <c r="E126" s="6"/>
       <c r="F126" s="6"/>
@@ -6433,10 +7054,16 @@
       <c r="Y126" s="6"/>
       <c r="Z126" s="6"/>
     </row>
-    <row r="127" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A127" s="6"/>
-      <c r="B127" s="6"/>
-      <c r="C127" s="6"/>
+    <row r="127" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A127" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="B127" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="C127" s="5">
+        <v>46189</v>
+      </c>
       <c r="D127" s="6"/>
       <c r="E127" s="6"/>
       <c r="F127" s="6"/>
@@ -6461,10 +7088,16 @@
       <c r="Y127" s="6"/>
       <c r="Z127" s="6"/>
     </row>
-    <row r="128" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A128" s="6"/>
-      <c r="B128" s="6"/>
-      <c r="C128" s="6"/>
+    <row r="128" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A128" s="11" t="s">
+        <v>298</v>
+      </c>
+      <c r="B128" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="C128" s="5">
+        <v>46190</v>
+      </c>
       <c r="D128" s="6"/>
       <c r="E128" s="6"/>
       <c r="F128" s="6"/>
@@ -6489,10 +7122,16 @@
       <c r="Y128" s="6"/>
       <c r="Z128" s="6"/>
     </row>
-    <row r="129" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A129" s="6"/>
-      <c r="B129" s="6"/>
-      <c r="C129" s="6"/>
+    <row r="129" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A129" s="11" t="s">
+        <v>299</v>
+      </c>
+      <c r="B129" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="C129" s="5">
+        <v>46191</v>
+      </c>
       <c r="D129" s="6"/>
       <c r="E129" s="6"/>
       <c r="F129" s="6"/>
@@ -6517,10 +7156,16 @@
       <c r="Y129" s="6"/>
       <c r="Z129" s="6"/>
     </row>
-    <row r="130" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A130" s="6"/>
-      <c r="B130" s="6"/>
-      <c r="C130" s="6"/>
+    <row r="130" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A130" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="B130" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C130" s="5">
+        <v>46192</v>
+      </c>
       <c r="D130" s="6"/>
       <c r="E130" s="6"/>
       <c r="F130" s="6"/>
@@ -6545,10 +7190,16 @@
       <c r="Y130" s="6"/>
       <c r="Z130" s="6"/>
     </row>
-    <row r="131" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A131" s="6"/>
-      <c r="B131" s="6"/>
-      <c r="C131" s="6"/>
+    <row r="131" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A131" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="B131" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="C131" s="5">
+        <v>46193</v>
+      </c>
       <c r="D131" s="6"/>
       <c r="E131" s="6"/>
       <c r="F131" s="6"/>
@@ -6573,10 +7224,16 @@
       <c r="Y131" s="6"/>
       <c r="Z131" s="6"/>
     </row>
-    <row r="132" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A132" s="6"/>
-      <c r="B132" s="6"/>
-      <c r="C132" s="6"/>
+    <row r="132" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A132" s="11" t="s">
+        <v>302</v>
+      </c>
+      <c r="B132" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="C132" s="5">
+        <v>46194</v>
+      </c>
       <c r="D132" s="6"/>
       <c r="E132" s="6"/>
       <c r="F132" s="6"/>
@@ -6601,10 +7258,16 @@
       <c r="Y132" s="6"/>
       <c r="Z132" s="6"/>
     </row>
-    <row r="133" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A133" s="6"/>
-      <c r="B133" s="6"/>
-      <c r="C133" s="6"/>
+    <row r="133" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A133" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="B133" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="C133" s="5">
+        <v>46195</v>
+      </c>
       <c r="D133" s="6"/>
       <c r="E133" s="6"/>
       <c r="F133" s="6"/>
@@ -6629,10 +7292,16 @@
       <c r="Y133" s="6"/>
       <c r="Z133" s="6"/>
     </row>
-    <row r="134" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A134" s="6"/>
-      <c r="B134" s="6"/>
-      <c r="C134" s="6"/>
+    <row r="134" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A134" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="B134" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="C134" s="5">
+        <v>46196</v>
+      </c>
       <c r="D134" s="6"/>
       <c r="E134" s="6"/>
       <c r="F134" s="6"/>
@@ -6657,10 +7326,16 @@
       <c r="Y134" s="6"/>
       <c r="Z134" s="6"/>
     </row>
-    <row r="135" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A135" s="6"/>
-      <c r="B135" s="6"/>
-      <c r="C135" s="6"/>
+    <row r="135" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A135" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="B135" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="C135" s="5">
+        <v>46197</v>
+      </c>
       <c r="D135" s="6"/>
       <c r="E135" s="6"/>
       <c r="F135" s="6"/>
@@ -6685,10 +7360,16 @@
       <c r="Y135" s="6"/>
       <c r="Z135" s="6"/>
     </row>
-    <row r="136" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A136" s="6"/>
-      <c r="B136" s="6"/>
-      <c r="C136" s="6"/>
+    <row r="136" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A136" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="B136" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="C136" s="5">
+        <v>46198</v>
+      </c>
       <c r="D136" s="6"/>
       <c r="E136" s="6"/>
       <c r="F136" s="6"/>
@@ -6713,10 +7394,16 @@
       <c r="Y136" s="6"/>
       <c r="Z136" s="6"/>
     </row>
-    <row r="137" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A137" s="6"/>
-      <c r="B137" s="6"/>
-      <c r="C137" s="6"/>
+    <row r="137" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A137" s="11" t="s">
+        <v>306</v>
+      </c>
+      <c r="B137" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C137" s="5">
+        <v>46199</v>
+      </c>
       <c r="D137" s="6"/>
       <c r="E137" s="6"/>
       <c r="F137" s="6"/>
@@ -6741,10 +7428,16 @@
       <c r="Y137" s="6"/>
       <c r="Z137" s="6"/>
     </row>
-    <row r="138" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A138" s="6"/>
-      <c r="B138" s="6"/>
-      <c r="C138" s="6"/>
+    <row r="138" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A138" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="B138" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="C138" s="5">
+        <v>46200</v>
+      </c>
       <c r="D138" s="6"/>
       <c r="E138" s="6"/>
       <c r="F138" s="6"/>
@@ -6769,10 +7462,16 @@
       <c r="Y138" s="6"/>
       <c r="Z138" s="6"/>
     </row>
-    <row r="139" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A139" s="6"/>
-      <c r="B139" s="6"/>
-      <c r="C139" s="6"/>
+    <row r="139" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A139" s="11" t="s">
+        <v>308</v>
+      </c>
+      <c r="B139" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="C139" s="5">
+        <v>46201</v>
+      </c>
       <c r="D139" s="6"/>
       <c r="E139" s="6"/>
       <c r="F139" s="6"/>
@@ -6797,10 +7496,16 @@
       <c r="Y139" s="6"/>
       <c r="Z139" s="6"/>
     </row>
-    <row r="140" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A140" s="6"/>
-      <c r="B140" s="6"/>
-      <c r="C140" s="6"/>
+    <row r="140" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A140" s="11" t="s">
+        <v>309</v>
+      </c>
+      <c r="B140" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="C140" s="5">
+        <v>46202</v>
+      </c>
       <c r="D140" s="6"/>
       <c r="E140" s="6"/>
       <c r="F140" s="6"/>
@@ -6825,10 +7530,16 @@
       <c r="Y140" s="6"/>
       <c r="Z140" s="6"/>
     </row>
-    <row r="141" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A141" s="6"/>
-      <c r="B141" s="6"/>
-      <c r="C141" s="6"/>
+    <row r="141" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A141" s="11" t="s">
+        <v>310</v>
+      </c>
+      <c r="B141" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C141" s="5">
+        <v>46203</v>
+      </c>
       <c r="D141" s="6"/>
       <c r="E141" s="6"/>
       <c r="F141" s="6"/>
@@ -6853,10 +7564,16 @@
       <c r="Y141" s="6"/>
       <c r="Z141" s="6"/>
     </row>
-    <row r="142" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A142" s="6"/>
-      <c r="B142" s="6"/>
-      <c r="C142" s="6"/>
+    <row r="142" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A142" s="11" t="s">
+        <v>311</v>
+      </c>
+      <c r="B142" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="C142" s="5">
+        <v>46204</v>
+      </c>
       <c r="D142" s="6"/>
       <c r="E142" s="6"/>
       <c r="F142" s="6"/>
@@ -6881,10 +7598,16 @@
       <c r="Y142" s="6"/>
       <c r="Z142" s="6"/>
     </row>
-    <row r="143" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A143" s="6"/>
-      <c r="B143" s="6"/>
-      <c r="C143" s="6"/>
+    <row r="143" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A143" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="B143" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="C143" s="5">
+        <v>46205</v>
+      </c>
       <c r="D143" s="6"/>
       <c r="E143" s="6"/>
       <c r="F143" s="6"/>
@@ -6909,10 +7632,16 @@
       <c r="Y143" s="6"/>
       <c r="Z143" s="6"/>
     </row>
-    <row r="144" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A144" s="6"/>
-      <c r="B144" s="6"/>
-      <c r="C144" s="6"/>
+    <row r="144" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A144" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="B144" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="C144" s="5">
+        <v>46206</v>
+      </c>
       <c r="D144" s="6"/>
       <c r="E144" s="6"/>
       <c r="F144" s="6"/>
@@ -6937,10 +7666,16 @@
       <c r="Y144" s="6"/>
       <c r="Z144" s="6"/>
     </row>
-    <row r="145" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A145" s="6"/>
-      <c r="B145" s="6"/>
-      <c r="C145" s="6"/>
+    <row r="145" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A145" s="11" t="s">
+        <v>314</v>
+      </c>
+      <c r="B145" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="C145" s="5">
+        <v>46207</v>
+      </c>
       <c r="D145" s="6"/>
       <c r="E145" s="6"/>
       <c r="F145" s="6"/>
@@ -6965,10 +7700,16 @@
       <c r="Y145" s="6"/>
       <c r="Z145" s="6"/>
     </row>
-    <row r="146" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A146" s="6"/>
-      <c r="B146" s="6"/>
-      <c r="C146" s="6"/>
+    <row r="146" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A146" s="11" t="s">
+        <v>315</v>
+      </c>
+      <c r="B146" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="C146" s="5">
+        <v>46208</v>
+      </c>
       <c r="D146" s="6"/>
       <c r="E146" s="6"/>
       <c r="F146" s="6"/>
@@ -29538,9 +30279,40 @@
     <hyperlink ref="A113" r:id="rId112" xr:uid="{D12CF023-7448-4AC2-B7FB-1284C1269E70}"/>
     <hyperlink ref="A114" r:id="rId113" xr:uid="{C30B01CE-4989-4ECD-80C5-EDBAE8EFD21B}"/>
     <hyperlink ref="A115" r:id="rId114" xr:uid="{6C99A764-2055-4805-923C-CC469CD6B5FE}"/>
+    <hyperlink ref="A116" r:id="rId115" xr:uid="{ECDF3447-DCDA-47FF-B932-EF7FB2DD89D2}"/>
+    <hyperlink ref="A117" r:id="rId116" display="https://www.youtube.com/watch?v=v0k-3xubT_A&amp;t=2s" xr:uid="{D062A032-C686-478E-8381-520A4A91C477}"/>
+    <hyperlink ref="A118" r:id="rId117" display="https://www.youtube.com/watch?v=g-a3_i0nbDI&amp;t=3s" xr:uid="{F42D60D2-713D-4737-8A7F-8FEEFBD23D52}"/>
+    <hyperlink ref="A119" r:id="rId118" display="https://www.youtube.com/watch?v=nriQoD9a1P0&amp;t=156s" xr:uid="{121FAC86-D1FD-4D4C-BC99-342A3CEFD694}"/>
+    <hyperlink ref="A120" r:id="rId119" display="https://www.youtube.com/watch?v=UK5oPnC023c&amp;t=1s" xr:uid="{8334C07C-F665-46FE-B719-4B7BAE4F6193}"/>
+    <hyperlink ref="A121" r:id="rId120" xr:uid="{2DF15B51-9C75-44E1-A56D-E1B1F977CEE5}"/>
+    <hyperlink ref="A122" r:id="rId121" xr:uid="{1C918299-FF19-4EF2-8CA0-87334C1118C9}"/>
+    <hyperlink ref="A123" r:id="rId122" display="https://www.youtube.com/watch?v=JwME3EdY2Iw&amp;t=1387s" xr:uid="{5FF807A5-E0D8-4E60-AA76-9B3D67FCF5C2}"/>
+    <hyperlink ref="A124" r:id="rId123" display="https://www.youtube.com/watch?v=IEVZuutf3mc&amp;t=1s" xr:uid="{8D92C7CF-8ABD-42B7-9B26-0DF48FED37E6}"/>
+    <hyperlink ref="A125" r:id="rId124" display="https://www.youtube.com/watch?v=De-oTCuZ0uc&amp;t=2s" xr:uid="{F459C874-2F60-4443-BC6D-C2187BB8FD8A}"/>
+    <hyperlink ref="A126" r:id="rId125" display="https://www.youtube.com/watch?v=AQjB4UAv0ts&amp;t=1s" xr:uid="{2E142956-C6D4-4283-B1BC-222CDEA9EDDD}"/>
+    <hyperlink ref="A127" r:id="rId126" xr:uid="{47F73EED-A970-4E58-9AF0-573B37295ECF}"/>
+    <hyperlink ref="A128" r:id="rId127" display="https://www.youtube.com/watch?v=l9JJ2kI5x6c&amp;t=29s" xr:uid="{D194CD88-EBB4-4182-B2BE-32412B9B275F}"/>
+    <hyperlink ref="A129" r:id="rId128" display="https://www.youtube.com/watch?v=UD5noYvuVFc&amp;t=1s" xr:uid="{4956CFC2-7661-4567-8059-0933001D9A97}"/>
+    <hyperlink ref="A130" r:id="rId129" display="https://www.youtube.com/watch?v=aiy6IqoBZgk&amp;t=526s" xr:uid="{9197DDC1-2370-475A-A49E-B276668355FE}"/>
+    <hyperlink ref="A131" r:id="rId130" xr:uid="{285878C5-6AA5-4CD7-BA6D-0B5AC449D69B}"/>
+    <hyperlink ref="A132" r:id="rId131" display="https://www.youtube.com/watch?v=Vt4XZNHQ_lk&amp;t=1s" xr:uid="{C9ED7C92-2ADC-4F60-99E3-8AB637C07AB7}"/>
+    <hyperlink ref="A133" r:id="rId132" display="https://www.youtube.com/watch?v=BERqX0kQIJU&amp;t=21s" xr:uid="{9F50BB0C-2D0E-4058-8BF6-6416C1237EC4}"/>
+    <hyperlink ref="A134" r:id="rId133" display="https://www.youtube.com/watch?v=_4fom5vhdyQ&amp;t=243s" xr:uid="{1A938863-A65F-41E4-BA28-F2F9E5EDF29D}"/>
+    <hyperlink ref="A135" r:id="rId134" display="https://www.youtube.com/watch?v=_4fom5vhdyQ&amp;t=243s" xr:uid="{09603758-60F8-4C5A-9F54-499C85889E2D}"/>
+    <hyperlink ref="A136" r:id="rId135" display="https://www.youtube.com/watch?v=Ut4UXig7mWQ&amp;t=38s" xr:uid="{4443F6D3-548C-4598-B114-73F8B15927E5}"/>
+    <hyperlink ref="A137" r:id="rId136" xr:uid="{4B89D2A7-B061-4C57-9C5C-4C2098B4B563}"/>
+    <hyperlink ref="A138" r:id="rId137" display="https://www.youtube.com/watch?v=igYTZO49JS8&amp;t=3s" xr:uid="{8DE096D7-6BEE-441E-8ACA-1564814CB7A4}"/>
+    <hyperlink ref="A139" r:id="rId138" xr:uid="{604A652E-08C1-4008-BE47-598808E42B75}"/>
+    <hyperlink ref="A140" r:id="rId139" display="https://www.youtube.com/watch?v=i8v5Fb_aDW8&amp;t=1s" xr:uid="{BD05834F-7D9C-4A8E-A6F1-4F53C0B55014}"/>
+    <hyperlink ref="A141" r:id="rId140" display="https://www.youtube.com/watch?v=Iu8AoQz7N0g&amp;t=2s" xr:uid="{D413952A-FFD5-4242-A2E2-B576B67E0876}"/>
+    <hyperlink ref="A142" r:id="rId141" display="https://www.youtube.com/watch?v=fH_TTaOlwiY&amp;t=1s" xr:uid="{BB6A14EB-CDED-4DB5-92C7-46A0CAF6602D}"/>
+    <hyperlink ref="A143" r:id="rId142" xr:uid="{F416E064-6693-4CD4-9563-754ED712397C}"/>
+    <hyperlink ref="A144" r:id="rId143" display="https://www.youtube.com/watch?v=U9FN1AMGujA&amp;t=8s" xr:uid="{9C79E9E9-BF43-4240-BF0E-3F8815EA2EF6}"/>
+    <hyperlink ref="A145" r:id="rId144" xr:uid="{F9449730-DBCF-4702-AB21-B2C54AF58C92}"/>
+    <hyperlink ref="A146" r:id="rId145" display="https://www.youtube.com/watch?v=gOFEVX_YC4k&amp;t=54s" xr:uid="{BC1B3516-9B46-451E-8EA7-309E5CE86C84}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId115"/>
+  <pageSetup orientation="portrait" r:id="rId146"/>
 </worksheet>
 </file>
 
@@ -32210,10 +32982,16 @@
       <c r="Y78" s="6"/>
       <c r="Z78" s="6"/>
     </row>
-    <row r="79" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A79" s="6"/>
-      <c r="B79" s="6"/>
-      <c r="C79" s="8"/>
+    <row r="79" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="C79" s="7">
+        <v>46178</v>
+      </c>
       <c r="D79" s="6"/>
       <c r="E79" s="6"/>
       <c r="F79" s="6"/>
@@ -32238,10 +33016,16 @@
       <c r="Y79" s="6"/>
       <c r="Z79" s="6"/>
     </row>
-    <row r="80" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A80" s="6"/>
-      <c r="B80" s="6"/>
-      <c r="C80" s="8"/>
+    <row r="80" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="C80" s="7">
+        <v>46179</v>
+      </c>
       <c r="D80" s="6"/>
       <c r="E80" s="6"/>
       <c r="F80" s="6"/>
@@ -32266,10 +33050,16 @@
       <c r="Y80" s="6"/>
       <c r="Z80" s="6"/>
     </row>
-    <row r="81" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A81" s="6"/>
-      <c r="B81" s="6"/>
-      <c r="C81" s="8"/>
+    <row r="81" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="C81" s="7">
+        <v>46180</v>
+      </c>
       <c r="D81" s="6"/>
       <c r="E81" s="6"/>
       <c r="F81" s="6"/>
@@ -32294,10 +33084,16 @@
       <c r="Y81" s="6"/>
       <c r="Z81" s="6"/>
     </row>
-    <row r="82" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A82" s="6"/>
-      <c r="B82" s="6"/>
-      <c r="C82" s="8"/>
+    <row r="82" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="C82" s="7">
+        <v>46181</v>
+      </c>
       <c r="D82" s="6"/>
       <c r="E82" s="6"/>
       <c r="F82" s="6"/>
@@ -32322,10 +33118,16 @@
       <c r="Y82" s="6"/>
       <c r="Z82" s="6"/>
     </row>
-    <row r="83" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A83" s="6"/>
-      <c r="B83" s="6"/>
-      <c r="C83" s="8"/>
+    <row r="83" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="11" t="s">
+        <v>290</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C83" s="7">
+        <v>46182</v>
+      </c>
       <c r="D83" s="6"/>
       <c r="E83" s="6"/>
       <c r="F83" s="6"/>
@@ -32350,10 +33152,16 @@
       <c r="Y83" s="6"/>
       <c r="Z83" s="6"/>
     </row>
-    <row r="84" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A84" s="6"/>
-      <c r="B84" s="6"/>
-      <c r="C84" s="8"/>
+    <row r="84" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="C84" s="7">
+        <v>46183</v>
+      </c>
       <c r="D84" s="6"/>
       <c r="E84" s="6"/>
       <c r="F84" s="6"/>
@@ -32378,10 +33186,16 @@
       <c r="Y84" s="6"/>
       <c r="Z84" s="6"/>
     </row>
-    <row r="85" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A85" s="6"/>
-      <c r="B85" s="6"/>
-      <c r="C85" s="8"/>
+    <row r="85" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="11" t="s">
+        <v>292</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="C85" s="7">
+        <v>46184</v>
+      </c>
       <c r="D85" s="6"/>
       <c r="E85" s="6"/>
       <c r="F85" s="6"/>
@@ -32406,10 +33220,16 @@
       <c r="Y85" s="6"/>
       <c r="Z85" s="6"/>
     </row>
-    <row r="86" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A86" s="6"/>
-      <c r="B86" s="6"/>
-      <c r="C86" s="8"/>
+    <row r="86" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="C86" s="7">
+        <v>46185</v>
+      </c>
       <c r="D86" s="6"/>
       <c r="E86" s="6"/>
       <c r="F86" s="6"/>
@@ -32434,10 +33254,16 @@
       <c r="Y86" s="6"/>
       <c r="Z86" s="6"/>
     </row>
-    <row r="87" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A87" s="6"/>
-      <c r="B87" s="6"/>
-      <c r="C87" s="8"/>
+    <row r="87" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="11" t="s">
+        <v>294</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="C87" s="7">
+        <v>46186</v>
+      </c>
       <c r="D87" s="6"/>
       <c r="E87" s="6"/>
       <c r="F87" s="6"/>
@@ -32462,10 +33288,16 @@
       <c r="Y87" s="6"/>
       <c r="Z87" s="6"/>
     </row>
-    <row r="88" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A88" s="6"/>
-      <c r="B88" s="6"/>
-      <c r="C88" s="8"/>
+    <row r="88" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="11" t="s">
+        <v>295</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="C88" s="7">
+        <v>46187</v>
+      </c>
       <c r="D88" s="6"/>
       <c r="E88" s="6"/>
       <c r="F88" s="6"/>
@@ -32490,10 +33322,16 @@
       <c r="Y88" s="6"/>
       <c r="Z88" s="6"/>
     </row>
-    <row r="89" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A89" s="6"/>
-      <c r="B89" s="6"/>
-      <c r="C89" s="8"/>
+    <row r="89" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="11" t="s">
+        <v>296</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="C89" s="7">
+        <v>46188</v>
+      </c>
       <c r="D89" s="6"/>
       <c r="E89" s="6"/>
       <c r="F89" s="6"/>
@@ -32518,10 +33356,16 @@
       <c r="Y89" s="6"/>
       <c r="Z89" s="6"/>
     </row>
-    <row r="90" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A90" s="6"/>
-      <c r="B90" s="6"/>
-      <c r="C90" s="8"/>
+    <row r="90" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="C90" s="7">
+        <v>46189</v>
+      </c>
       <c r="D90" s="6"/>
       <c r="E90" s="6"/>
       <c r="F90" s="6"/>
@@ -32546,10 +33390,16 @@
       <c r="Y90" s="6"/>
       <c r="Z90" s="6"/>
     </row>
-    <row r="91" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A91" s="6"/>
-      <c r="B91" s="6"/>
-      <c r="C91" s="8"/>
+    <row r="91" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="11" t="s">
+        <v>298</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="C91" s="7">
+        <v>46190</v>
+      </c>
       <c r="D91" s="6"/>
       <c r="E91" s="6"/>
       <c r="F91" s="6"/>
@@ -32574,10 +33424,16 @@
       <c r="Y91" s="6"/>
       <c r="Z91" s="6"/>
     </row>
-    <row r="92" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A92" s="6"/>
-      <c r="B92" s="6"/>
-      <c r="C92" s="8"/>
+    <row r="92" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="11" t="s">
+        <v>299</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="C92" s="7">
+        <v>46191</v>
+      </c>
       <c r="D92" s="6"/>
       <c r="E92" s="6"/>
       <c r="F92" s="6"/>
@@ -32602,10 +33458,16 @@
       <c r="Y92" s="6"/>
       <c r="Z92" s="6"/>
     </row>
-    <row r="93" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A93" s="6"/>
-      <c r="B93" s="6"/>
-      <c r="C93" s="8"/>
+    <row r="93" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="B93" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="C93" s="7">
+        <v>46192</v>
+      </c>
       <c r="D93" s="6"/>
       <c r="E93" s="6"/>
       <c r="F93" s="6"/>
@@ -32630,10 +33492,16 @@
       <c r="Y93" s="6"/>
       <c r="Z93" s="6"/>
     </row>
-    <row r="94" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A94" s="6"/>
-      <c r="B94" s="6"/>
-      <c r="C94" s="8"/>
+    <row r="94" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="B94" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="C94" s="7">
+        <v>46193</v>
+      </c>
       <c r="D94" s="6"/>
       <c r="E94" s="6"/>
       <c r="F94" s="6"/>
@@ -32658,10 +33526,16 @@
       <c r="Y94" s="6"/>
       <c r="Z94" s="6"/>
     </row>
-    <row r="95" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A95" s="6"/>
-      <c r="B95" s="6"/>
-      <c r="C95" s="8"/>
+    <row r="95" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="11" t="s">
+        <v>302</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="C95" s="7">
+        <v>46194</v>
+      </c>
       <c r="D95" s="6"/>
       <c r="E95" s="6"/>
       <c r="F95" s="6"/>
@@ -32686,10 +33560,16 @@
       <c r="Y95" s="6"/>
       <c r="Z95" s="6"/>
     </row>
-    <row r="96" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A96" s="6"/>
-      <c r="B96" s="6"/>
-      <c r="C96" s="8"/>
+    <row r="96" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="B96" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C96" s="7">
+        <v>46195</v>
+      </c>
       <c r="D96" s="6"/>
       <c r="E96" s="6"/>
       <c r="F96" s="6"/>
@@ -32714,10 +33594,16 @@
       <c r="Y96" s="6"/>
       <c r="Z96" s="6"/>
     </row>
-    <row r="97" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A97" s="6"/>
-      <c r="B97" s="6"/>
-      <c r="C97" s="8"/>
+    <row r="97" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="B97" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="C97" s="7">
+        <v>46196</v>
+      </c>
       <c r="D97" s="6"/>
       <c r="E97" s="6"/>
       <c r="F97" s="6"/>
@@ -32742,10 +33628,16 @@
       <c r="Y97" s="6"/>
       <c r="Z97" s="6"/>
     </row>
-    <row r="98" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A98" s="6"/>
-      <c r="B98" s="6"/>
-      <c r="C98" s="8"/>
+    <row r="98" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="B98" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="C98" s="7">
+        <v>46197</v>
+      </c>
       <c r="D98" s="6"/>
       <c r="E98" s="6"/>
       <c r="F98" s="6"/>
@@ -32770,10 +33662,16 @@
       <c r="Y98" s="6"/>
       <c r="Z98" s="6"/>
     </row>
-    <row r="99" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A99" s="6"/>
-      <c r="B99" s="6"/>
-      <c r="C99" s="8"/>
+    <row r="99" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="B99" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="C99" s="7">
+        <v>46198</v>
+      </c>
       <c r="D99" s="6"/>
       <c r="E99" s="6"/>
       <c r="F99" s="6"/>
@@ -32798,10 +33696,16 @@
       <c r="Y99" s="6"/>
       <c r="Z99" s="6"/>
     </row>
-    <row r="100" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A100" s="6"/>
-      <c r="B100" s="6"/>
-      <c r="C100" s="8"/>
+    <row r="100" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="11" t="s">
+        <v>306</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="C100" s="7">
+        <v>46199</v>
+      </c>
       <c r="D100" s="6"/>
       <c r="E100" s="6"/>
       <c r="F100" s="6"/>
@@ -32826,10 +33730,16 @@
       <c r="Y100" s="6"/>
       <c r="Z100" s="6"/>
     </row>
-    <row r="101" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A101" s="6"/>
-      <c r="B101" s="6"/>
-      <c r="C101" s="8"/>
+    <row r="101" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C101" s="7">
+        <v>46200</v>
+      </c>
       <c r="D101" s="6"/>
       <c r="E101" s="6"/>
       <c r="F101" s="6"/>
@@ -32854,10 +33764,16 @@
       <c r="Y101" s="6"/>
       <c r="Z101" s="6"/>
     </row>
-    <row r="102" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A102" s="6"/>
-      <c r="B102" s="6"/>
-      <c r="C102" s="8"/>
+    <row r="102" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="11" t="s">
+        <v>308</v>
+      </c>
+      <c r="B102" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C102" s="7">
+        <v>46201</v>
+      </c>
       <c r="D102" s="6"/>
       <c r="E102" s="6"/>
       <c r="F102" s="6"/>
@@ -32882,10 +33798,16 @@
       <c r="Y102" s="6"/>
       <c r="Z102" s="6"/>
     </row>
-    <row r="103" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A103" s="6"/>
-      <c r="B103" s="6"/>
-      <c r="C103" s="8"/>
+    <row r="103" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="11" t="s">
+        <v>309</v>
+      </c>
+      <c r="B103" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C103" s="7">
+        <v>46202</v>
+      </c>
       <c r="D103" s="6"/>
       <c r="E103" s="6"/>
       <c r="F103" s="6"/>
@@ -32910,10 +33832,16 @@
       <c r="Y103" s="6"/>
       <c r="Z103" s="6"/>
     </row>
-    <row r="104" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A104" s="6"/>
-      <c r="B104" s="6"/>
-      <c r="C104" s="8"/>
+    <row r="104" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="11" t="s">
+        <v>310</v>
+      </c>
+      <c r="B104" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C104" s="7">
+        <v>46203</v>
+      </c>
       <c r="D104" s="6"/>
       <c r="E104" s="6"/>
       <c r="F104" s="6"/>
@@ -32938,10 +33866,16 @@
       <c r="Y104" s="6"/>
       <c r="Z104" s="6"/>
     </row>
-    <row r="105" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A105" s="6"/>
-      <c r="B105" s="6"/>
-      <c r="C105" s="8"/>
+    <row r="105" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A105" s="11" t="s">
+        <v>311</v>
+      </c>
+      <c r="B105" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C105" s="7">
+        <v>46204</v>
+      </c>
       <c r="D105" s="6"/>
       <c r="E105" s="6"/>
       <c r="F105" s="6"/>
@@ -32966,10 +33900,16 @@
       <c r="Y105" s="6"/>
       <c r="Z105" s="6"/>
     </row>
-    <row r="106" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A106" s="6"/>
-      <c r="B106" s="6"/>
-      <c r="C106" s="8"/>
+    <row r="106" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A106" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="B106" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C106" s="7">
+        <v>46205</v>
+      </c>
       <c r="D106" s="6"/>
       <c r="E106" s="6"/>
       <c r="F106" s="6"/>
@@ -32994,10 +33934,16 @@
       <c r="Y106" s="6"/>
       <c r="Z106" s="6"/>
     </row>
-    <row r="107" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A107" s="6"/>
-      <c r="B107" s="6"/>
-      <c r="C107" s="8"/>
+    <row r="107" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A107" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="B107" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="C107" s="7">
+        <v>46206</v>
+      </c>
       <c r="D107" s="6"/>
       <c r="E107" s="6"/>
       <c r="F107" s="6"/>
@@ -33022,10 +33968,16 @@
       <c r="Y107" s="6"/>
       <c r="Z107" s="6"/>
     </row>
-    <row r="108" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A108" s="6"/>
-      <c r="B108" s="6"/>
-      <c r="C108" s="8"/>
+    <row r="108" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A108" s="11" t="s">
+        <v>314</v>
+      </c>
+      <c r="B108" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="C108" s="7">
+        <v>46207</v>
+      </c>
       <c r="D108" s="6"/>
       <c r="E108" s="6"/>
       <c r="F108" s="6"/>
@@ -33050,10 +34002,16 @@
       <c r="Y108" s="6"/>
       <c r="Z108" s="6"/>
     </row>
-    <row r="109" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A109" s="6"/>
-      <c r="B109" s="6"/>
-      <c r="C109" s="8"/>
+    <row r="109" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A109" s="11" t="s">
+        <v>315</v>
+      </c>
+      <c r="B109" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="C109" s="7">
+        <v>46208</v>
+      </c>
       <c r="D109" s="6"/>
       <c r="E109" s="6"/>
       <c r="F109" s="6"/>
@@ -56622,6 +57580,37 @@
     <hyperlink ref="A76" r:id="rId75" xr:uid="{75E7BB78-DF66-4014-A336-4686E780F9BF}"/>
     <hyperlink ref="A77" r:id="rId76" xr:uid="{DE1E9B7F-5063-48B2-8A6A-ED3B133AEE70}"/>
     <hyperlink ref="A78" r:id="rId77" xr:uid="{4C325121-69F3-47B7-B8BA-1C9C5CF3F4C5}"/>
+    <hyperlink ref="A79" r:id="rId78" xr:uid="{5DA25033-4D10-4F3B-BE90-A104656764C2}"/>
+    <hyperlink ref="A80" r:id="rId79" display="https://www.youtube.com/watch?v=v0k-3xubT_A&amp;t=2s" xr:uid="{7B9BA893-3442-4805-97A8-C50FD91FC960}"/>
+    <hyperlink ref="A81" r:id="rId80" display="https://www.youtube.com/watch?v=g-a3_i0nbDI&amp;t=3s" xr:uid="{102E8EB1-FB7C-4BA7-9F03-B31273897B85}"/>
+    <hyperlink ref="A82" r:id="rId81" display="https://www.youtube.com/watch?v=nriQoD9a1P0&amp;t=156s" xr:uid="{833DD344-6E49-4B94-9C1F-6C7FDF63BD51}"/>
+    <hyperlink ref="A83" r:id="rId82" display="https://www.youtube.com/watch?v=UK5oPnC023c&amp;t=1s" xr:uid="{302BEBA4-F5A8-4D5E-948B-392F872395DF}"/>
+    <hyperlink ref="A84" r:id="rId83" xr:uid="{7788D9A0-8B42-4C58-8CA9-2B4DA5235DC9}"/>
+    <hyperlink ref="A85" r:id="rId84" xr:uid="{419AD8BF-CCE6-4DAD-AC5F-51E3AA2DDC2A}"/>
+    <hyperlink ref="A86" r:id="rId85" display="https://www.youtube.com/watch?v=JwME3EdY2Iw&amp;t=1387s" xr:uid="{BF8C886D-34FD-49DB-9223-8B3F56ECC3B1}"/>
+    <hyperlink ref="A87" r:id="rId86" display="https://www.youtube.com/watch?v=IEVZuutf3mc&amp;t=1s" xr:uid="{C79B5A95-2AC3-4809-9511-1C20CD0714B6}"/>
+    <hyperlink ref="A88" r:id="rId87" display="https://www.youtube.com/watch?v=De-oTCuZ0uc&amp;t=2s" xr:uid="{D051B3FD-9134-455E-9CAF-FCF83A0C1686}"/>
+    <hyperlink ref="A89" r:id="rId88" display="https://www.youtube.com/watch?v=AQjB4UAv0ts&amp;t=1s" xr:uid="{B10D1AC6-6262-4174-BE71-B0F47702A823}"/>
+    <hyperlink ref="A90" r:id="rId89" xr:uid="{20BB80A8-CD1E-4A35-B4E1-19C2169F4ED2}"/>
+    <hyperlink ref="A91" r:id="rId90" display="https://www.youtube.com/watch?v=l9JJ2kI5x6c&amp;t=29s" xr:uid="{CAEC6860-25E1-471C-B75C-A83D608D85CD}"/>
+    <hyperlink ref="A92" r:id="rId91" display="https://www.youtube.com/watch?v=UD5noYvuVFc&amp;t=1s" xr:uid="{F131F53A-6A69-457B-A473-071D6A1AEDE8}"/>
+    <hyperlink ref="A93" r:id="rId92" display="https://www.youtube.com/watch?v=aiy6IqoBZgk&amp;t=526s" xr:uid="{13251C89-7F80-474E-AD01-9FAFF26B8676}"/>
+    <hyperlink ref="A94" r:id="rId93" xr:uid="{660C8834-DDBB-4CFE-898E-1B8B7E095B66}"/>
+    <hyperlink ref="A95" r:id="rId94" display="https://www.youtube.com/watch?v=Vt4XZNHQ_lk&amp;t=1s" xr:uid="{C2ABA024-0A03-46F9-A2D3-864A1DA63D5C}"/>
+    <hyperlink ref="A96" r:id="rId95" display="https://www.youtube.com/watch?v=BERqX0kQIJU&amp;t=21s" xr:uid="{5B43D85A-0FD3-4784-B894-0FF63026FCEF}"/>
+    <hyperlink ref="A97" r:id="rId96" display="https://www.youtube.com/watch?v=_4fom5vhdyQ&amp;t=243s" xr:uid="{9AB26B01-2E32-4723-B2DE-41898FA857D0}"/>
+    <hyperlink ref="A98" r:id="rId97" display="https://www.youtube.com/watch?v=_4fom5vhdyQ&amp;t=243s" xr:uid="{D36C1FA2-F247-44F6-A363-B404570F9D0E}"/>
+    <hyperlink ref="A99" r:id="rId98" display="https://www.youtube.com/watch?v=Ut4UXig7mWQ&amp;t=38s" xr:uid="{46F42C0D-0C9B-4EC1-9976-88B18AA6FFA5}"/>
+    <hyperlink ref="A100" r:id="rId99" xr:uid="{C12692FC-F9B6-4733-9A70-8FD7739D382A}"/>
+    <hyperlink ref="A101" r:id="rId100" display="https://www.youtube.com/watch?v=igYTZO49JS8&amp;t=3s" xr:uid="{838CF357-F057-4BF1-AE55-43D6C276CD5B}"/>
+    <hyperlink ref="A102" r:id="rId101" xr:uid="{5F29FC01-779B-46EC-AD66-E5689D454F01}"/>
+    <hyperlink ref="A103" r:id="rId102" display="https://www.youtube.com/watch?v=i8v5Fb_aDW8&amp;t=1s" xr:uid="{0FC6439D-AAD9-4590-B4CE-0F3B2444FE0D}"/>
+    <hyperlink ref="A104" r:id="rId103" display="https://www.youtube.com/watch?v=Iu8AoQz7N0g&amp;t=2s" xr:uid="{D07B0666-9C6B-4E96-A346-8823A6EC563B}"/>
+    <hyperlink ref="A105" r:id="rId104" display="https://www.youtube.com/watch?v=fH_TTaOlwiY&amp;t=1s" xr:uid="{DF208513-408A-449C-9C54-FE4DE9E41600}"/>
+    <hyperlink ref="A106" r:id="rId105" xr:uid="{D90BA747-35F2-430F-A5E3-EE15BB400E1E}"/>
+    <hyperlink ref="A107" r:id="rId106" display="https://www.youtube.com/watch?v=U9FN1AMGujA&amp;t=8s" xr:uid="{B16CD34E-9D32-4CA6-A89F-AEAAE72430F2}"/>
+    <hyperlink ref="A108" r:id="rId107" xr:uid="{234CC86D-47B3-4630-8C23-0C9F599CA73C}"/>
+    <hyperlink ref="A109" r:id="rId108" display="https://www.youtube.com/watch?v=gOFEVX_YC4k&amp;t=54s" xr:uid="{A49D831C-CF59-450C-BA85-4E2DDEAEC907}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
new daily listening added
</commit_message>
<xml_diff>
--- a/public/Daily Sadhana.xlsx
+++ b/public/Daily Sadhana.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sahaa\Documents\github_anandasvarupa\give_web\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F157EE2E-7221-4A84-8C21-0E639FB25753}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8816264A-140B-4C26-9259-258AA92B200F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1273" uniqueCount="528">
   <si>
     <t>url</t>
   </si>
@@ -1249,6 +1249,369 @@
   <si>
     <t>Today's listening to Srila Prabhupada - 227</t>
   </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=IEZVq01Q7go</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=jiFJXvMc2SY</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=fr6B3EtlZVM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=PBNhMcRKu24</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ZHFNRrT8WA4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=mXLQFJ-W7xc</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=gN9bQHaOKg8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=BXylPudUUek</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=tbluAPW3aLs</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=6u3ZNTvmQAI</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=WhQTbrP-HFM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=DtLPcgkw0mM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Yd38cByixQE</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=lXOsdbNL5lg</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=UGGJBgg4064</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Y1MU9Z4qP_8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=SkUK89Mp5Zc</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=8e4gw8yeQIo</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=8FH3k4foVIw</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=EQtDBtPA5oM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=AxSLP6fwE-E</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=tBIG11CRXmM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=S-ZrxzifoQ0</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=8anpFagF9VU</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=cx2wkrKymok</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=sQK0VjZqs-g</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=r1LzlV1lPRk</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=tIEfQYHiSgY</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=-5m27NO8AP4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=zTcUuXS6i4Q</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=5RbaPlzKbFk</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=lIrOM7FbYts</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=5KsLgOZmb-I</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=GNiV-xOIqwo</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=bQfWMQFzU14</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Hm-A0QLvOmI</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=yY7yaqJomcs</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=vcnndeYVw9k</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Y1zBcg4QJgE</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=1Ilgi75Y6Ac</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=F09CIYFG30g</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=TJI67LY52Os</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=V4RzPKgzWmk</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=zgLWXkOMOGE</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=r-DPvpwMOdw</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=4sMrz_5leyI</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=s8ips1eyAF4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=6E_PDZdGuZs</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=7DlCphkX0b4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=X6XNEMBmPrk</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=S7rTG9pCQB8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=EYJjJX076X8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=qCOWcKURVzk</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=7owmPnw27iw</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=IS1Fcnh-W-M</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Rssbr11AO1o</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=7rdJOSgHgg4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=sQgepxd5T5A</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=tS58CDMrFxA</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 228</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 229</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 230</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 231</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 232</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 233</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 234</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 235</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 236</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 237</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 238</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 239</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 240</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 241</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 242</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 243</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 244</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 245</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 246</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 247</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 248</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 249</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 250</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 251</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 252</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 253</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 254</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 255</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 256</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 257</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 258</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 259</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 260</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 261</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 262</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 263</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 264</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 265</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 266</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 267</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 268</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 269</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 270</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 271</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 272</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 273</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 274</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 275</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 276</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 277</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 278</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 279</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 280</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 281</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 282</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 283</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 284</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 285</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 286</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 287</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 288</t>
+  </si>
+  <si>
+    <t>Today's listening to Srila Prabhupada - 289</t>
+  </si>
 </sst>
 </file>
 
@@ -1649,7 +2012,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z134"/>
+  <dimension ref="A1:Z196"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="56.81640625" customWidth="1"/>
@@ -3152,6 +3515,688 @@
       </c>
       <c r="C134" s="5">
         <v>46238</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A135" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="B135" s="6" t="s">
+        <v>466</v>
+      </c>
+      <c r="C135" s="5">
+        <v>46239</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A136" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="B136" s="6" t="s">
+        <v>467</v>
+      </c>
+      <c r="C136" s="5">
+        <v>46240</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A137" s="11" t="s">
+        <v>409</v>
+      </c>
+      <c r="B137" s="6" t="s">
+        <v>468</v>
+      </c>
+      <c r="C137" s="5">
+        <v>46241</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A138" s="11" t="s">
+        <v>410</v>
+      </c>
+      <c r="B138" s="6" t="s">
+        <v>469</v>
+      </c>
+      <c r="C138" s="5">
+        <v>46242</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A139" s="11" t="s">
+        <v>411</v>
+      </c>
+      <c r="B139" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="C139" s="5">
+        <v>46243</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A140" s="11" t="s">
+        <v>412</v>
+      </c>
+      <c r="B140" s="6" t="s">
+        <v>471</v>
+      </c>
+      <c r="C140" s="5">
+        <v>46244</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A141" s="11" t="s">
+        <v>413</v>
+      </c>
+      <c r="B141" s="6" t="s">
+        <v>472</v>
+      </c>
+      <c r="C141" s="5">
+        <v>46245</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A142" s="11" t="s">
+        <v>414</v>
+      </c>
+      <c r="B142" s="6" t="s">
+        <v>473</v>
+      </c>
+      <c r="C142" s="5">
+        <v>46246</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A143" s="11" t="s">
+        <v>415</v>
+      </c>
+      <c r="B143" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="C143" s="5">
+        <v>46247</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A144" s="11" t="s">
+        <v>416</v>
+      </c>
+      <c r="B144" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="C144" s="5">
+        <v>46248</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A145" s="11" t="s">
+        <v>417</v>
+      </c>
+      <c r="B145" s="6" t="s">
+        <v>476</v>
+      </c>
+      <c r="C145" s="5">
+        <v>46249</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A146" s="11" t="s">
+        <v>418</v>
+      </c>
+      <c r="B146" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="C146" s="5">
+        <v>46250</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A147" s="11" t="s">
+        <v>419</v>
+      </c>
+      <c r="B147" s="6" t="s">
+        <v>478</v>
+      </c>
+      <c r="C147" s="5">
+        <v>46251</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A148" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="B148" s="6" t="s">
+        <v>479</v>
+      </c>
+      <c r="C148" s="5">
+        <v>46252</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A149" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="B149" s="6" t="s">
+        <v>480</v>
+      </c>
+      <c r="C149" s="5">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A150" s="11" t="s">
+        <v>422</v>
+      </c>
+      <c r="B150" s="6" t="s">
+        <v>481</v>
+      </c>
+      <c r="C150" s="5">
+        <v>46254</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A151" s="11" t="s">
+        <v>423</v>
+      </c>
+      <c r="B151" s="6" t="s">
+        <v>482</v>
+      </c>
+      <c r="C151" s="5">
+        <v>46255</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A152" s="11" t="s">
+        <v>309</v>
+      </c>
+      <c r="B152" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="C152" s="5">
+        <v>46256</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A153" s="11" t="s">
+        <v>424</v>
+      </c>
+      <c r="B153" s="6" t="s">
+        <v>484</v>
+      </c>
+      <c r="C153" s="5">
+        <v>46257</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A154" s="11" t="s">
+        <v>425</v>
+      </c>
+      <c r="B154" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="C154" s="5">
+        <v>46258</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A155" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="B155" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="C155" s="5">
+        <v>46259</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A156" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="B156" s="6" t="s">
+        <v>487</v>
+      </c>
+      <c r="C156" s="5">
+        <v>46260</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A157" s="11" t="s">
+        <v>428</v>
+      </c>
+      <c r="B157" s="6" t="s">
+        <v>488</v>
+      </c>
+      <c r="C157" s="5">
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A158" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="B158" s="6" t="s">
+        <v>489</v>
+      </c>
+      <c r="C158" s="5">
+        <v>46262</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A159" s="11" t="s">
+        <v>430</v>
+      </c>
+      <c r="B159" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="C159" s="5">
+        <v>46263</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A160" s="11" t="s">
+        <v>431</v>
+      </c>
+      <c r="B160" s="6" t="s">
+        <v>491</v>
+      </c>
+      <c r="C160" s="5">
+        <v>46264</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A161" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="B161" s="6" t="s">
+        <v>492</v>
+      </c>
+      <c r="C161" s="5">
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A162" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="B162" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="C162" s="5">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A163" s="11" t="s">
+        <v>434</v>
+      </c>
+      <c r="B163" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="C163" s="5">
+        <v>46267</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A164" s="11" t="s">
+        <v>435</v>
+      </c>
+      <c r="B164" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="C164" s="5">
+        <v>46268</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A165" s="11" t="s">
+        <v>413</v>
+      </c>
+      <c r="B165" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="C165" s="5">
+        <v>46269</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A166" s="11" t="s">
+        <v>436</v>
+      </c>
+      <c r="B166" s="6" t="s">
+        <v>497</v>
+      </c>
+      <c r="C166" s="5">
+        <v>46270</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A167" s="11" t="s">
+        <v>437</v>
+      </c>
+      <c r="B167" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C167" s="5">
+        <v>46271</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A168" s="11" t="s">
+        <v>438</v>
+      </c>
+      <c r="B168" s="6" t="s">
+        <v>499</v>
+      </c>
+      <c r="C168" s="5">
+        <v>46272</v>
+      </c>
+    </row>
+    <row r="169" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A169" s="11" t="s">
+        <v>439</v>
+      </c>
+      <c r="B169" s="6" t="s">
+        <v>500</v>
+      </c>
+      <c r="C169" s="5">
+        <v>46273</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A170" s="11" t="s">
+        <v>440</v>
+      </c>
+      <c r="B170" s="6" t="s">
+        <v>501</v>
+      </c>
+      <c r="C170" s="5">
+        <v>46274</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A171" s="11" t="s">
+        <v>441</v>
+      </c>
+      <c r="B171" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="C171" s="5">
+        <v>46275</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A172" s="11" t="s">
+        <v>442</v>
+      </c>
+      <c r="B172" s="6" t="s">
+        <v>503</v>
+      </c>
+      <c r="C172" s="5">
+        <v>46276</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A173" s="11" t="s">
+        <v>443</v>
+      </c>
+      <c r="B173" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="C173" s="5">
+        <v>46277</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A174" s="11" t="s">
+        <v>444</v>
+      </c>
+      <c r="B174" s="6" t="s">
+        <v>505</v>
+      </c>
+      <c r="C174" s="5">
+        <v>46278</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A175" s="11" t="s">
+        <v>445</v>
+      </c>
+      <c r="B175" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="C175" s="5">
+        <v>46279</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A176" s="11" t="s">
+        <v>446</v>
+      </c>
+      <c r="B176" s="6" t="s">
+        <v>507</v>
+      </c>
+      <c r="C176" s="5">
+        <v>46280</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A177" s="11" t="s">
+        <v>447</v>
+      </c>
+      <c r="B177" s="6" t="s">
+        <v>508</v>
+      </c>
+      <c r="C177" s="5">
+        <v>46281</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A178" s="11" t="s">
+        <v>448</v>
+      </c>
+      <c r="B178" s="6" t="s">
+        <v>509</v>
+      </c>
+      <c r="C178" s="5">
+        <v>46282</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A179" s="11" t="s">
+        <v>449</v>
+      </c>
+      <c r="B179" s="6" t="s">
+        <v>510</v>
+      </c>
+      <c r="C179" s="5">
+        <v>46283</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A180" s="11" t="s">
+        <v>450</v>
+      </c>
+      <c r="B180" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="C180" s="5">
+        <v>46284</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A181" s="11" t="s">
+        <v>451</v>
+      </c>
+      <c r="B181" s="6" t="s">
+        <v>512</v>
+      </c>
+      <c r="C181" s="5">
+        <v>46285</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A182" s="11" t="s">
+        <v>452</v>
+      </c>
+      <c r="B182" s="6" t="s">
+        <v>513</v>
+      </c>
+      <c r="C182" s="5">
+        <v>46286</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A183" s="11" t="s">
+        <v>453</v>
+      </c>
+      <c r="B183" s="6" t="s">
+        <v>514</v>
+      </c>
+      <c r="C183" s="5">
+        <v>46287</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A184" s="11" t="s">
+        <v>454</v>
+      </c>
+      <c r="B184" s="6" t="s">
+        <v>515</v>
+      </c>
+      <c r="C184" s="5">
+        <v>46288</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A185" s="11" t="s">
+        <v>455</v>
+      </c>
+      <c r="B185" s="6" t="s">
+        <v>516</v>
+      </c>
+      <c r="C185" s="5">
+        <v>46289</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A186" s="11" t="s">
+        <v>456</v>
+      </c>
+      <c r="B186" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C186" s="5">
+        <v>46290</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A187" s="11" t="s">
+        <v>457</v>
+      </c>
+      <c r="B187" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="C187" s="5">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A188" s="11" t="s">
+        <v>458</v>
+      </c>
+      <c r="B188" s="6" t="s">
+        <v>519</v>
+      </c>
+      <c r="C188" s="5">
+        <v>46292</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A189" s="11" t="s">
+        <v>459</v>
+      </c>
+      <c r="B189" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="C189" s="5">
+        <v>46293</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A190" s="11" t="s">
+        <v>460</v>
+      </c>
+      <c r="B190" s="6" t="s">
+        <v>521</v>
+      </c>
+      <c r="C190" s="5">
+        <v>46294</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A191" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="B191" s="6" t="s">
+        <v>522</v>
+      </c>
+      <c r="C191" s="5">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A192" s="11" t="s">
+        <v>461</v>
+      </c>
+      <c r="B192" s="6" t="s">
+        <v>523</v>
+      </c>
+      <c r="C192" s="5">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A193" s="11" t="s">
+        <v>462</v>
+      </c>
+      <c r="B193" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="C193" s="5">
+        <v>46297</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A194" s="11" t="s">
+        <v>463</v>
+      </c>
+      <c r="B194" s="6" t="s">
+        <v>525</v>
+      </c>
+      <c r="C194" s="5">
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="195" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A195" s="11" t="s">
+        <v>464</v>
+      </c>
+      <c r="B195" s="6" t="s">
+        <v>526</v>
+      </c>
+      <c r="C195" s="5">
+        <v>46299</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A196" s="11" t="s">
+        <v>465</v>
+      </c>
+      <c r="B196" s="6" t="s">
+        <v>527</v>
+      </c>
+      <c r="C196" s="5">
+        <v>46300</v>
       </c>
     </row>
   </sheetData>
@@ -3290,9 +4335,71 @@
     <hyperlink ref="A132" r:id="rId131" xr:uid="{44367F7B-ADC1-4D8C-84B6-A16DD96C1EEB}"/>
     <hyperlink ref="A133" r:id="rId132" xr:uid="{5929A428-4297-4A8E-9082-39B244B7BDCC}"/>
     <hyperlink ref="A134" r:id="rId133" xr:uid="{BB847391-36FC-4DAB-A9BA-709947B20823}"/>
+    <hyperlink ref="A135" r:id="rId134" display="https://www.youtube.com/watch?v=IEZVq01Q7go&amp;t=14s" xr:uid="{32D29B3A-A161-4690-819D-5E5148452239}"/>
+    <hyperlink ref="A136" r:id="rId135" display="https://www.youtube.com/watch?v=jiFJXvMc2SY&amp;t=321s" xr:uid="{8519747E-3570-47F8-94F1-32D85A4E036E}"/>
+    <hyperlink ref="A137" r:id="rId136" display="https://www.youtube.com/watch?v=fr6B3EtlZVM&amp;t=3s" xr:uid="{661692C7-0FEE-4366-8AE9-9BD22F833B2A}"/>
+    <hyperlink ref="A138" r:id="rId137" display="https://www.youtube.com/watch?v=PBNhMcRKu24&amp;t=1s" xr:uid="{C31123FA-8E40-437B-88A7-3401AD266B73}"/>
+    <hyperlink ref="A139" r:id="rId138" display="https://www.youtube.com/watch?v=ZHFNRrT8WA4&amp;t=3s" xr:uid="{206B54D7-243C-4F7E-98E6-4EF567951608}"/>
+    <hyperlink ref="A140" r:id="rId139" display="https://www.youtube.com/watch?v=mXLQFJ-W7xc&amp;t=23s" xr:uid="{AC61567E-6618-418A-8AFF-64456F118B2B}"/>
+    <hyperlink ref="A141" r:id="rId140" display="https://www.youtube.com/watch?v=gN9bQHaOKg8&amp;t=96s" xr:uid="{97360246-5947-4BFC-A72F-A15F08905474}"/>
+    <hyperlink ref="A142" r:id="rId141" display="https://www.youtube.com/watch?v=BXylPudUUek&amp;t=13s" xr:uid="{FFE0B416-A80D-48B6-8D05-3CF0F67C94A0}"/>
+    <hyperlink ref="A143" r:id="rId142" display="https://www.youtube.com/watch?v=tbluAPW3aLs&amp;t=3s" xr:uid="{FFD7F37A-3A98-4F65-B5BC-2363E1D31539}"/>
+    <hyperlink ref="A144" r:id="rId143" xr:uid="{0C59AF75-CF36-42F2-93A0-C867D4FF9431}"/>
+    <hyperlink ref="A145" r:id="rId144" xr:uid="{C0DB5623-38DA-49D0-8FBE-14C38E627CFD}"/>
+    <hyperlink ref="A146" r:id="rId145" xr:uid="{A7CFD07A-06E9-4A59-B659-37E7C4EB0262}"/>
+    <hyperlink ref="A147" r:id="rId146" xr:uid="{2C3DA091-DE31-4887-BACA-9C15A11DC82B}"/>
+    <hyperlink ref="A148" r:id="rId147" xr:uid="{1938B025-A903-4BB2-80F3-363EA0243E81}"/>
+    <hyperlink ref="A149" r:id="rId148" xr:uid="{FC0979CE-3EA4-48F9-A949-52028EEF01F5}"/>
+    <hyperlink ref="A150" r:id="rId149" xr:uid="{B0110974-D859-48C6-BC65-D97514171BCB}"/>
+    <hyperlink ref="A151" r:id="rId150" xr:uid="{0BCF23CB-29AC-4B36-AB75-016CF0A70C19}"/>
+    <hyperlink ref="A152" r:id="rId151" display="https://www.youtube.com/watch?v=i8v5Fb_aDW8&amp;t=351s" xr:uid="{676E1168-F529-4D8C-8B84-F1A8A63AB908}"/>
+    <hyperlink ref="A153" r:id="rId152" display="https://www.youtube.com/watch?v=8e4gw8yeQIo&amp;t=109s" xr:uid="{40E37FA6-C11B-4AE7-808E-97C215696326}"/>
+    <hyperlink ref="A154" r:id="rId153" xr:uid="{0ED37E9C-23E6-4A2C-BDE6-107F33901A09}"/>
+    <hyperlink ref="A155" r:id="rId154" xr:uid="{3AEFD97F-C633-460B-9296-45ACE6CDE7C3}"/>
+    <hyperlink ref="A156" r:id="rId155" xr:uid="{295BA521-B71C-4592-851D-7329B0487310}"/>
+    <hyperlink ref="A157" r:id="rId156" display="https://www.youtube.com/watch?v=tBIG11CRXmM&amp;t=14s" xr:uid="{7F012730-E8DE-40EB-8AF9-8EE661217A9C}"/>
+    <hyperlink ref="A158" r:id="rId157" display="https://www.youtube.com/watch?v=S-ZrxzifoQ0&amp;t=3s" xr:uid="{726EDF0F-F13D-4714-8B81-5926AC807DB8}"/>
+    <hyperlink ref="A159" r:id="rId158" display="https://www.youtube.com/watch?v=8anpFagF9VU&amp;t=23s" xr:uid="{BD3E941A-54F3-40EC-ADF4-78044B2CC85D}"/>
+    <hyperlink ref="A160" r:id="rId159" display="https://www.youtube.com/watch?v=cx2wkrKymok&amp;t=221s" xr:uid="{A5BE64BE-5D94-4EC7-8F66-D6A940C3F42B}"/>
+    <hyperlink ref="A161" r:id="rId160" xr:uid="{B9BE74F2-CDBC-4467-87EF-640398285821}"/>
+    <hyperlink ref="A162" r:id="rId161" xr:uid="{734D9C5C-7DDC-41F9-BF0F-8965328A525B}"/>
+    <hyperlink ref="A163" r:id="rId162" xr:uid="{C397F3DF-0441-4769-A814-A201AD723B05}"/>
+    <hyperlink ref="A164" r:id="rId163" xr:uid="{C8C8755A-99A4-4164-9F5A-C9D8C343820C}"/>
+    <hyperlink ref="A165" r:id="rId164" xr:uid="{6CD31249-2227-460C-A21A-6707E30B4E36}"/>
+    <hyperlink ref="A166" r:id="rId165" xr:uid="{26E7BFD3-01EF-4508-B3E3-B356BA9ECCCA}"/>
+    <hyperlink ref="A167" r:id="rId166" display="https://www.youtube.com/watch?v=5RbaPlzKbFk&amp;t=6s" xr:uid="{584521F5-3524-452B-8C17-8C383539CB03}"/>
+    <hyperlink ref="A168" r:id="rId167" xr:uid="{15D72B4B-230A-4776-A0A8-A228C0FBB147}"/>
+    <hyperlink ref="A169" r:id="rId168" xr:uid="{3791A13D-6B40-4E68-9693-34E2A7641003}"/>
+    <hyperlink ref="A170" r:id="rId169" xr:uid="{760E4DBA-4E08-452E-8A14-9B574DCFF1A9}"/>
+    <hyperlink ref="A171" r:id="rId170" xr:uid="{B393D8A8-B578-4614-A75A-D71AC5F431D4}"/>
+    <hyperlink ref="A172" r:id="rId171" xr:uid="{32E5E549-B5B1-49BF-9316-D5FBEA78A19A}"/>
+    <hyperlink ref="A173" r:id="rId172" xr:uid="{13668FB1-A7B6-4206-AD12-DA880CB28D69}"/>
+    <hyperlink ref="A174" r:id="rId173" display="https://www.youtube.com/watch?v=vcnndeYVw9k&amp;t=4s" xr:uid="{28188605-A039-4464-AA26-26639E657847}"/>
+    <hyperlink ref="A175" r:id="rId174" display="https://www.youtube.com/watch?v=Y1zBcg4QJgE&amp;t=8s" xr:uid="{19A05DD3-3F1B-4E9B-82DC-6E02D24AD960}"/>
+    <hyperlink ref="A176" r:id="rId175" display="https://www.youtube.com/watch?v=1Ilgi75Y6Ac&amp;t=9s" xr:uid="{6EA4F39A-087E-40C8-80FA-0F9C19A1671A}"/>
+    <hyperlink ref="A177" r:id="rId176" xr:uid="{DCCC24F2-01BF-4608-9767-4A0A78827B09}"/>
+    <hyperlink ref="A178" r:id="rId177" xr:uid="{06C26E17-1680-4247-A82B-794F05729286}"/>
+    <hyperlink ref="A179" r:id="rId178" xr:uid="{5645E3B6-E403-4F60-B7F8-B3EDB58256D8}"/>
+    <hyperlink ref="A180" r:id="rId179" display="https://www.youtube.com/watch?v=zgLWXkOMOGE&amp;t=20s" xr:uid="{09527CE3-C7F9-4C9A-B230-6069D300E042}"/>
+    <hyperlink ref="A181" r:id="rId180" display="https://www.youtube.com/watch?v=r-DPvpwMOdw&amp;t=144s" xr:uid="{72B96006-BA54-4D42-8F61-80B2F8DDD887}"/>
+    <hyperlink ref="A182" r:id="rId181" xr:uid="{DE808E75-5A53-455A-8648-84BA20456B34}"/>
+    <hyperlink ref="A183" r:id="rId182" xr:uid="{A0D0A24B-BDB5-42D0-95EC-FC1AF7CB6101}"/>
+    <hyperlink ref="A184" r:id="rId183" xr:uid="{287F3C8A-8B17-4809-9470-B948069F6CE0}"/>
+    <hyperlink ref="A185" r:id="rId184" xr:uid="{CA8DE3ED-F548-4707-BB76-C6DBFD5C71C4}"/>
+    <hyperlink ref="A186" r:id="rId185" display="https://www.youtube.com/watch?v=X6XNEMBmPrk&amp;t=149s" xr:uid="{1CFE2E1A-F0CC-4997-BF2A-4C5D1C936D58}"/>
+    <hyperlink ref="A187" r:id="rId186" xr:uid="{EE2F52E2-9A3A-477F-9ABF-A3754BA14319}"/>
+    <hyperlink ref="A188" r:id="rId187" xr:uid="{C5A32D11-4AAF-4E67-8FC9-0E0497844142}"/>
+    <hyperlink ref="A189" r:id="rId188" display="https://www.youtube.com/watch?v=qCOWcKURVzk&amp;t=1s" xr:uid="{C2E7176C-E865-4D2D-B62F-F95B7903C556}"/>
+    <hyperlink ref="A190" r:id="rId189" xr:uid="{A45BC7FA-A440-4F1B-BB1B-55C1716C51EE}"/>
+    <hyperlink ref="A191" r:id="rId190" display="https://www.youtube.com/watch?v=-NHHdVWUcwo&amp;t=3s" xr:uid="{655E5248-B9A8-4E1D-AD5E-8F1461CD7490}"/>
+    <hyperlink ref="A192" r:id="rId191" display="https://www.youtube.com/watch?v=IS1Fcnh-W-M&amp;t=9s" xr:uid="{E3FCD810-E15F-4E52-A6BB-C672C3603155}"/>
+    <hyperlink ref="A193" r:id="rId192" display="https://www.youtube.com/watch?v=Rssbr11AO1o&amp;t=1s" xr:uid="{9F021A1A-C8C8-46B5-916F-C322CD757894}"/>
+    <hyperlink ref="A194" r:id="rId193" display="https://www.youtube.com/watch?v=7rdJOSgHgg4&amp;t=559s" xr:uid="{E32B95CD-2286-4E4C-A479-248D65243279}"/>
+    <hyperlink ref="A195" r:id="rId194" xr:uid="{1D736B2E-23D1-45FB-932F-B87290328240}"/>
+    <hyperlink ref="A196" r:id="rId195" display="https://www.youtube.com/watch?v=tS58CDMrFxA&amp;t=23s" xr:uid="{DB8FD2AE-9C9C-411A-AD03-265E506F09A4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId134"/>
+  <pageSetup orientation="portrait" r:id="rId196"/>
 </worksheet>
 </file>
 
@@ -9294,10 +10401,16 @@
       <c r="Y176" s="6"/>
       <c r="Z176" s="6"/>
     </row>
-    <row r="177" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A177" s="6"/>
-      <c r="B177" s="6"/>
-      <c r="C177" s="6"/>
+    <row r="177" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A177" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="B177" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="C177" s="5">
+        <v>46239</v>
+      </c>
       <c r="D177" s="6"/>
       <c r="E177" s="6"/>
       <c r="F177" s="6"/>
@@ -9322,10 +10435,16 @@
       <c r="Y177" s="6"/>
       <c r="Z177" s="6"/>
     </row>
-    <row r="178" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A178" s="6"/>
-      <c r="B178" s="6"/>
-      <c r="C178" s="6"/>
+    <row r="178" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A178" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="B178" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="C178" s="5">
+        <v>46240</v>
+      </c>
       <c r="D178" s="6"/>
       <c r="E178" s="6"/>
       <c r="F178" s="6"/>
@@ -9350,10 +10469,16 @@
       <c r="Y178" s="6"/>
       <c r="Z178" s="6"/>
     </row>
-    <row r="179" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A179" s="6"/>
-      <c r="B179" s="6"/>
-      <c r="C179" s="6"/>
+    <row r="179" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A179" s="11" t="s">
+        <v>409</v>
+      </c>
+      <c r="B179" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="C179" s="5">
+        <v>46241</v>
+      </c>
       <c r="D179" s="6"/>
       <c r="E179" s="6"/>
       <c r="F179" s="6"/>
@@ -9378,10 +10503,16 @@
       <c r="Y179" s="6"/>
       <c r="Z179" s="6"/>
     </row>
-    <row r="180" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A180" s="6"/>
-      <c r="B180" s="6"/>
-      <c r="C180" s="6"/>
+    <row r="180" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A180" s="11" t="s">
+        <v>410</v>
+      </c>
+      <c r="B180" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="C180" s="5">
+        <v>46242</v>
+      </c>
       <c r="D180" s="6"/>
       <c r="E180" s="6"/>
       <c r="F180" s="6"/>
@@ -9406,10 +10537,16 @@
       <c r="Y180" s="6"/>
       <c r="Z180" s="6"/>
     </row>
-    <row r="181" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A181" s="6"/>
-      <c r="B181" s="6"/>
-      <c r="C181" s="6"/>
+    <row r="181" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A181" s="11" t="s">
+        <v>411</v>
+      </c>
+      <c r="B181" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="C181" s="5">
+        <v>46243</v>
+      </c>
       <c r="D181" s="6"/>
       <c r="E181" s="6"/>
       <c r="F181" s="6"/>
@@ -9434,10 +10571,16 @@
       <c r="Y181" s="6"/>
       <c r="Z181" s="6"/>
     </row>
-    <row r="182" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A182" s="6"/>
-      <c r="B182" s="6"/>
-      <c r="C182" s="6"/>
+    <row r="182" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A182" s="11" t="s">
+        <v>412</v>
+      </c>
+      <c r="B182" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="C182" s="5">
+        <v>46244</v>
+      </c>
       <c r="D182" s="6"/>
       <c r="E182" s="6"/>
       <c r="F182" s="6"/>
@@ -9462,10 +10605,16 @@
       <c r="Y182" s="6"/>
       <c r="Z182" s="6"/>
     </row>
-    <row r="183" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A183" s="6"/>
-      <c r="B183" s="6"/>
-      <c r="C183" s="6"/>
+    <row r="183" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A183" s="11" t="s">
+        <v>413</v>
+      </c>
+      <c r="B183" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="C183" s="5">
+        <v>46245</v>
+      </c>
       <c r="D183" s="6"/>
       <c r="E183" s="6"/>
       <c r="F183" s="6"/>
@@ -9490,10 +10639,16 @@
       <c r="Y183" s="6"/>
       <c r="Z183" s="6"/>
     </row>
-    <row r="184" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A184" s="6"/>
-      <c r="B184" s="6"/>
-      <c r="C184" s="6"/>
+    <row r="184" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A184" s="11" t="s">
+        <v>414</v>
+      </c>
+      <c r="B184" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="C184" s="5">
+        <v>46246</v>
+      </c>
       <c r="D184" s="6"/>
       <c r="E184" s="6"/>
       <c r="F184" s="6"/>
@@ -9518,10 +10673,16 @@
       <c r="Y184" s="6"/>
       <c r="Z184" s="6"/>
     </row>
-    <row r="185" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A185" s="6"/>
-      <c r="B185" s="6"/>
-      <c r="C185" s="6"/>
+    <row r="185" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A185" s="11" t="s">
+        <v>415</v>
+      </c>
+      <c r="B185" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="C185" s="5">
+        <v>46247</v>
+      </c>
       <c r="D185" s="6"/>
       <c r="E185" s="6"/>
       <c r="F185" s="6"/>
@@ -9546,10 +10707,16 @@
       <c r="Y185" s="6"/>
       <c r="Z185" s="6"/>
     </row>
-    <row r="186" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A186" s="6"/>
-      <c r="B186" s="6"/>
-      <c r="C186" s="6"/>
+    <row r="186" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A186" s="11" t="s">
+        <v>416</v>
+      </c>
+      <c r="B186" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="C186" s="5">
+        <v>46248</v>
+      </c>
       <c r="D186" s="6"/>
       <c r="E186" s="6"/>
       <c r="F186" s="6"/>
@@ -9574,10 +10741,16 @@
       <c r="Y186" s="6"/>
       <c r="Z186" s="6"/>
     </row>
-    <row r="187" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A187" s="6"/>
-      <c r="B187" s="6"/>
-      <c r="C187" s="6"/>
+    <row r="187" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A187" s="11" t="s">
+        <v>417</v>
+      </c>
+      <c r="B187" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="C187" s="5">
+        <v>46249</v>
+      </c>
       <c r="D187" s="6"/>
       <c r="E187" s="6"/>
       <c r="F187" s="6"/>
@@ -9602,10 +10775,16 @@
       <c r="Y187" s="6"/>
       <c r="Z187" s="6"/>
     </row>
-    <row r="188" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A188" s="6"/>
-      <c r="B188" s="6"/>
-      <c r="C188" s="6"/>
+    <row r="188" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A188" s="11" t="s">
+        <v>418</v>
+      </c>
+      <c r="B188" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="C188" s="5">
+        <v>46250</v>
+      </c>
       <c r="D188" s="6"/>
       <c r="E188" s="6"/>
       <c r="F188" s="6"/>
@@ -9630,10 +10809,16 @@
       <c r="Y188" s="6"/>
       <c r="Z188" s="6"/>
     </row>
-    <row r="189" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A189" s="6"/>
-      <c r="B189" s="6"/>
-      <c r="C189" s="6"/>
+    <row r="189" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A189" s="11" t="s">
+        <v>419</v>
+      </c>
+      <c r="B189" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C189" s="5">
+        <v>46251</v>
+      </c>
       <c r="D189" s="6"/>
       <c r="E189" s="6"/>
       <c r="F189" s="6"/>
@@ -9658,10 +10843,16 @@
       <c r="Y189" s="6"/>
       <c r="Z189" s="6"/>
     </row>
-    <row r="190" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A190" s="6"/>
-      <c r="B190" s="6"/>
-      <c r="C190" s="6"/>
+    <row r="190" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A190" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="B190" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="C190" s="5">
+        <v>46252</v>
+      </c>
       <c r="D190" s="6"/>
       <c r="E190" s="6"/>
       <c r="F190" s="6"/>
@@ -9686,10 +10877,16 @@
       <c r="Y190" s="6"/>
       <c r="Z190" s="6"/>
     </row>
-    <row r="191" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A191" s="6"/>
-      <c r="B191" s="6"/>
-      <c r="C191" s="6"/>
+    <row r="191" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A191" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="B191" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="C191" s="5">
+        <v>46253</v>
+      </c>
       <c r="D191" s="6"/>
       <c r="E191" s="6"/>
       <c r="F191" s="6"/>
@@ -9714,10 +10911,16 @@
       <c r="Y191" s="6"/>
       <c r="Z191" s="6"/>
     </row>
-    <row r="192" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A192" s="6"/>
-      <c r="B192" s="6"/>
-      <c r="C192" s="6"/>
+    <row r="192" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A192" s="11" t="s">
+        <v>422</v>
+      </c>
+      <c r="B192" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="C192" s="5">
+        <v>46254</v>
+      </c>
       <c r="D192" s="6"/>
       <c r="E192" s="6"/>
       <c r="F192" s="6"/>
@@ -9742,10 +10945,16 @@
       <c r="Y192" s="6"/>
       <c r="Z192" s="6"/>
     </row>
-    <row r="193" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A193" s="6"/>
-      <c r="B193" s="6"/>
-      <c r="C193" s="6"/>
+    <row r="193" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A193" s="11" t="s">
+        <v>423</v>
+      </c>
+      <c r="B193" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="C193" s="5">
+        <v>46255</v>
+      </c>
       <c r="D193" s="6"/>
       <c r="E193" s="6"/>
       <c r="F193" s="6"/>
@@ -9770,10 +10979,16 @@
       <c r="Y193" s="6"/>
       <c r="Z193" s="6"/>
     </row>
-    <row r="194" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A194" s="6"/>
-      <c r="B194" s="6"/>
-      <c r="C194" s="6"/>
+    <row r="194" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A194" s="11" t="s">
+        <v>309</v>
+      </c>
+      <c r="B194" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="C194" s="5">
+        <v>46256</v>
+      </c>
       <c r="D194" s="6"/>
       <c r="E194" s="6"/>
       <c r="F194" s="6"/>
@@ -9798,10 +11013,16 @@
       <c r="Y194" s="6"/>
       <c r="Z194" s="6"/>
     </row>
-    <row r="195" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A195" s="6"/>
-      <c r="B195" s="6"/>
-      <c r="C195" s="6"/>
+    <row r="195" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A195" s="11" t="s">
+        <v>424</v>
+      </c>
+      <c r="B195" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="C195" s="5">
+        <v>46257</v>
+      </c>
       <c r="D195" s="6"/>
       <c r="E195" s="6"/>
       <c r="F195" s="6"/>
@@ -9826,10 +11047,16 @@
       <c r="Y195" s="6"/>
       <c r="Z195" s="6"/>
     </row>
-    <row r="196" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A196" s="6"/>
-      <c r="B196" s="6"/>
-      <c r="C196" s="6"/>
+    <row r="196" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A196" s="11" t="s">
+        <v>425</v>
+      </c>
+      <c r="B196" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="C196" s="5">
+        <v>46258</v>
+      </c>
       <c r="D196" s="6"/>
       <c r="E196" s="6"/>
       <c r="F196" s="6"/>
@@ -9854,10 +11081,16 @@
       <c r="Y196" s="6"/>
       <c r="Z196" s="6"/>
     </row>
-    <row r="197" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A197" s="6"/>
-      <c r="B197" s="6"/>
-      <c r="C197" s="6"/>
+    <row r="197" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A197" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="B197" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="C197" s="5">
+        <v>46259</v>
+      </c>
       <c r="D197" s="6"/>
       <c r="E197" s="6"/>
       <c r="F197" s="6"/>
@@ -9882,10 +11115,16 @@
       <c r="Y197" s="6"/>
       <c r="Z197" s="6"/>
     </row>
-    <row r="198" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A198" s="6"/>
-      <c r="B198" s="6"/>
-      <c r="C198" s="6"/>
+    <row r="198" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A198" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="B198" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="C198" s="5">
+        <v>46260</v>
+      </c>
       <c r="D198" s="6"/>
       <c r="E198" s="6"/>
       <c r="F198" s="6"/>
@@ -9910,10 +11149,16 @@
       <c r="Y198" s="6"/>
       <c r="Z198" s="6"/>
     </row>
-    <row r="199" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A199" s="6"/>
-      <c r="B199" s="6"/>
-      <c r="C199" s="6"/>
+    <row r="199" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A199" s="11" t="s">
+        <v>428</v>
+      </c>
+      <c r="B199" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="C199" s="5">
+        <v>46261</v>
+      </c>
       <c r="D199" s="6"/>
       <c r="E199" s="6"/>
       <c r="F199" s="6"/>
@@ -9938,10 +11183,16 @@
       <c r="Y199" s="6"/>
       <c r="Z199" s="6"/>
     </row>
-    <row r="200" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A200" s="6"/>
-      <c r="B200" s="6"/>
-      <c r="C200" s="6"/>
+    <row r="200" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A200" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="B200" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="C200" s="5">
+        <v>46262</v>
+      </c>
       <c r="D200" s="6"/>
       <c r="E200" s="6"/>
       <c r="F200" s="6"/>
@@ -9966,10 +11217,16 @@
       <c r="Y200" s="6"/>
       <c r="Z200" s="6"/>
     </row>
-    <row r="201" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A201" s="6"/>
-      <c r="B201" s="6"/>
-      <c r="C201" s="6"/>
+    <row r="201" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A201" s="11" t="s">
+        <v>430</v>
+      </c>
+      <c r="B201" s="6" t="s">
+        <v>379</v>
+      </c>
+      <c r="C201" s="5">
+        <v>46263</v>
+      </c>
       <c r="D201" s="6"/>
       <c r="E201" s="6"/>
       <c r="F201" s="6"/>
@@ -9994,10 +11251,16 @@
       <c r="Y201" s="6"/>
       <c r="Z201" s="6"/>
     </row>
-    <row r="202" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A202" s="6"/>
-      <c r="B202" s="6"/>
-      <c r="C202" s="6"/>
+    <row r="202" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A202" s="11" t="s">
+        <v>431</v>
+      </c>
+      <c r="B202" s="6" t="s">
+        <v>380</v>
+      </c>
+      <c r="C202" s="5">
+        <v>46264</v>
+      </c>
       <c r="D202" s="6"/>
       <c r="E202" s="6"/>
       <c r="F202" s="6"/>
@@ -10022,10 +11285,16 @@
       <c r="Y202" s="6"/>
       <c r="Z202" s="6"/>
     </row>
-    <row r="203" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A203" s="6"/>
-      <c r="B203" s="6"/>
-      <c r="C203" s="6"/>
+    <row r="203" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A203" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="B203" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="C203" s="5">
+        <v>46265</v>
+      </c>
       <c r="D203" s="6"/>
       <c r="E203" s="6"/>
       <c r="F203" s="6"/>
@@ -10050,10 +11319,16 @@
       <c r="Y203" s="6"/>
       <c r="Z203" s="6"/>
     </row>
-    <row r="204" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A204" s="6"/>
-      <c r="B204" s="6"/>
-      <c r="C204" s="6"/>
+    <row r="204" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A204" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="B204" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="C204" s="5">
+        <v>46266</v>
+      </c>
       <c r="D204" s="6"/>
       <c r="E204" s="6"/>
       <c r="F204" s="6"/>
@@ -10078,10 +11353,16 @@
       <c r="Y204" s="6"/>
       <c r="Z204" s="6"/>
     </row>
-    <row r="205" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A205" s="6"/>
-      <c r="B205" s="6"/>
-      <c r="C205" s="6"/>
+    <row r="205" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A205" s="11" t="s">
+        <v>434</v>
+      </c>
+      <c r="B205" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="C205" s="5">
+        <v>46267</v>
+      </c>
       <c r="D205" s="6"/>
       <c r="E205" s="6"/>
       <c r="F205" s="6"/>
@@ -10106,10 +11387,16 @@
       <c r="Y205" s="6"/>
       <c r="Z205" s="6"/>
     </row>
-    <row r="206" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A206" s="6"/>
-      <c r="B206" s="6"/>
-      <c r="C206" s="6"/>
+    <row r="206" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A206" s="11" t="s">
+        <v>435</v>
+      </c>
+      <c r="B206" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="C206" s="5">
+        <v>46268</v>
+      </c>
       <c r="D206" s="6"/>
       <c r="E206" s="6"/>
       <c r="F206" s="6"/>
@@ -10134,10 +11421,16 @@
       <c r="Y206" s="6"/>
       <c r="Z206" s="6"/>
     </row>
-    <row r="207" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A207" s="6"/>
-      <c r="B207" s="6"/>
-      <c r="C207" s="6"/>
+    <row r="207" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A207" s="11" t="s">
+        <v>413</v>
+      </c>
+      <c r="B207" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="C207" s="5">
+        <v>46269</v>
+      </c>
       <c r="D207" s="6"/>
       <c r="E207" s="6"/>
       <c r="F207" s="6"/>
@@ -10162,10 +11455,16 @@
       <c r="Y207" s="6"/>
       <c r="Z207" s="6"/>
     </row>
-    <row r="208" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A208" s="6"/>
-      <c r="B208" s="6"/>
-      <c r="C208" s="6"/>
+    <row r="208" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A208" s="11" t="s">
+        <v>436</v>
+      </c>
+      <c r="B208" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="C208" s="5">
+        <v>46270</v>
+      </c>
       <c r="D208" s="6"/>
       <c r="E208" s="6"/>
       <c r="F208" s="6"/>
@@ -10190,10 +11489,16 @@
       <c r="Y208" s="6"/>
       <c r="Z208" s="6"/>
     </row>
-    <row r="209" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A209" s="6"/>
-      <c r="B209" s="6"/>
-      <c r="C209" s="6"/>
+    <row r="209" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A209" s="11" t="s">
+        <v>437</v>
+      </c>
+      <c r="B209" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="C209" s="5">
+        <v>46271</v>
+      </c>
       <c r="D209" s="6"/>
       <c r="E209" s="6"/>
       <c r="F209" s="6"/>
@@ -10218,10 +11523,16 @@
       <c r="Y209" s="6"/>
       <c r="Z209" s="6"/>
     </row>
-    <row r="210" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A210" s="6"/>
-      <c r="B210" s="6"/>
-      <c r="C210" s="6"/>
+    <row r="210" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A210" s="11" t="s">
+        <v>438</v>
+      </c>
+      <c r="B210" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="C210" s="5">
+        <v>46272</v>
+      </c>
       <c r="D210" s="6"/>
       <c r="E210" s="6"/>
       <c r="F210" s="6"/>
@@ -10246,10 +11557,16 @@
       <c r="Y210" s="6"/>
       <c r="Z210" s="6"/>
     </row>
-    <row r="211" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A211" s="6"/>
-      <c r="B211" s="6"/>
-      <c r="C211" s="6"/>
+    <row r="211" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A211" s="11" t="s">
+        <v>439</v>
+      </c>
+      <c r="B211" s="6" t="s">
+        <v>389</v>
+      </c>
+      <c r="C211" s="5">
+        <v>46273</v>
+      </c>
       <c r="D211" s="6"/>
       <c r="E211" s="6"/>
       <c r="F211" s="6"/>
@@ -10274,10 +11591,16 @@
       <c r="Y211" s="6"/>
       <c r="Z211" s="6"/>
     </row>
-    <row r="212" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A212" s="6"/>
-      <c r="B212" s="6"/>
-      <c r="C212" s="6"/>
+    <row r="212" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A212" s="11" t="s">
+        <v>440</v>
+      </c>
+      <c r="B212" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="C212" s="5">
+        <v>46274</v>
+      </c>
       <c r="D212" s="6"/>
       <c r="E212" s="6"/>
       <c r="F212" s="6"/>
@@ -10302,10 +11625,16 @@
       <c r="Y212" s="6"/>
       <c r="Z212" s="6"/>
     </row>
-    <row r="213" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A213" s="6"/>
-      <c r="B213" s="6"/>
-      <c r="C213" s="6"/>
+    <row r="213" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A213" s="11" t="s">
+        <v>441</v>
+      </c>
+      <c r="B213" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="C213" s="5">
+        <v>46275</v>
+      </c>
       <c r="D213" s="6"/>
       <c r="E213" s="6"/>
       <c r="F213" s="6"/>
@@ -10330,10 +11659,16 @@
       <c r="Y213" s="6"/>
       <c r="Z213" s="6"/>
     </row>
-    <row r="214" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A214" s="6"/>
-      <c r="B214" s="6"/>
-      <c r="C214" s="6"/>
+    <row r="214" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A214" s="11" t="s">
+        <v>442</v>
+      </c>
+      <c r="B214" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="C214" s="5">
+        <v>46276</v>
+      </c>
       <c r="D214" s="6"/>
       <c r="E214" s="6"/>
       <c r="F214" s="6"/>
@@ -10358,10 +11693,16 @@
       <c r="Y214" s="6"/>
       <c r="Z214" s="6"/>
     </row>
-    <row r="215" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A215" s="6"/>
-      <c r="B215" s="6"/>
-      <c r="C215" s="6"/>
+    <row r="215" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A215" s="11" t="s">
+        <v>443</v>
+      </c>
+      <c r="B215" s="6" t="s">
+        <v>393</v>
+      </c>
+      <c r="C215" s="5">
+        <v>46277</v>
+      </c>
       <c r="D215" s="6"/>
       <c r="E215" s="6"/>
       <c r="F215" s="6"/>
@@ -10386,10 +11727,16 @@
       <c r="Y215" s="6"/>
       <c r="Z215" s="6"/>
     </row>
-    <row r="216" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A216" s="6"/>
-      <c r="B216" s="6"/>
-      <c r="C216" s="6"/>
+    <row r="216" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A216" s="11" t="s">
+        <v>444</v>
+      </c>
+      <c r="B216" s="6" t="s">
+        <v>394</v>
+      </c>
+      <c r="C216" s="5">
+        <v>46278</v>
+      </c>
       <c r="D216" s="6"/>
       <c r="E216" s="6"/>
       <c r="F216" s="6"/>
@@ -10414,10 +11761,16 @@
       <c r="Y216" s="6"/>
       <c r="Z216" s="6"/>
     </row>
-    <row r="217" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A217" s="6"/>
-      <c r="B217" s="6"/>
-      <c r="C217" s="6"/>
+    <row r="217" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A217" s="11" t="s">
+        <v>445</v>
+      </c>
+      <c r="B217" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="C217" s="5">
+        <v>46279</v>
+      </c>
       <c r="D217" s="6"/>
       <c r="E217" s="6"/>
       <c r="F217" s="6"/>
@@ -10442,10 +11795,16 @@
       <c r="Y217" s="6"/>
       <c r="Z217" s="6"/>
     </row>
-    <row r="218" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A218" s="6"/>
-      <c r="B218" s="6"/>
-      <c r="C218" s="6"/>
+    <row r="218" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A218" s="11" t="s">
+        <v>446</v>
+      </c>
+      <c r="B218" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="C218" s="5">
+        <v>46280</v>
+      </c>
       <c r="D218" s="6"/>
       <c r="E218" s="6"/>
       <c r="F218" s="6"/>
@@ -10470,10 +11829,16 @@
       <c r="Y218" s="6"/>
       <c r="Z218" s="6"/>
     </row>
-    <row r="219" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A219" s="6"/>
-      <c r="B219" s="6"/>
-      <c r="C219" s="6"/>
+    <row r="219" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A219" s="11" t="s">
+        <v>447</v>
+      </c>
+      <c r="B219" s="6" t="s">
+        <v>397</v>
+      </c>
+      <c r="C219" s="5">
+        <v>46281</v>
+      </c>
       <c r="D219" s="6"/>
       <c r="E219" s="6"/>
       <c r="F219" s="6"/>
@@ -10498,10 +11863,16 @@
       <c r="Y219" s="6"/>
       <c r="Z219" s="6"/>
     </row>
-    <row r="220" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A220" s="6"/>
-      <c r="B220" s="6"/>
-      <c r="C220" s="6"/>
+    <row r="220" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A220" s="11" t="s">
+        <v>448</v>
+      </c>
+      <c r="B220" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="C220" s="5">
+        <v>46282</v>
+      </c>
       <c r="D220" s="6"/>
       <c r="E220" s="6"/>
       <c r="F220" s="6"/>
@@ -10526,10 +11897,16 @@
       <c r="Y220" s="6"/>
       <c r="Z220" s="6"/>
     </row>
-    <row r="221" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A221" s="6"/>
-      <c r="B221" s="6"/>
-      <c r="C221" s="6"/>
+    <row r="221" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A221" s="11" t="s">
+        <v>449</v>
+      </c>
+      <c r="B221" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="C221" s="5">
+        <v>46283</v>
+      </c>
       <c r="D221" s="6"/>
       <c r="E221" s="6"/>
       <c r="F221" s="6"/>
@@ -10554,10 +11931,16 @@
       <c r="Y221" s="6"/>
       <c r="Z221" s="6"/>
     </row>
-    <row r="222" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A222" s="6"/>
-      <c r="B222" s="6"/>
-      <c r="C222" s="6"/>
+    <row r="222" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A222" s="11" t="s">
+        <v>450</v>
+      </c>
+      <c r="B222" s="6" t="s">
+        <v>400</v>
+      </c>
+      <c r="C222" s="5">
+        <v>46284</v>
+      </c>
       <c r="D222" s="6"/>
       <c r="E222" s="6"/>
       <c r="F222" s="6"/>
@@ -10582,10 +11965,16 @@
       <c r="Y222" s="6"/>
       <c r="Z222" s="6"/>
     </row>
-    <row r="223" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A223" s="6"/>
-      <c r="B223" s="6"/>
-      <c r="C223" s="6"/>
+    <row r="223" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A223" s="11" t="s">
+        <v>451</v>
+      </c>
+      <c r="B223" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="C223" s="5">
+        <v>46285</v>
+      </c>
       <c r="D223" s="6"/>
       <c r="E223" s="6"/>
       <c r="F223" s="6"/>
@@ -10610,10 +11999,16 @@
       <c r="Y223" s="6"/>
       <c r="Z223" s="6"/>
     </row>
-    <row r="224" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A224" s="6"/>
-      <c r="B224" s="6"/>
-      <c r="C224" s="6"/>
+    <row r="224" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A224" s="11" t="s">
+        <v>452</v>
+      </c>
+      <c r="B224" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="C224" s="5">
+        <v>46286</v>
+      </c>
       <c r="D224" s="6"/>
       <c r="E224" s="6"/>
       <c r="F224" s="6"/>
@@ -10638,10 +12033,16 @@
       <c r="Y224" s="6"/>
       <c r="Z224" s="6"/>
     </row>
-    <row r="225" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A225" s="6"/>
-      <c r="B225" s="6"/>
-      <c r="C225" s="6"/>
+    <row r="225" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A225" s="11" t="s">
+        <v>453</v>
+      </c>
+      <c r="B225" s="6" t="s">
+        <v>403</v>
+      </c>
+      <c r="C225" s="5">
+        <v>46287</v>
+      </c>
       <c r="D225" s="6"/>
       <c r="E225" s="6"/>
       <c r="F225" s="6"/>
@@ -10666,10 +12067,16 @@
       <c r="Y225" s="6"/>
       <c r="Z225" s="6"/>
     </row>
-    <row r="226" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A226" s="6"/>
-      <c r="B226" s="6"/>
-      <c r="C226" s="6"/>
+    <row r="226" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A226" s="11" t="s">
+        <v>454</v>
+      </c>
+      <c r="B226" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="C226" s="5">
+        <v>46288</v>
+      </c>
       <c r="D226" s="6"/>
       <c r="E226" s="6"/>
       <c r="F226" s="6"/>
@@ -10694,10 +12101,16 @@
       <c r="Y226" s="6"/>
       <c r="Z226" s="6"/>
     </row>
-    <row r="227" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A227" s="6"/>
-      <c r="B227" s="6"/>
-      <c r="C227" s="6"/>
+    <row r="227" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A227" s="11" t="s">
+        <v>455</v>
+      </c>
+      <c r="B227" s="6" t="s">
+        <v>405</v>
+      </c>
+      <c r="C227" s="5">
+        <v>46289</v>
+      </c>
       <c r="D227" s="6"/>
       <c r="E227" s="6"/>
       <c r="F227" s="6"/>
@@ -10722,10 +12135,16 @@
       <c r="Y227" s="6"/>
       <c r="Z227" s="6"/>
     </row>
-    <row r="228" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A228" s="6"/>
-      <c r="B228" s="6"/>
-      <c r="C228" s="6"/>
+    <row r="228" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A228" s="11" t="s">
+        <v>456</v>
+      </c>
+      <c r="B228" s="6" t="s">
+        <v>406</v>
+      </c>
+      <c r="C228" s="5">
+        <v>46290</v>
+      </c>
       <c r="D228" s="6"/>
       <c r="E228" s="6"/>
       <c r="F228" s="6"/>
@@ -10750,10 +12169,16 @@
       <c r="Y228" s="6"/>
       <c r="Z228" s="6"/>
     </row>
-    <row r="229" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A229" s="6"/>
-      <c r="B229" s="6"/>
-      <c r="C229" s="6"/>
+    <row r="229" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A229" s="11" t="s">
+        <v>457</v>
+      </c>
+      <c r="B229" s="6" t="s">
+        <v>466</v>
+      </c>
+      <c r="C229" s="5">
+        <v>46291</v>
+      </c>
       <c r="D229" s="6"/>
       <c r="E229" s="6"/>
       <c r="F229" s="6"/>
@@ -10778,10 +12203,16 @@
       <c r="Y229" s="6"/>
       <c r="Z229" s="6"/>
     </row>
-    <row r="230" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A230" s="6"/>
-      <c r="B230" s="6"/>
-      <c r="C230" s="6"/>
+    <row r="230" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A230" s="11" t="s">
+        <v>458</v>
+      </c>
+      <c r="B230" s="6" t="s">
+        <v>467</v>
+      </c>
+      <c r="C230" s="5">
+        <v>46292</v>
+      </c>
       <c r="D230" s="6"/>
       <c r="E230" s="6"/>
       <c r="F230" s="6"/>
@@ -10806,10 +12237,16 @@
       <c r="Y230" s="6"/>
       <c r="Z230" s="6"/>
     </row>
-    <row r="231" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A231" s="6"/>
-      <c r="B231" s="6"/>
-      <c r="C231" s="6"/>
+    <row r="231" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A231" s="11" t="s">
+        <v>459</v>
+      </c>
+      <c r="B231" s="6" t="s">
+        <v>468</v>
+      </c>
+      <c r="C231" s="5">
+        <v>46293</v>
+      </c>
       <c r="D231" s="6"/>
       <c r="E231" s="6"/>
       <c r="F231" s="6"/>
@@ -10834,10 +12271,16 @@
       <c r="Y231" s="6"/>
       <c r="Z231" s="6"/>
     </row>
-    <row r="232" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A232" s="6"/>
-      <c r="B232" s="6"/>
-      <c r="C232" s="6"/>
+    <row r="232" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A232" s="11" t="s">
+        <v>460</v>
+      </c>
+      <c r="B232" s="6" t="s">
+        <v>469</v>
+      </c>
+      <c r="C232" s="5">
+        <v>46294</v>
+      </c>
       <c r="D232" s="6"/>
       <c r="E232" s="6"/>
       <c r="F232" s="6"/>
@@ -10862,10 +12305,16 @@
       <c r="Y232" s="6"/>
       <c r="Z232" s="6"/>
     </row>
-    <row r="233" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A233" s="6"/>
-      <c r="B233" s="6"/>
-      <c r="C233" s="6"/>
+    <row r="233" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A233" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="B233" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="C233" s="5">
+        <v>46295</v>
+      </c>
       <c r="D233" s="6"/>
       <c r="E233" s="6"/>
       <c r="F233" s="6"/>
@@ -10890,10 +12339,16 @@
       <c r="Y233" s="6"/>
       <c r="Z233" s="6"/>
     </row>
-    <row r="234" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A234" s="6"/>
-      <c r="B234" s="6"/>
-      <c r="C234" s="6"/>
+    <row r="234" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A234" s="11" t="s">
+        <v>461</v>
+      </c>
+      <c r="B234" s="6" t="s">
+        <v>471</v>
+      </c>
+      <c r="C234" s="5">
+        <v>46296</v>
+      </c>
       <c r="D234" s="6"/>
       <c r="E234" s="6"/>
       <c r="F234" s="6"/>
@@ -10918,10 +12373,16 @@
       <c r="Y234" s="6"/>
       <c r="Z234" s="6"/>
     </row>
-    <row r="235" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A235" s="6"/>
-      <c r="B235" s="6"/>
-      <c r="C235" s="6"/>
+    <row r="235" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A235" s="11" t="s">
+        <v>462</v>
+      </c>
+      <c r="B235" s="6" t="s">
+        <v>472</v>
+      </c>
+      <c r="C235" s="5">
+        <v>46297</v>
+      </c>
       <c r="D235" s="6"/>
       <c r="E235" s="6"/>
       <c r="F235" s="6"/>
@@ -10946,10 +12407,16 @@
       <c r="Y235" s="6"/>
       <c r="Z235" s="6"/>
     </row>
-    <row r="236" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A236" s="6"/>
-      <c r="B236" s="6"/>
-      <c r="C236" s="6"/>
+    <row r="236" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A236" s="11" t="s">
+        <v>463</v>
+      </c>
+      <c r="B236" s="6" t="s">
+        <v>473</v>
+      </c>
+      <c r="C236" s="5">
+        <v>46298</v>
+      </c>
       <c r="D236" s="6"/>
       <c r="E236" s="6"/>
       <c r="F236" s="6"/>
@@ -10974,10 +12441,16 @@
       <c r="Y236" s="6"/>
       <c r="Z236" s="6"/>
     </row>
-    <row r="237" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A237" s="6"/>
-      <c r="B237" s="6"/>
-      <c r="C237" s="6"/>
+    <row r="237" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A237" s="11" t="s">
+        <v>464</v>
+      </c>
+      <c r="B237" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="C237" s="5">
+        <v>46299</v>
+      </c>
       <c r="D237" s="6"/>
       <c r="E237" s="6"/>
       <c r="F237" s="6"/>
@@ -11002,10 +12475,16 @@
       <c r="Y237" s="6"/>
       <c r="Z237" s="6"/>
     </row>
-    <row r="238" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A238" s="6"/>
-      <c r="B238" s="6"/>
-      <c r="C238" s="6"/>
+    <row r="238" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A238" s="11" t="s">
+        <v>465</v>
+      </c>
+      <c r="B238" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="C238" s="5">
+        <v>46300</v>
+      </c>
       <c r="D238" s="6"/>
       <c r="E238" s="6"/>
       <c r="F238" s="6"/>
@@ -31060,9 +32539,71 @@
     <hyperlink ref="A174" r:id="rId173" xr:uid="{06F09D2A-4425-4C50-85DB-F62375E004D0}"/>
     <hyperlink ref="A175" r:id="rId174" xr:uid="{F8A19440-A55E-4E98-BEDC-39E42358315C}"/>
     <hyperlink ref="A176" r:id="rId175" xr:uid="{FDA1E3AC-3D0F-4790-A831-6278D352C318}"/>
+    <hyperlink ref="A177" r:id="rId176" display="https://www.youtube.com/watch?v=IEZVq01Q7go&amp;t=14s" xr:uid="{6E2E46C9-5A93-4FEC-83F8-FA862ED3F394}"/>
+    <hyperlink ref="A178" r:id="rId177" display="https://www.youtube.com/watch?v=jiFJXvMc2SY&amp;t=321s" xr:uid="{AF547EB6-0570-4CCB-8C4A-506C59C63EB2}"/>
+    <hyperlink ref="A179" r:id="rId178" display="https://www.youtube.com/watch?v=fr6B3EtlZVM&amp;t=3s" xr:uid="{80501AC0-2505-454C-86BD-FC8CC562B3EF}"/>
+    <hyperlink ref="A180" r:id="rId179" display="https://www.youtube.com/watch?v=PBNhMcRKu24&amp;t=1s" xr:uid="{31F702F7-E8DF-42BC-B03E-3A37CC8E8D21}"/>
+    <hyperlink ref="A181" r:id="rId180" display="https://www.youtube.com/watch?v=ZHFNRrT8WA4&amp;t=3s" xr:uid="{A716B794-C0BC-4B0F-A077-3E84C8B29FE9}"/>
+    <hyperlink ref="A182" r:id="rId181" display="https://www.youtube.com/watch?v=mXLQFJ-W7xc&amp;t=23s" xr:uid="{ECD8F234-D871-4C12-948F-B179A63113BE}"/>
+    <hyperlink ref="A183" r:id="rId182" display="https://www.youtube.com/watch?v=gN9bQHaOKg8&amp;t=96s" xr:uid="{9C782EFC-44A8-4A9E-AD7C-B5325020CDC6}"/>
+    <hyperlink ref="A184" r:id="rId183" display="https://www.youtube.com/watch?v=BXylPudUUek&amp;t=13s" xr:uid="{E88C8B2C-49FB-46B0-BF60-DD1F4190D19F}"/>
+    <hyperlink ref="A185" r:id="rId184" display="https://www.youtube.com/watch?v=tbluAPW3aLs&amp;t=3s" xr:uid="{0084ADE7-C7E7-4B65-AE2F-86D28F496E0E}"/>
+    <hyperlink ref="A186" r:id="rId185" xr:uid="{35406A36-FEF6-4FDB-B8A6-3326A895E21F}"/>
+    <hyperlink ref="A187" r:id="rId186" xr:uid="{CE3CF289-745E-41E3-9691-9BAB4F8813FA}"/>
+    <hyperlink ref="A188" r:id="rId187" xr:uid="{A7C8FFD5-FBFD-43D6-ABE1-BBDE0CD644DC}"/>
+    <hyperlink ref="A189" r:id="rId188" xr:uid="{DBE7879E-87E5-4598-B430-DC72C82B1B19}"/>
+    <hyperlink ref="A190" r:id="rId189" xr:uid="{2E6C0C5C-6EDD-4884-AA19-96F63E3D51D8}"/>
+    <hyperlink ref="A191" r:id="rId190" xr:uid="{DCECAB24-2242-47E3-888C-F0C3C8250435}"/>
+    <hyperlink ref="A192" r:id="rId191" xr:uid="{4DE76AA1-BF64-4307-A6AA-EFA588762F5D}"/>
+    <hyperlink ref="A193" r:id="rId192" xr:uid="{17496152-ABF8-43B9-B256-BE990524C716}"/>
+    <hyperlink ref="A194" r:id="rId193" display="https://www.youtube.com/watch?v=i8v5Fb_aDW8&amp;t=351s" xr:uid="{332CC6B2-CE6B-4C93-97C3-44A94E2D24A5}"/>
+    <hyperlink ref="A195" r:id="rId194" display="https://www.youtube.com/watch?v=8e4gw8yeQIo&amp;t=109s" xr:uid="{8480EBE9-7FFB-4EF5-88E2-ABE2CF7440A7}"/>
+    <hyperlink ref="A196" r:id="rId195" xr:uid="{A5B15A64-A51B-40E6-9ACF-134376194723}"/>
+    <hyperlink ref="A197" r:id="rId196" xr:uid="{A48D676D-A605-4338-96BD-0AC6D5A9E382}"/>
+    <hyperlink ref="A198" r:id="rId197" xr:uid="{569A539E-AD38-4703-AB22-F61803D30CF2}"/>
+    <hyperlink ref="A199" r:id="rId198" display="https://www.youtube.com/watch?v=tBIG11CRXmM&amp;t=14s" xr:uid="{2F471218-82DF-40CF-B015-C4B2875C41E5}"/>
+    <hyperlink ref="A200" r:id="rId199" display="https://www.youtube.com/watch?v=S-ZrxzifoQ0&amp;t=3s" xr:uid="{701DB842-0F58-472A-9C5E-A01CEF4C0A8C}"/>
+    <hyperlink ref="A201" r:id="rId200" display="https://www.youtube.com/watch?v=8anpFagF9VU&amp;t=23s" xr:uid="{071F122F-7A1B-4BBF-A654-58C3AFD89DF9}"/>
+    <hyperlink ref="A202" r:id="rId201" display="https://www.youtube.com/watch?v=cx2wkrKymok&amp;t=221s" xr:uid="{A5101831-6B0E-4AB2-8A33-61B5CABC0D62}"/>
+    <hyperlink ref="A203" r:id="rId202" xr:uid="{BD0EF7C4-7884-458B-85A2-224EAE2DB3F7}"/>
+    <hyperlink ref="A204" r:id="rId203" xr:uid="{2B59D218-FF4D-481E-A174-5EE4C40704B5}"/>
+    <hyperlink ref="A205" r:id="rId204" xr:uid="{54FB46A7-493B-45BB-8286-121F86406EC6}"/>
+    <hyperlink ref="A206" r:id="rId205" xr:uid="{6B545943-CE0C-4030-A330-E3FD83BCFAB1}"/>
+    <hyperlink ref="A207" r:id="rId206" xr:uid="{A7C2EA8C-213D-45AA-B60B-8CF4ABBF4422}"/>
+    <hyperlink ref="A208" r:id="rId207" xr:uid="{A6B8B852-0068-4D49-90E7-B07869CB6C27}"/>
+    <hyperlink ref="A209" r:id="rId208" display="https://www.youtube.com/watch?v=5RbaPlzKbFk&amp;t=6s" xr:uid="{251826EC-5AA2-40C1-97DB-BF1F6A00C627}"/>
+    <hyperlink ref="A210" r:id="rId209" xr:uid="{25020D0E-7831-4DCC-98C0-7D15D8B3C0C5}"/>
+    <hyperlink ref="A211" r:id="rId210" xr:uid="{3AE2A21A-B8FF-4E8E-BECB-6E3E425164B3}"/>
+    <hyperlink ref="A212" r:id="rId211" xr:uid="{544959B0-0B1F-4C15-9755-0E24A91C037B}"/>
+    <hyperlink ref="A213" r:id="rId212" xr:uid="{70B2D394-120F-492A-A71A-B06A09F93695}"/>
+    <hyperlink ref="A214" r:id="rId213" xr:uid="{E76CC7CB-8875-49C8-9AC4-56339180A13D}"/>
+    <hyperlink ref="A215" r:id="rId214" xr:uid="{B67602ED-599F-41DF-AAFF-A261F7A2628F}"/>
+    <hyperlink ref="A216" r:id="rId215" display="https://www.youtube.com/watch?v=vcnndeYVw9k&amp;t=4s" xr:uid="{924F2667-71CD-4B18-8F38-74728A6EDAD4}"/>
+    <hyperlink ref="A217" r:id="rId216" display="https://www.youtube.com/watch?v=Y1zBcg4QJgE&amp;t=8s" xr:uid="{952A5D9D-520E-47C0-AFF4-8512A9BE29E8}"/>
+    <hyperlink ref="A218" r:id="rId217" display="https://www.youtube.com/watch?v=1Ilgi75Y6Ac&amp;t=9s" xr:uid="{72C682B9-B076-49EB-A29C-9BB45054A7EA}"/>
+    <hyperlink ref="A219" r:id="rId218" xr:uid="{7F41CE59-AE00-40C9-BE6A-F18C335C3A0E}"/>
+    <hyperlink ref="A220" r:id="rId219" xr:uid="{CF321F14-C269-42A4-91C0-840F4C823C70}"/>
+    <hyperlink ref="A221" r:id="rId220" xr:uid="{A7E7CAF7-A997-4B12-90E1-26A93C1B1072}"/>
+    <hyperlink ref="A222" r:id="rId221" display="https://www.youtube.com/watch?v=zgLWXkOMOGE&amp;t=20s" xr:uid="{03889847-6FB9-4050-ACC7-E8FB0BEC97AF}"/>
+    <hyperlink ref="A223" r:id="rId222" display="https://www.youtube.com/watch?v=r-DPvpwMOdw&amp;t=144s" xr:uid="{092B3088-44A7-4CE4-BA66-7B47B148A1A0}"/>
+    <hyperlink ref="A224" r:id="rId223" xr:uid="{0136ABBE-D936-4875-B2D1-CFC31CF17809}"/>
+    <hyperlink ref="A225" r:id="rId224" xr:uid="{30C16BD5-C9D0-4EB1-9CA8-75AFA5411020}"/>
+    <hyperlink ref="A226" r:id="rId225" xr:uid="{C72C881F-CF23-4064-91DB-74DEE8981619}"/>
+    <hyperlink ref="A227" r:id="rId226" xr:uid="{A80B5652-DD44-4448-9AD7-475B83CD2CC5}"/>
+    <hyperlink ref="A228" r:id="rId227" display="https://www.youtube.com/watch?v=X6XNEMBmPrk&amp;t=149s" xr:uid="{EE260E8B-DAF8-4D9E-BE02-F58B89498785}"/>
+    <hyperlink ref="A229" r:id="rId228" xr:uid="{BB71C43A-EDC5-4361-9D22-EC8718BF072A}"/>
+    <hyperlink ref="A230" r:id="rId229" xr:uid="{732C0A5B-9BB4-415F-8AD8-C7C3F6202BA7}"/>
+    <hyperlink ref="A231" r:id="rId230" display="https://www.youtube.com/watch?v=qCOWcKURVzk&amp;t=1s" xr:uid="{A77C1056-BFED-4056-8D1D-003D38800C08}"/>
+    <hyperlink ref="A232" r:id="rId231" xr:uid="{9A7F76BD-8F39-45AC-9B67-1AB2C5A163C5}"/>
+    <hyperlink ref="A233" r:id="rId232" display="https://www.youtube.com/watch?v=-NHHdVWUcwo&amp;t=3s" xr:uid="{5ABBA3E2-3DB1-4043-84CB-5FA2E85A7167}"/>
+    <hyperlink ref="A234" r:id="rId233" display="https://www.youtube.com/watch?v=IS1Fcnh-W-M&amp;t=9s" xr:uid="{017A6139-68A6-4430-B3D6-B1E4D82AE209}"/>
+    <hyperlink ref="A235" r:id="rId234" display="https://www.youtube.com/watch?v=Rssbr11AO1o&amp;t=1s" xr:uid="{C56A432D-4EDF-46AE-B5AA-D2144300E7A0}"/>
+    <hyperlink ref="A236" r:id="rId235" display="https://www.youtube.com/watch?v=7rdJOSgHgg4&amp;t=559s" xr:uid="{01909B77-657A-491C-B14B-54B0CAC58311}"/>
+    <hyperlink ref="A237" r:id="rId236" xr:uid="{5A1B9525-3FD4-4576-B6C2-C275598276F5}"/>
+    <hyperlink ref="A238" r:id="rId237" display="https://www.youtube.com/watch?v=tS58CDMrFxA&amp;t=23s" xr:uid="{8BDBC4D2-1AEC-4538-A0AB-264071C82E94}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId176"/>
+  <pageSetup orientation="portrait" r:id="rId238"/>
 </worksheet>
 </file>
 
@@ -35806,10 +37347,16 @@
       <c r="Y139" s="6"/>
       <c r="Z139" s="6"/>
     </row>
-    <row r="140" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A140" s="6"/>
-      <c r="B140" s="6"/>
-      <c r="C140" s="8"/>
+    <row r="140" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A140" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="B140" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="C140" s="7">
+        <v>46239</v>
+      </c>
       <c r="D140" s="6"/>
       <c r="E140" s="6"/>
       <c r="F140" s="6"/>
@@ -35834,10 +37381,16 @@
       <c r="Y140" s="6"/>
       <c r="Z140" s="6"/>
     </row>
-    <row r="141" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A141" s="6"/>
-      <c r="B141" s="6"/>
-      <c r="C141" s="8"/>
+    <row r="141" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A141" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="B141" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="C141" s="7">
+        <v>46240</v>
+      </c>
       <c r="D141" s="6"/>
       <c r="E141" s="6"/>
       <c r="F141" s="6"/>
@@ -35862,10 +37415,16 @@
       <c r="Y141" s="6"/>
       <c r="Z141" s="6"/>
     </row>
-    <row r="142" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A142" s="6"/>
-      <c r="B142" s="6"/>
-      <c r="C142" s="8"/>
+    <row r="142" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A142" s="11" t="s">
+        <v>409</v>
+      </c>
+      <c r="B142" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="C142" s="7">
+        <v>46241</v>
+      </c>
       <c r="D142" s="6"/>
       <c r="E142" s="6"/>
       <c r="F142" s="6"/>
@@ -35890,10 +37449,16 @@
       <c r="Y142" s="6"/>
       <c r="Z142" s="6"/>
     </row>
-    <row r="143" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A143" s="6"/>
-      <c r="B143" s="6"/>
-      <c r="C143" s="8"/>
+    <row r="143" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A143" s="11" t="s">
+        <v>410</v>
+      </c>
+      <c r="B143" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="C143" s="7">
+        <v>46242</v>
+      </c>
       <c r="D143" s="6"/>
       <c r="E143" s="6"/>
       <c r="F143" s="6"/>
@@ -35918,10 +37483,16 @@
       <c r="Y143" s="6"/>
       <c r="Z143" s="6"/>
     </row>
-    <row r="144" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A144" s="6"/>
-      <c r="B144" s="6"/>
-      <c r="C144" s="8"/>
+    <row r="144" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A144" s="11" t="s">
+        <v>411</v>
+      </c>
+      <c r="B144" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="C144" s="7">
+        <v>46243</v>
+      </c>
       <c r="D144" s="6"/>
       <c r="E144" s="6"/>
       <c r="F144" s="6"/>
@@ -35946,10 +37517,16 @@
       <c r="Y144" s="6"/>
       <c r="Z144" s="6"/>
     </row>
-    <row r="145" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A145" s="6"/>
-      <c r="B145" s="6"/>
-      <c r="C145" s="8"/>
+    <row r="145" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A145" s="11" t="s">
+        <v>412</v>
+      </c>
+      <c r="B145" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="C145" s="7">
+        <v>46244</v>
+      </c>
       <c r="D145" s="6"/>
       <c r="E145" s="6"/>
       <c r="F145" s="6"/>
@@ -35974,10 +37551,16 @@
       <c r="Y145" s="6"/>
       <c r="Z145" s="6"/>
     </row>
-    <row r="146" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A146" s="6"/>
-      <c r="B146" s="6"/>
-      <c r="C146" s="8"/>
+    <row r="146" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A146" s="11" t="s">
+        <v>413</v>
+      </c>
+      <c r="B146" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="C146" s="7">
+        <v>46245</v>
+      </c>
       <c r="D146" s="6"/>
       <c r="E146" s="6"/>
       <c r="F146" s="6"/>
@@ -36002,10 +37585,16 @@
       <c r="Y146" s="6"/>
       <c r="Z146" s="6"/>
     </row>
-    <row r="147" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A147" s="6"/>
-      <c r="B147" s="6"/>
-      <c r="C147" s="8"/>
+    <row r="147" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A147" s="11" t="s">
+        <v>414</v>
+      </c>
+      <c r="B147" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="C147" s="7">
+        <v>46246</v>
+      </c>
       <c r="D147" s="6"/>
       <c r="E147" s="6"/>
       <c r="F147" s="6"/>
@@ -36030,10 +37619,16 @@
       <c r="Y147" s="6"/>
       <c r="Z147" s="6"/>
     </row>
-    <row r="148" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A148" s="6"/>
-      <c r="B148" s="6"/>
-      <c r="C148" s="8"/>
+    <row r="148" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A148" s="11" t="s">
+        <v>415</v>
+      </c>
+      <c r="B148" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="C148" s="7">
+        <v>46247</v>
+      </c>
       <c r="D148" s="6"/>
       <c r="E148" s="6"/>
       <c r="F148" s="6"/>
@@ -36058,10 +37653,16 @@
       <c r="Y148" s="6"/>
       <c r="Z148" s="6"/>
     </row>
-    <row r="149" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A149" s="6"/>
-      <c r="B149" s="6"/>
-      <c r="C149" s="8"/>
+    <row r="149" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A149" s="11" t="s">
+        <v>416</v>
+      </c>
+      <c r="B149" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="C149" s="7">
+        <v>46248</v>
+      </c>
       <c r="D149" s="6"/>
       <c r="E149" s="6"/>
       <c r="F149" s="6"/>
@@ -36086,10 +37687,16 @@
       <c r="Y149" s="6"/>
       <c r="Z149" s="6"/>
     </row>
-    <row r="150" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A150" s="6"/>
-      <c r="B150" s="6"/>
-      <c r="C150" s="8"/>
+    <row r="150" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A150" s="11" t="s">
+        <v>417</v>
+      </c>
+      <c r="B150" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="C150" s="7">
+        <v>46249</v>
+      </c>
       <c r="D150" s="6"/>
       <c r="E150" s="6"/>
       <c r="F150" s="6"/>
@@ -36114,10 +37721,16 @@
       <c r="Y150" s="6"/>
       <c r="Z150" s="6"/>
     </row>
-    <row r="151" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A151" s="6"/>
-      <c r="B151" s="6"/>
-      <c r="C151" s="8"/>
+    <row r="151" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A151" s="11" t="s">
+        <v>418</v>
+      </c>
+      <c r="B151" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="C151" s="7">
+        <v>46250</v>
+      </c>
       <c r="D151" s="6"/>
       <c r="E151" s="6"/>
       <c r="F151" s="6"/>
@@ -36142,10 +37755,16 @@
       <c r="Y151" s="6"/>
       <c r="Z151" s="6"/>
     </row>
-    <row r="152" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A152" s="6"/>
-      <c r="B152" s="6"/>
-      <c r="C152" s="8"/>
+    <row r="152" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A152" s="11" t="s">
+        <v>419</v>
+      </c>
+      <c r="B152" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="C152" s="7">
+        <v>46251</v>
+      </c>
       <c r="D152" s="6"/>
       <c r="E152" s="6"/>
       <c r="F152" s="6"/>
@@ -36170,10 +37789,16 @@
       <c r="Y152" s="6"/>
       <c r="Z152" s="6"/>
     </row>
-    <row r="153" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A153" s="6"/>
-      <c r="B153" s="6"/>
-      <c r="C153" s="8"/>
+    <row r="153" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A153" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="B153" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C153" s="7">
+        <v>46252</v>
+      </c>
       <c r="D153" s="6"/>
       <c r="E153" s="6"/>
       <c r="F153" s="6"/>
@@ -36198,10 +37823,16 @@
       <c r="Y153" s="6"/>
       <c r="Z153" s="6"/>
     </row>
-    <row r="154" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A154" s="6"/>
-      <c r="B154" s="6"/>
-      <c r="C154" s="8"/>
+    <row r="154" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A154" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="B154" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="C154" s="7">
+        <v>46253</v>
+      </c>
       <c r="D154" s="6"/>
       <c r="E154" s="6"/>
       <c r="F154" s="6"/>
@@ -36226,10 +37857,16 @@
       <c r="Y154" s="6"/>
       <c r="Z154" s="6"/>
     </row>
-    <row r="155" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A155" s="6"/>
-      <c r="B155" s="6"/>
-      <c r="C155" s="8"/>
+    <row r="155" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A155" s="11" t="s">
+        <v>422</v>
+      </c>
+      <c r="B155" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="C155" s="7">
+        <v>46254</v>
+      </c>
       <c r="D155" s="6"/>
       <c r="E155" s="6"/>
       <c r="F155" s="6"/>
@@ -36254,10 +37891,16 @@
       <c r="Y155" s="6"/>
       <c r="Z155" s="6"/>
     </row>
-    <row r="156" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A156" s="6"/>
-      <c r="B156" s="6"/>
-      <c r="C156" s="8"/>
+    <row r="156" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A156" s="11" t="s">
+        <v>423</v>
+      </c>
+      <c r="B156" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="C156" s="7">
+        <v>46255</v>
+      </c>
       <c r="D156" s="6"/>
       <c r="E156" s="6"/>
       <c r="F156" s="6"/>
@@ -36282,10 +37925,16 @@
       <c r="Y156" s="6"/>
       <c r="Z156" s="6"/>
     </row>
-    <row r="157" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A157" s="6"/>
-      <c r="B157" s="6"/>
-      <c r="C157" s="8"/>
+    <row r="157" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A157" s="11" t="s">
+        <v>309</v>
+      </c>
+      <c r="B157" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="C157" s="7">
+        <v>46256</v>
+      </c>
       <c r="D157" s="6"/>
       <c r="E157" s="6"/>
       <c r="F157" s="6"/>
@@ -36310,10 +37959,16 @@
       <c r="Y157" s="6"/>
       <c r="Z157" s="6"/>
     </row>
-    <row r="158" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A158" s="6"/>
-      <c r="B158" s="6"/>
-      <c r="C158" s="8"/>
+    <row r="158" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A158" s="11" t="s">
+        <v>424</v>
+      </c>
+      <c r="B158" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="C158" s="7">
+        <v>46257</v>
+      </c>
       <c r="D158" s="6"/>
       <c r="E158" s="6"/>
       <c r="F158" s="6"/>
@@ -36338,10 +37993,16 @@
       <c r="Y158" s="6"/>
       <c r="Z158" s="6"/>
     </row>
-    <row r="159" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A159" s="6"/>
-      <c r="B159" s="6"/>
-      <c r="C159" s="8"/>
+    <row r="159" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A159" s="11" t="s">
+        <v>425</v>
+      </c>
+      <c r="B159" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="C159" s="7">
+        <v>46258</v>
+      </c>
       <c r="D159" s="6"/>
       <c r="E159" s="6"/>
       <c r="F159" s="6"/>
@@ -36366,10 +38027,16 @@
       <c r="Y159" s="6"/>
       <c r="Z159" s="6"/>
     </row>
-    <row r="160" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A160" s="6"/>
-      <c r="B160" s="6"/>
-      <c r="C160" s="8"/>
+    <row r="160" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A160" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="B160" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="C160" s="7">
+        <v>46259</v>
+      </c>
       <c r="D160" s="6"/>
       <c r="E160" s="6"/>
       <c r="F160" s="6"/>
@@ -36394,10 +38061,16 @@
       <c r="Y160" s="6"/>
       <c r="Z160" s="6"/>
     </row>
-    <row r="161" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A161" s="6"/>
-      <c r="B161" s="6"/>
-      <c r="C161" s="8"/>
+    <row r="161" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A161" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="B161" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="C161" s="7">
+        <v>46260</v>
+      </c>
       <c r="D161" s="6"/>
       <c r="E161" s="6"/>
       <c r="F161" s="6"/>
@@ -36422,10 +38095,16 @@
       <c r="Y161" s="6"/>
       <c r="Z161" s="6"/>
     </row>
-    <row r="162" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A162" s="6"/>
-      <c r="B162" s="6"/>
-      <c r="C162" s="8"/>
+    <row r="162" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A162" s="11" t="s">
+        <v>428</v>
+      </c>
+      <c r="B162" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="C162" s="7">
+        <v>46261</v>
+      </c>
       <c r="D162" s="6"/>
       <c r="E162" s="6"/>
       <c r="F162" s="6"/>
@@ -36450,10 +38129,16 @@
       <c r="Y162" s="6"/>
       <c r="Z162" s="6"/>
     </row>
-    <row r="163" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A163" s="6"/>
-      <c r="B163" s="6"/>
-      <c r="C163" s="8"/>
+    <row r="163" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A163" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="B163" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="C163" s="7">
+        <v>46262</v>
+      </c>
       <c r="D163" s="6"/>
       <c r="E163" s="6"/>
       <c r="F163" s="6"/>
@@ -36478,10 +38163,16 @@
       <c r="Y163" s="6"/>
       <c r="Z163" s="6"/>
     </row>
-    <row r="164" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A164" s="6"/>
-      <c r="B164" s="6"/>
-      <c r="C164" s="8"/>
+    <row r="164" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A164" s="11" t="s">
+        <v>430</v>
+      </c>
+      <c r="B164" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="C164" s="7">
+        <v>46263</v>
+      </c>
       <c r="D164" s="6"/>
       <c r="E164" s="6"/>
       <c r="F164" s="6"/>
@@ -36506,10 +38197,16 @@
       <c r="Y164" s="6"/>
       <c r="Z164" s="6"/>
     </row>
-    <row r="165" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A165" s="6"/>
-      <c r="B165" s="6"/>
-      <c r="C165" s="8"/>
+    <row r="165" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A165" s="11" t="s">
+        <v>431</v>
+      </c>
+      <c r="B165" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="C165" s="7">
+        <v>46264</v>
+      </c>
       <c r="D165" s="6"/>
       <c r="E165" s="6"/>
       <c r="F165" s="6"/>
@@ -36534,10 +38231,16 @@
       <c r="Y165" s="6"/>
       <c r="Z165" s="6"/>
     </row>
-    <row r="166" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A166" s="6"/>
-      <c r="B166" s="6"/>
-      <c r="C166" s="8"/>
+    <row r="166" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A166" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="B166" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="C166" s="7">
+        <v>46265</v>
+      </c>
       <c r="D166" s="6"/>
       <c r="E166" s="6"/>
       <c r="F166" s="6"/>
@@ -36562,10 +38265,16 @@
       <c r="Y166" s="6"/>
       <c r="Z166" s="6"/>
     </row>
-    <row r="167" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A167" s="6"/>
-      <c r="B167" s="6"/>
-      <c r="C167" s="8"/>
+    <row r="167" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A167" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="B167" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="C167" s="7">
+        <v>46266</v>
+      </c>
       <c r="D167" s="6"/>
       <c r="E167" s="6"/>
       <c r="F167" s="6"/>
@@ -36590,10 +38299,16 @@
       <c r="Y167" s="6"/>
       <c r="Z167" s="6"/>
     </row>
-    <row r="168" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A168" s="6"/>
-      <c r="B168" s="6"/>
-      <c r="C168" s="8"/>
+    <row r="168" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A168" s="11" t="s">
+        <v>434</v>
+      </c>
+      <c r="B168" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="C168" s="7">
+        <v>46267</v>
+      </c>
       <c r="D168" s="6"/>
       <c r="E168" s="6"/>
       <c r="F168" s="6"/>
@@ -36618,10 +38333,16 @@
       <c r="Y168" s="6"/>
       <c r="Z168" s="6"/>
     </row>
-    <row r="169" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A169" s="6"/>
-      <c r="B169" s="6"/>
-      <c r="C169" s="8"/>
+    <row r="169" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A169" s="11" t="s">
+        <v>435</v>
+      </c>
+      <c r="B169" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="C169" s="7">
+        <v>46268</v>
+      </c>
       <c r="D169" s="6"/>
       <c r="E169" s="6"/>
       <c r="F169" s="6"/>
@@ -36646,10 +38367,16 @@
       <c r="Y169" s="6"/>
       <c r="Z169" s="6"/>
     </row>
-    <row r="170" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A170" s="6"/>
-      <c r="B170" s="6"/>
-      <c r="C170" s="8"/>
+    <row r="170" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A170" s="11" t="s">
+        <v>413</v>
+      </c>
+      <c r="B170" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="C170" s="7">
+        <v>46269</v>
+      </c>
       <c r="D170" s="6"/>
       <c r="E170" s="6"/>
       <c r="F170" s="6"/>
@@ -36674,10 +38401,16 @@
       <c r="Y170" s="6"/>
       <c r="Z170" s="6"/>
     </row>
-    <row r="171" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A171" s="6"/>
-      <c r="B171" s="6"/>
-      <c r="C171" s="8"/>
+    <row r="171" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A171" s="11" t="s">
+        <v>436</v>
+      </c>
+      <c r="B171" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="C171" s="7">
+        <v>46270</v>
+      </c>
       <c r="D171" s="6"/>
       <c r="E171" s="6"/>
       <c r="F171" s="6"/>
@@ -36702,10 +38435,16 @@
       <c r="Y171" s="6"/>
       <c r="Z171" s="6"/>
     </row>
-    <row r="172" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A172" s="6"/>
-      <c r="B172" s="6"/>
-      <c r="C172" s="8"/>
+    <row r="172" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A172" s="11" t="s">
+        <v>437</v>
+      </c>
+      <c r="B172" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="C172" s="7">
+        <v>46271</v>
+      </c>
       <c r="D172" s="6"/>
       <c r="E172" s="6"/>
       <c r="F172" s="6"/>
@@ -36730,10 +38469,16 @@
       <c r="Y172" s="6"/>
       <c r="Z172" s="6"/>
     </row>
-    <row r="173" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A173" s="6"/>
-      <c r="B173" s="6"/>
-      <c r="C173" s="8"/>
+    <row r="173" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A173" s="11" t="s">
+        <v>438</v>
+      </c>
+      <c r="B173" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="C173" s="7">
+        <v>46272</v>
+      </c>
       <c r="D173" s="6"/>
       <c r="E173" s="6"/>
       <c r="F173" s="6"/>
@@ -36758,10 +38503,16 @@
       <c r="Y173" s="6"/>
       <c r="Z173" s="6"/>
     </row>
-    <row r="174" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A174" s="6"/>
-      <c r="B174" s="6"/>
-      <c r="C174" s="8"/>
+    <row r="174" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A174" s="11" t="s">
+        <v>439</v>
+      </c>
+      <c r="B174" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="C174" s="7">
+        <v>46273</v>
+      </c>
       <c r="D174" s="6"/>
       <c r="E174" s="6"/>
       <c r="F174" s="6"/>
@@ -36786,10 +38537,16 @@
       <c r="Y174" s="6"/>
       <c r="Z174" s="6"/>
     </row>
-    <row r="175" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A175" s="6"/>
-      <c r="B175" s="6"/>
-      <c r="C175" s="8"/>
+    <row r="175" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A175" s="11" t="s">
+        <v>440</v>
+      </c>
+      <c r="B175" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="C175" s="7">
+        <v>46274</v>
+      </c>
       <c r="D175" s="6"/>
       <c r="E175" s="6"/>
       <c r="F175" s="6"/>
@@ -36814,10 +38571,16 @@
       <c r="Y175" s="6"/>
       <c r="Z175" s="6"/>
     </row>
-    <row r="176" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A176" s="6"/>
-      <c r="B176" s="6"/>
-      <c r="C176" s="8"/>
+    <row r="176" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A176" s="11" t="s">
+        <v>441</v>
+      </c>
+      <c r="B176" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="C176" s="7">
+        <v>46275</v>
+      </c>
       <c r="D176" s="6"/>
       <c r="E176" s="6"/>
       <c r="F176" s="6"/>
@@ -36842,10 +38605,16 @@
       <c r="Y176" s="6"/>
       <c r="Z176" s="6"/>
     </row>
-    <row r="177" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A177" s="6"/>
-      <c r="B177" s="6"/>
-      <c r="C177" s="8"/>
+    <row r="177" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A177" s="11" t="s">
+        <v>442</v>
+      </c>
+      <c r="B177" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="C177" s="7">
+        <v>46276</v>
+      </c>
       <c r="D177" s="6"/>
       <c r="E177" s="6"/>
       <c r="F177" s="6"/>
@@ -36870,10 +38639,16 @@
       <c r="Y177" s="6"/>
       <c r="Z177" s="6"/>
     </row>
-    <row r="178" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A178" s="6"/>
-      <c r="B178" s="6"/>
-      <c r="C178" s="8"/>
+    <row r="178" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A178" s="11" t="s">
+        <v>443</v>
+      </c>
+      <c r="B178" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="C178" s="7">
+        <v>46277</v>
+      </c>
       <c r="D178" s="6"/>
       <c r="E178" s="6"/>
       <c r="F178" s="6"/>
@@ -36898,10 +38673,16 @@
       <c r="Y178" s="6"/>
       <c r="Z178" s="6"/>
     </row>
-    <row r="179" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A179" s="6"/>
-      <c r="B179" s="6"/>
-      <c r="C179" s="8"/>
+    <row r="179" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A179" s="11" t="s">
+        <v>444</v>
+      </c>
+      <c r="B179" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="C179" s="7">
+        <v>46278</v>
+      </c>
       <c r="D179" s="6"/>
       <c r="E179" s="6"/>
       <c r="F179" s="6"/>
@@ -36926,10 +38707,16 @@
       <c r="Y179" s="6"/>
       <c r="Z179" s="6"/>
     </row>
-    <row r="180" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A180" s="6"/>
-      <c r="B180" s="6"/>
-      <c r="C180" s="8"/>
+    <row r="180" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A180" s="11" t="s">
+        <v>445</v>
+      </c>
+      <c r="B180" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="C180" s="7">
+        <v>46279</v>
+      </c>
       <c r="D180" s="6"/>
       <c r="E180" s="6"/>
       <c r="F180" s="6"/>
@@ -36954,10 +38741,16 @@
       <c r="Y180" s="6"/>
       <c r="Z180" s="6"/>
     </row>
-    <row r="181" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A181" s="6"/>
-      <c r="B181" s="6"/>
-      <c r="C181" s="8"/>
+    <row r="181" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A181" s="11" t="s">
+        <v>446</v>
+      </c>
+      <c r="B181" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="C181" s="7">
+        <v>46280</v>
+      </c>
       <c r="D181" s="6"/>
       <c r="E181" s="6"/>
       <c r="F181" s="6"/>
@@ -36982,10 +38775,16 @@
       <c r="Y181" s="6"/>
       <c r="Z181" s="6"/>
     </row>
-    <row r="182" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A182" s="6"/>
-      <c r="B182" s="6"/>
-      <c r="C182" s="8"/>
+    <row r="182" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A182" s="11" t="s">
+        <v>447</v>
+      </c>
+      <c r="B182" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="C182" s="7">
+        <v>46281</v>
+      </c>
       <c r="D182" s="6"/>
       <c r="E182" s="6"/>
       <c r="F182" s="6"/>
@@ -37010,10 +38809,16 @@
       <c r="Y182" s="6"/>
       <c r="Z182" s="6"/>
     </row>
-    <row r="183" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A183" s="6"/>
-      <c r="B183" s="6"/>
-      <c r="C183" s="8"/>
+    <row r="183" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A183" s="11" t="s">
+        <v>448</v>
+      </c>
+      <c r="B183" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="C183" s="7">
+        <v>46282</v>
+      </c>
       <c r="D183" s="6"/>
       <c r="E183" s="6"/>
       <c r="F183" s="6"/>
@@ -37038,10 +38843,16 @@
       <c r="Y183" s="6"/>
       <c r="Z183" s="6"/>
     </row>
-    <row r="184" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A184" s="6"/>
-      <c r="B184" s="6"/>
-      <c r="C184" s="8"/>
+    <row r="184" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A184" s="11" t="s">
+        <v>449</v>
+      </c>
+      <c r="B184" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="C184" s="7">
+        <v>46283</v>
+      </c>
       <c r="D184" s="6"/>
       <c r="E184" s="6"/>
       <c r="F184" s="6"/>
@@ -37066,10 +38877,16 @@
       <c r="Y184" s="6"/>
       <c r="Z184" s="6"/>
     </row>
-    <row r="185" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A185" s="6"/>
-      <c r="B185" s="6"/>
-      <c r="C185" s="8"/>
+    <row r="185" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A185" s="11" t="s">
+        <v>450</v>
+      </c>
+      <c r="B185" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="C185" s="7">
+        <v>46284</v>
+      </c>
       <c r="D185" s="6"/>
       <c r="E185" s="6"/>
       <c r="F185" s="6"/>
@@ -37094,10 +38911,16 @@
       <c r="Y185" s="6"/>
       <c r="Z185" s="6"/>
     </row>
-    <row r="186" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A186" s="6"/>
-      <c r="B186" s="6"/>
-      <c r="C186" s="8"/>
+    <row r="186" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A186" s="11" t="s">
+        <v>451</v>
+      </c>
+      <c r="B186" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="C186" s="7">
+        <v>46285</v>
+      </c>
       <c r="D186" s="6"/>
       <c r="E186" s="6"/>
       <c r="F186" s="6"/>
@@ -37122,10 +38945,16 @@
       <c r="Y186" s="6"/>
       <c r="Z186" s="6"/>
     </row>
-    <row r="187" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A187" s="6"/>
-      <c r="B187" s="6"/>
-      <c r="C187" s="8"/>
+    <row r="187" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A187" s="11" t="s">
+        <v>452</v>
+      </c>
+      <c r="B187" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="C187" s="7">
+        <v>46286</v>
+      </c>
       <c r="D187" s="6"/>
       <c r="E187" s="6"/>
       <c r="F187" s="6"/>
@@ -37150,10 +38979,16 @@
       <c r="Y187" s="6"/>
       <c r="Z187" s="6"/>
     </row>
-    <row r="188" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A188" s="6"/>
-      <c r="B188" s="6"/>
-      <c r="C188" s="8"/>
+    <row r="188" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A188" s="11" t="s">
+        <v>453</v>
+      </c>
+      <c r="B188" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="C188" s="7">
+        <v>46287</v>
+      </c>
       <c r="D188" s="6"/>
       <c r="E188" s="6"/>
       <c r="F188" s="6"/>
@@ -37178,10 +39013,16 @@
       <c r="Y188" s="6"/>
       <c r="Z188" s="6"/>
     </row>
-    <row r="189" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A189" s="6"/>
-      <c r="B189" s="6"/>
-      <c r="C189" s="8"/>
+    <row r="189" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A189" s="11" t="s">
+        <v>454</v>
+      </c>
+      <c r="B189" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="C189" s="7">
+        <v>46288</v>
+      </c>
       <c r="D189" s="6"/>
       <c r="E189" s="6"/>
       <c r="F189" s="6"/>
@@ -37206,10 +39047,16 @@
       <c r="Y189" s="6"/>
       <c r="Z189" s="6"/>
     </row>
-    <row r="190" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A190" s="6"/>
-      <c r="B190" s="6"/>
-      <c r="C190" s="8"/>
+    <row r="190" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A190" s="11" t="s">
+        <v>455</v>
+      </c>
+      <c r="B190" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="C190" s="7">
+        <v>46289</v>
+      </c>
       <c r="D190" s="6"/>
       <c r="E190" s="6"/>
       <c r="F190" s="6"/>
@@ -37234,10 +39081,16 @@
       <c r="Y190" s="6"/>
       <c r="Z190" s="6"/>
     </row>
-    <row r="191" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A191" s="6"/>
-      <c r="B191" s="6"/>
-      <c r="C191" s="8"/>
+    <row r="191" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A191" s="11" t="s">
+        <v>456</v>
+      </c>
+      <c r="B191" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="C191" s="7">
+        <v>46290</v>
+      </c>
       <c r="D191" s="6"/>
       <c r="E191" s="6"/>
       <c r="F191" s="6"/>
@@ -37262,10 +39115,16 @@
       <c r="Y191" s="6"/>
       <c r="Z191" s="6"/>
     </row>
-    <row r="192" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A192" s="6"/>
-      <c r="B192" s="6"/>
-      <c r="C192" s="8"/>
+    <row r="192" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A192" s="11" t="s">
+        <v>457</v>
+      </c>
+      <c r="B192" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="C192" s="7">
+        <v>46291</v>
+      </c>
       <c r="D192" s="6"/>
       <c r="E192" s="6"/>
       <c r="F192" s="6"/>
@@ -37290,10 +39149,16 @@
       <c r="Y192" s="6"/>
       <c r="Z192" s="6"/>
     </row>
-    <row r="193" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A193" s="6"/>
-      <c r="B193" s="6"/>
-      <c r="C193" s="8"/>
+    <row r="193" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A193" s="11" t="s">
+        <v>458</v>
+      </c>
+      <c r="B193" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="C193" s="7">
+        <v>46292</v>
+      </c>
       <c r="D193" s="6"/>
       <c r="E193" s="6"/>
       <c r="F193" s="6"/>
@@ -37318,10 +39183,16 @@
       <c r="Y193" s="6"/>
       <c r="Z193" s="6"/>
     </row>
-    <row r="194" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A194" s="6"/>
-      <c r="B194" s="6"/>
-      <c r="C194" s="8"/>
+    <row r="194" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A194" s="11" t="s">
+        <v>459</v>
+      </c>
+      <c r="B194" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="C194" s="7">
+        <v>46293</v>
+      </c>
       <c r="D194" s="6"/>
       <c r="E194" s="6"/>
       <c r="F194" s="6"/>
@@ -37346,10 +39217,16 @@
       <c r="Y194" s="6"/>
       <c r="Z194" s="6"/>
     </row>
-    <row r="195" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A195" s="6"/>
-      <c r="B195" s="6"/>
-      <c r="C195" s="8"/>
+    <row r="195" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A195" s="11" t="s">
+        <v>460</v>
+      </c>
+      <c r="B195" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="C195" s="7">
+        <v>46294</v>
+      </c>
       <c r="D195" s="6"/>
       <c r="E195" s="6"/>
       <c r="F195" s="6"/>
@@ -37374,10 +39251,16 @@
       <c r="Y195" s="6"/>
       <c r="Z195" s="6"/>
     </row>
-    <row r="196" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A196" s="6"/>
-      <c r="B196" s="6"/>
-      <c r="C196" s="8"/>
+    <row r="196" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A196" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="B196" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="C196" s="7">
+        <v>46295</v>
+      </c>
       <c r="D196" s="6"/>
       <c r="E196" s="6"/>
       <c r="F196" s="6"/>
@@ -37402,10 +39285,16 @@
       <c r="Y196" s="6"/>
       <c r="Z196" s="6"/>
     </row>
-    <row r="197" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A197" s="6"/>
-      <c r="B197" s="6"/>
-      <c r="C197" s="8"/>
+    <row r="197" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A197" s="11" t="s">
+        <v>461</v>
+      </c>
+      <c r="B197" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="C197" s="7">
+        <v>46296</v>
+      </c>
       <c r="D197" s="6"/>
       <c r="E197" s="6"/>
       <c r="F197" s="6"/>
@@ -37430,10 +39319,16 @@
       <c r="Y197" s="6"/>
       <c r="Z197" s="6"/>
     </row>
-    <row r="198" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A198" s="6"/>
-      <c r="B198" s="6"/>
-      <c r="C198" s="8"/>
+    <row r="198" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A198" s="11" t="s">
+        <v>462</v>
+      </c>
+      <c r="B198" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="C198" s="7">
+        <v>46297</v>
+      </c>
       <c r="D198" s="6"/>
       <c r="E198" s="6"/>
       <c r="F198" s="6"/>
@@ -37458,10 +39353,16 @@
       <c r="Y198" s="6"/>
       <c r="Z198" s="6"/>
     </row>
-    <row r="199" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A199" s="6"/>
-      <c r="B199" s="6"/>
-      <c r="C199" s="8"/>
+    <row r="199" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A199" s="11" t="s">
+        <v>463</v>
+      </c>
+      <c r="B199" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="C199" s="7">
+        <v>46298</v>
+      </c>
       <c r="D199" s="6"/>
       <c r="E199" s="6"/>
       <c r="F199" s="6"/>
@@ -37486,10 +39387,16 @@
       <c r="Y199" s="6"/>
       <c r="Z199" s="6"/>
     </row>
-    <row r="200" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A200" s="6"/>
-      <c r="B200" s="6"/>
-      <c r="C200" s="8"/>
+    <row r="200" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A200" s="11" t="s">
+        <v>464</v>
+      </c>
+      <c r="B200" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="C200" s="7">
+        <v>46299</v>
+      </c>
       <c r="D200" s="6"/>
       <c r="E200" s="6"/>
       <c r="F200" s="6"/>
@@ -37514,10 +39421,16 @@
       <c r="Y200" s="6"/>
       <c r="Z200" s="6"/>
     </row>
-    <row r="201" spans="1:26" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A201" s="6"/>
-      <c r="B201" s="6"/>
-      <c r="C201" s="8"/>
+    <row r="201" spans="1:26" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A201" s="11" t="s">
+        <v>465</v>
+      </c>
+      <c r="B201" s="6" t="s">
+        <v>379</v>
+      </c>
+      <c r="C201" s="7">
+        <v>46300</v>
+      </c>
       <c r="D201" s="6"/>
       <c r="E201" s="6"/>
       <c r="F201" s="6"/>
@@ -58571,6 +60484,68 @@
     <hyperlink ref="A137" r:id="rId136" xr:uid="{7A5C1420-CA71-4CD4-B611-B441B73D8453}"/>
     <hyperlink ref="A138" r:id="rId137" xr:uid="{D19F617A-EF9B-4BAD-8D9A-A7FE415CEFBF}"/>
     <hyperlink ref="A139" r:id="rId138" xr:uid="{F556C6CD-2AF6-4C75-9085-55B396B6094D}"/>
+    <hyperlink ref="A140" r:id="rId139" display="https://www.youtube.com/watch?v=IEZVq01Q7go&amp;t=14s" xr:uid="{D173B189-BF96-4FBF-8488-FE82DCBDC4D9}"/>
+    <hyperlink ref="A141" r:id="rId140" display="https://www.youtube.com/watch?v=jiFJXvMc2SY&amp;t=321s" xr:uid="{193D0DB7-3852-4743-AF0C-FC894AEA968D}"/>
+    <hyperlink ref="A142" r:id="rId141" display="https://www.youtube.com/watch?v=fr6B3EtlZVM&amp;t=3s" xr:uid="{95722412-6DDC-4FD9-8AF5-681F4CFFC3CA}"/>
+    <hyperlink ref="A143" r:id="rId142" display="https://www.youtube.com/watch?v=PBNhMcRKu24&amp;t=1s" xr:uid="{91BB30D1-04C4-4C5A-99EE-4206CA26BCD2}"/>
+    <hyperlink ref="A144" r:id="rId143" display="https://www.youtube.com/watch?v=ZHFNRrT8WA4&amp;t=3s" xr:uid="{84E31E27-C270-41B8-B1F5-2C57BAAF42C1}"/>
+    <hyperlink ref="A145" r:id="rId144" display="https://www.youtube.com/watch?v=mXLQFJ-W7xc&amp;t=23s" xr:uid="{AE2C0C8B-F0BE-40AE-918F-0CD0142D254A}"/>
+    <hyperlink ref="A146" r:id="rId145" display="https://www.youtube.com/watch?v=gN9bQHaOKg8&amp;t=96s" xr:uid="{B92FE323-D57D-45CD-81BA-BF63E2302514}"/>
+    <hyperlink ref="A147" r:id="rId146" display="https://www.youtube.com/watch?v=BXylPudUUek&amp;t=13s" xr:uid="{B8DCDB84-D756-4D73-95B4-F5D6359BF687}"/>
+    <hyperlink ref="A148" r:id="rId147" display="https://www.youtube.com/watch?v=tbluAPW3aLs&amp;t=3s" xr:uid="{466A606A-0501-4F7E-AA75-727CC7754953}"/>
+    <hyperlink ref="A149" r:id="rId148" xr:uid="{A5346734-07B4-4835-9B43-C3B9ED58B42F}"/>
+    <hyperlink ref="A150" r:id="rId149" xr:uid="{76858C4E-0F01-4C01-8BDA-8699CC36850F}"/>
+    <hyperlink ref="A151" r:id="rId150" xr:uid="{A6E3AB01-399D-40AC-B027-D25BDC450CDF}"/>
+    <hyperlink ref="A152" r:id="rId151" xr:uid="{88B5C54D-6F60-4D26-BAB0-C16794149DE8}"/>
+    <hyperlink ref="A153" r:id="rId152" xr:uid="{DB68D4DB-0B36-4330-8FC5-CF6B47A3E50C}"/>
+    <hyperlink ref="A154" r:id="rId153" xr:uid="{C095A84A-3354-433F-96A4-40E010233845}"/>
+    <hyperlink ref="A155" r:id="rId154" xr:uid="{33D2BC74-047E-4C78-BC3C-8A71B3C817F0}"/>
+    <hyperlink ref="A156" r:id="rId155" xr:uid="{B6DA7DB2-5B44-42EF-A704-02412CC0101D}"/>
+    <hyperlink ref="A157" r:id="rId156" display="https://www.youtube.com/watch?v=i8v5Fb_aDW8&amp;t=351s" xr:uid="{0F94D7AF-51EB-4C45-BEC3-0A967119C46E}"/>
+    <hyperlink ref="A158" r:id="rId157" display="https://www.youtube.com/watch?v=8e4gw8yeQIo&amp;t=109s" xr:uid="{0E0F5F2F-8CDB-4DA7-A94E-C9A35EB45CE5}"/>
+    <hyperlink ref="A159" r:id="rId158" xr:uid="{47FA3F0C-6011-4CD5-88E0-757C410FACCF}"/>
+    <hyperlink ref="A160" r:id="rId159" xr:uid="{010E51B2-7447-4B75-8AD2-B3A4614B83CB}"/>
+    <hyperlink ref="A161" r:id="rId160" xr:uid="{DA703F68-94C8-400F-86F9-490D8FE4E346}"/>
+    <hyperlink ref="A162" r:id="rId161" display="https://www.youtube.com/watch?v=tBIG11CRXmM&amp;t=14s" xr:uid="{8B37758C-AF6C-45E0-8016-B2CD8F019813}"/>
+    <hyperlink ref="A163" r:id="rId162" display="https://www.youtube.com/watch?v=S-ZrxzifoQ0&amp;t=3s" xr:uid="{79C15996-D9B0-433B-8106-554C6A9EB0A0}"/>
+    <hyperlink ref="A164" r:id="rId163" display="https://www.youtube.com/watch?v=8anpFagF9VU&amp;t=23s" xr:uid="{F47636CE-F71B-4C3C-9DC4-FDD8DACE48CE}"/>
+    <hyperlink ref="A165" r:id="rId164" display="https://www.youtube.com/watch?v=cx2wkrKymok&amp;t=221s" xr:uid="{D27D8308-59DC-4C8A-9EB0-C3E2400F659C}"/>
+    <hyperlink ref="A166" r:id="rId165" xr:uid="{3CFC55E0-31B7-413B-984C-EAB3C9DD54B7}"/>
+    <hyperlink ref="A167" r:id="rId166" xr:uid="{29513E09-8B23-46F3-9526-0451D51848AD}"/>
+    <hyperlink ref="A168" r:id="rId167" xr:uid="{80694DBA-2352-4D28-84A9-790684B699C6}"/>
+    <hyperlink ref="A169" r:id="rId168" xr:uid="{0433783A-B592-4774-8528-0690230071EA}"/>
+    <hyperlink ref="A170" r:id="rId169" xr:uid="{98A32DF7-0643-441D-9FBB-7DC68E55A810}"/>
+    <hyperlink ref="A171" r:id="rId170" xr:uid="{F065709C-632C-4BEA-B657-AE7F5BBC19FE}"/>
+    <hyperlink ref="A172" r:id="rId171" display="https://www.youtube.com/watch?v=5RbaPlzKbFk&amp;t=6s" xr:uid="{4F05C23B-7678-481B-8766-0290EA09B8BE}"/>
+    <hyperlink ref="A173" r:id="rId172" xr:uid="{ADF948DB-3FEB-4E31-BAB1-121EF29FB3FC}"/>
+    <hyperlink ref="A174" r:id="rId173" xr:uid="{9A11025D-EB50-4917-BA93-30A0E1B5C03E}"/>
+    <hyperlink ref="A175" r:id="rId174" xr:uid="{D899E78D-477E-4C1F-B493-4534DFF6C5BA}"/>
+    <hyperlink ref="A176" r:id="rId175" xr:uid="{78950D1C-54ED-40B6-A5B4-828EA307D434}"/>
+    <hyperlink ref="A177" r:id="rId176" xr:uid="{B6BF2869-A8C9-4670-8D5C-B5F4A57BB34B}"/>
+    <hyperlink ref="A178" r:id="rId177" xr:uid="{E878939A-A8A2-4556-BBE5-5AB328F525D8}"/>
+    <hyperlink ref="A179" r:id="rId178" display="https://www.youtube.com/watch?v=vcnndeYVw9k&amp;t=4s" xr:uid="{6C60A267-21E6-41CA-AC8F-C22D682B1B35}"/>
+    <hyperlink ref="A180" r:id="rId179" display="https://www.youtube.com/watch?v=Y1zBcg4QJgE&amp;t=8s" xr:uid="{8F6FF15A-2F2B-4E27-85E0-060CE2908DE4}"/>
+    <hyperlink ref="A181" r:id="rId180" display="https://www.youtube.com/watch?v=1Ilgi75Y6Ac&amp;t=9s" xr:uid="{76531606-BD9A-42DB-9344-0A471E2B73BA}"/>
+    <hyperlink ref="A182" r:id="rId181" xr:uid="{B7E0B424-71C3-4332-A184-4BCFC7B5EC52}"/>
+    <hyperlink ref="A183" r:id="rId182" xr:uid="{DEC9FD41-2D26-4AEE-A2AD-991B90B0A393}"/>
+    <hyperlink ref="A184" r:id="rId183" xr:uid="{C47CC242-DEF3-46BB-9AE6-4FFFF504EC7D}"/>
+    <hyperlink ref="A185" r:id="rId184" display="https://www.youtube.com/watch?v=zgLWXkOMOGE&amp;t=20s" xr:uid="{A517013C-9D2C-4C87-94AC-46E43155B0F5}"/>
+    <hyperlink ref="A186" r:id="rId185" display="https://www.youtube.com/watch?v=r-DPvpwMOdw&amp;t=144s" xr:uid="{97EF298D-1A01-4B67-A991-EF3A497F119A}"/>
+    <hyperlink ref="A187" r:id="rId186" xr:uid="{15487E72-35D7-4763-8257-7F555B62BA65}"/>
+    <hyperlink ref="A188" r:id="rId187" xr:uid="{9E1BA6B8-2CDE-4D6F-B3BE-016D6E683834}"/>
+    <hyperlink ref="A189" r:id="rId188" xr:uid="{2D63301B-60D8-4FF6-8B45-DA4ED9863E59}"/>
+    <hyperlink ref="A190" r:id="rId189" xr:uid="{3BBFF293-9144-4761-85A5-F181493DAF82}"/>
+    <hyperlink ref="A191" r:id="rId190" display="https://www.youtube.com/watch?v=X6XNEMBmPrk&amp;t=149s" xr:uid="{0793F0FF-39A7-41FD-8155-2DE0A2903A74}"/>
+    <hyperlink ref="A192" r:id="rId191" xr:uid="{623E966B-0E4F-4DF8-996E-BF1817DD7DC4}"/>
+    <hyperlink ref="A193" r:id="rId192" xr:uid="{9A4AAEAD-B4F7-40D4-BFD3-78724ADE7B61}"/>
+    <hyperlink ref="A194" r:id="rId193" display="https://www.youtube.com/watch?v=qCOWcKURVzk&amp;t=1s" xr:uid="{8F3EBA6A-67CC-4C8B-B8E3-77A6C26CDC61}"/>
+    <hyperlink ref="A195" r:id="rId194" xr:uid="{99D89B2D-C8D4-4BD0-A2B3-4953E14B2EA4}"/>
+    <hyperlink ref="A196" r:id="rId195" display="https://www.youtube.com/watch?v=-NHHdVWUcwo&amp;t=3s" xr:uid="{ACE8DB35-485E-42CB-B586-939F57F2D798}"/>
+    <hyperlink ref="A197" r:id="rId196" display="https://www.youtube.com/watch?v=IS1Fcnh-W-M&amp;t=9s" xr:uid="{5D228E77-B6D8-4A69-AA3A-A482077C84E5}"/>
+    <hyperlink ref="A198" r:id="rId197" display="https://www.youtube.com/watch?v=Rssbr11AO1o&amp;t=1s" xr:uid="{C759FCE7-4EAF-4165-A0AE-43FA748DE6A8}"/>
+    <hyperlink ref="A199" r:id="rId198" display="https://www.youtube.com/watch?v=7rdJOSgHgg4&amp;t=559s" xr:uid="{5AE9086F-C88B-4904-B4B1-017E953B6112}"/>
+    <hyperlink ref="A200" r:id="rId199" xr:uid="{F88CFF51-F646-4EC3-B430-19E5215C4A65}"/>
+    <hyperlink ref="A201" r:id="rId200" display="https://www.youtube.com/watch?v=tS58CDMrFxA&amp;t=23s" xr:uid="{9C56800F-7A09-4835-95ED-C639EFD179DF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>